<commit_message>
chore: monitoring 23/04/2026 16:21
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (14/07/2026)</t>
+          <t>Valide 81j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 321j (05/03/2027)</t>
+          <t>Valide 315j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 106j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 111j (07/08/2026)</t>
+          <t>Valide 105j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (05/07/2026)</t>
+          <t>Valide 72j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 283j (26/01/2027)</t>
+          <t>Valide 277j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,25 +1152,29 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (20/05/2026)</t>
+          <t>Expire dans 27j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>27j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 199j (02/11/2026)</t>
+          <t>Valide 192j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr"/>
+          <t>23/04/2026 16:16</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1258,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 298j (09/02/2027)</t>
+          <t>Valide 292j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>298j</t>
+          <t>292j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 317j (28/02/2027)</t>
+          <t>Valide 310j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (14/06/2026)</t>
+          <t>Valide 51j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 110j (05/08/2026)</t>
+          <t>Valide 104j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 96j (22/07/2026)</t>
+          <t>Valide 89j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (14/10/2026)</t>
+          <t>Valide 174j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>174j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (29/06/2026)</t>
+          <t>Valide 67j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 234j (07/12/2026)</t>
+          <t>Valide 228j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (09/10/2026)</t>
+          <t>Valide 169j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>169j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 227j (30/11/2026)</t>
+          <t>Valide 220j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 298j (09/02/2027)</t>
+          <t>Valide 292j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>298j</t>
+          <t>292j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 217j (20/11/2026)</t>
+          <t>Valide 210j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 246j (19/12/2026)</t>
+          <t>Valide 240j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>246j</t>
+          <t>240j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 105j (31/07/2026)</t>
+          <t>Valide 98j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (13/10/2026)</t>
+          <t>Valide 173j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>179j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (10/10/2026)</t>
+          <t>Valide 169j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
+          <t>23/04/2026 16:16</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 24/04/2026 09:08
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (14/07/2026)</t>
+          <t>Valide 80j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 315j (05/03/2027)</t>
+          <t>Valide 314j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 106j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 105j (07/08/2026)</t>
+          <t>Valide 104j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (05/07/2026)</t>
+          <t>Valide 71j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 277j (26/01/2027)</t>
+          <t>Valide 276j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 27j (20/05/2026)</t>
+          <t>Expire dans 26j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>27j</t>
+          <t>26j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,12 +1262,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 292j (09/02/2027)</t>
+          <t>Valide 291j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>292j</t>
+          <t>291j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 104j (05/08/2026)</t>
+          <t>Valide 103j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (14/10/2026)</t>
+          <t>Valide 173j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>174j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (29/06/2026)</t>
+          <t>Valide 66j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 228j (07/12/2026)</t>
+          <t>Valide 227j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,12 +2001,12 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (09/10/2026)</t>
+          <t>Valide 168j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>169j</t>
+          <t>168j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,12 +2203,12 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 292j (09/02/2027)</t>
+          <t>Valide 291j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>292j</t>
+          <t>291j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,12 +2449,12 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 240j (19/12/2026)</t>
+          <t>Valide 239j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>240j</t>
+          <t>239j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,12 +2691,12 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (13/10/2026)</t>
+          <t>Valide 172j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>173j</t>
+          <t>172j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>23/04/2026 16:16</t>
+          <t>24/04/2026 09:02</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 25/04/2026 08:11
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (14/07/2026)</t>
+          <t>Valide 79j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 314j (05/03/2027)</t>
+          <t>Valide 313j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 104j (07/08/2026)</t>
+          <t>Valide 103j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (05/07/2026)</t>
+          <t>Valide 70j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 276j (26/01/2027)</t>
+          <t>Valide 275j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 26j (20/05/2026)</t>
+          <t>Expire dans 25j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>26j</t>
+          <t>25j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (02/11/2026)</t>
+          <t>Valide 191j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 291j (09/02/2027)</t>
+          <t>Valide 290j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>291j</t>
+          <t>290j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 310j (28/02/2027)</t>
+          <t>Valide 309j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (14/06/2026)</t>
+          <t>Valide 50j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 103j (05/08/2026)</t>
+          <t>Valide 102j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (22/07/2026)</t>
+          <t>Valide 88j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (14/10/2026)</t>
+          <t>Valide 172j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>173j</t>
+          <t>172j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (29/06/2026)</t>
+          <t>Valide 65j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 227j (07/12/2026)</t>
+          <t>Valide 226j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (09/10/2026)</t>
+          <t>Valide 167j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>168j</t>
+          <t>167j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 220j (30/11/2026)</t>
+          <t>Valide 219j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 291j (09/02/2027)</t>
+          <t>Valide 290j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>291j</t>
+          <t>290j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 210j (20/11/2026)</t>
+          <t>Valide 209j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 239j (19/12/2026)</t>
+          <t>Valide 238j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>239j</t>
+          <t>238j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 98j (31/07/2026)</t>
+          <t>Valide 97j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (13/10/2026)</t>
+          <t>Valide 171j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>172j</t>
+          <t>171j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (10/10/2026)</t>
+          <t>Valide 168j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>24/04/2026 09:02</t>
+          <t>25/04/2026 08:06</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 26/04/2026 08:21
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (14/07/2026)</t>
+          <t>Valide 78j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 313j (05/03/2027)</t>
+          <t>Valide 312j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 103j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 103j (07/08/2026)</t>
+          <t>Valide 102j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (05/07/2026)</t>
+          <t>Valide 69j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 275j (26/01/2027)</t>
+          <t>Valide 274j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 25j (20/05/2026)</t>
+          <t>Expire dans 24j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>25j</t>
+          <t>24j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (02/11/2026)</t>
+          <t>Valide 190j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 290j (09/02/2027)</t>
+          <t>Valide 289j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>290j</t>
+          <t>289j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 309j (28/02/2027)</t>
+          <t>Valide 308j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (14/06/2026)</t>
+          <t>Valide 49j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 102j (05/08/2026)</t>
+          <t>Valide 101j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 88j (22/07/2026)</t>
+          <t>Valide 87j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (14/10/2026)</t>
+          <t>Valide 171j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>172j</t>
+          <t>171j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (29/06/2026)</t>
+          <t>Valide 64j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 226j (07/12/2026)</t>
+          <t>Valide 225j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (09/10/2026)</t>
+          <t>Valide 166j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>167j</t>
+          <t>166j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 219j (30/11/2026)</t>
+          <t>Valide 218j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 290j (09/02/2027)</t>
+          <t>Valide 289j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>290j</t>
+          <t>289j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 209j (20/11/2026)</t>
+          <t>Valide 208j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 238j (19/12/2026)</t>
+          <t>Valide 237j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>238j</t>
+          <t>237j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 97j (31/07/2026)</t>
+          <t>Valide 96j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (13/10/2026)</t>
+          <t>Valide 170j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>171j</t>
+          <t>170j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (10/10/2026)</t>
+          <t>Valide 167j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>25/04/2026 08:06</t>
+          <t>26/04/2026 08:16</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 27/04/2026 09:29
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (14/07/2026)</t>
+          <t>Valide 77j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 312j (05/03/2027)</t>
+          <t>Valide 311j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 103j (07/08/2026)</t>
+          <t>Valide 102j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 102j (07/08/2026)</t>
+          <t>Valide 101j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (05/07/2026)</t>
+          <t>Valide 68j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 274j (26/01/2027)</t>
+          <t>Valide 273j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 24j (20/05/2026)</t>
+          <t>Expire dans 23j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>24j</t>
+          <t>23j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (02/11/2026)</t>
+          <t>Valide 189j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 289j (09/02/2027)</t>
+          <t>Valide 288j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>289j</t>
+          <t>288j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 308j (28/02/2027)</t>
+          <t>Valide 307j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (14/06/2026)</t>
+          <t>Valide 48j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 101j (05/08/2026)</t>
+          <t>Valide 100j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>101j</t>
+          <t>100j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (22/07/2026)</t>
+          <t>Valide 86j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (14/10/2026)</t>
+          <t>Valide 170j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>171j</t>
+          <t>170j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (29/06/2026)</t>
+          <t>Valide 63j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 225j (07/12/2026)</t>
+          <t>Valide 224j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (09/10/2026)</t>
+          <t>Valide 165j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>166j</t>
+          <t>165j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 218j (30/11/2026)</t>
+          <t>Valide 217j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 289j (09/02/2027)</t>
+          <t>Valide 288j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>289j</t>
+          <t>288j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 208j (20/11/2026)</t>
+          <t>Valide 207j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 237j (19/12/2026)</t>
+          <t>Valide 236j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>237j</t>
+          <t>236j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 96j (31/07/2026)</t>
+          <t>Valide 95j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (13/10/2026)</t>
+          <t>Valide 169j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>170j</t>
+          <t>169j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (10/10/2026)</t>
+          <t>Valide 166j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>26/04/2026 08:16</t>
+          <t>27/04/2026 09:23</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 28/04/2026 09:31
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (14/07/2026)</t>
+          <t>Valide 76j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 311j (05/03/2027)</t>
+          <t>Valide 310j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 102j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 101j (07/08/2026)</t>
+          <t>Valide 100j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (05/07/2026)</t>
+          <t>Valide 67j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 273j (26/01/2027)</t>
+          <t>Valide 272j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 23j (20/05/2026)</t>
+          <t>Expire dans 22j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>23j</t>
+          <t>22j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (02/11/2026)</t>
+          <t>Valide 188j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 288j (09/02/2027)</t>
+          <t>Valide 287j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>288j</t>
+          <t>287j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 307j (28/02/2027)</t>
+          <t>Valide 306j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (14/06/2026)</t>
+          <t>Valide 47j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 100j (05/08/2026)</t>
+          <t>Valide 99j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>100j</t>
+          <t>99j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (22/07/2026)</t>
+          <t>Valide 85j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (14/10/2026)</t>
+          <t>Valide 169j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>170j</t>
+          <t>169j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (29/06/2026)</t>
+          <t>Valide 62j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 224j (07/12/2026)</t>
+          <t>Valide 223j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (09/10/2026)</t>
+          <t>Valide 164j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>165j</t>
+          <t>164j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 217j (30/11/2026)</t>
+          <t>Valide 216j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 288j (09/02/2027)</t>
+          <t>Valide 287j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>288j</t>
+          <t>287j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 207j (20/11/2026)</t>
+          <t>Valide 206j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 236j (19/12/2026)</t>
+          <t>Valide 235j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>236j</t>
+          <t>235j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 95j (31/07/2026)</t>
+          <t>Valide 94j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (13/10/2026)</t>
+          <t>Valide 168j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>169j</t>
+          <t>168j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (10/10/2026)</t>
+          <t>Valide 165j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>27/04/2026 09:23</t>
+          <t>28/04/2026 09:26</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 29/04/2026 09:17
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (14/07/2026)</t>
+          <t>Valide 75j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 310j (05/03/2027)</t>
+          <t>[Errno -2] Name or service not known</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 100j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>100j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 100j (07/08/2026)</t>
+          <t>Valide 99j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (05/07/2026)</t>
+          <t>Valide 66j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 272j (26/01/2027)</t>
+          <t>[Errno -2] Name or service not known</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 22j (20/05/2026)</t>
+          <t>Expire dans 21j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>22j</t>
+          <t>21j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (02/11/2026)</t>
+          <t>Valide 187j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 287j (09/02/2027)</t>
+          <t>Valide 286j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>287j</t>
+          <t>286j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 306j (28/02/2027)</t>
+          <t>Valide 305j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (14/06/2026)</t>
+          <t>Valide 46j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 99j (05/08/2026)</t>
+          <t>Valide 98j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>99j</t>
+          <t>98j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (22/07/2026)</t>
+          <t>Valide 84j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (14/10/2026)</t>
+          <t>Valide 168j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>169j</t>
+          <t>168j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (29/06/2026)</t>
+          <t>Valide 61j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 223j (07/12/2026)</t>
+          <t>Valide 222j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (09/10/2026)</t>
+          <t>Valide 163j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>164j</t>
+          <t>163j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 216j (30/11/2026)</t>
+          <t>Valide 215j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 287j (09/02/2027)</t>
+          <t>Valide 286j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>287j</t>
+          <t>286j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 206j (20/11/2026)</t>
+          <t>Valide 205j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 235j (19/12/2026)</t>
+          <t>Valide 234j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>235j</t>
+          <t>234j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 94j (31/07/2026)</t>
+          <t>Valide 93j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (13/10/2026)</t>
+          <t>Valide 167j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>168j</t>
+          <t>167j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (10/10/2026)</t>
+          <t>Valide 164j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>28/04/2026 09:26</t>
+          <t>29/04/2026 09:12</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 30/04/2026 09:24
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (14/07/2026)</t>
+          <t>Valide 74j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>[Errno -2] Name or service not known</t>
+          <t>Valide 308j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 100j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>100j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 99j (07/08/2026)</t>
+          <t>Valide 98j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (05/07/2026)</t>
+          <t>Valide 65j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>[Errno -2] Name or service not known</t>
+          <t>Valide 270j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 21j (20/05/2026)</t>
+          <t>Expire dans 20j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>21j</t>
+          <t>20j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (02/11/2026)</t>
+          <t>Valide 186j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 286j (09/02/2027)</t>
+          <t>Valide 285j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>286j</t>
+          <t>285j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 305j (28/02/2027)</t>
+          <t>Valide 304j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (14/06/2026)</t>
+          <t>Valide 45j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 98j (05/08/2026)</t>
+          <t>Valide 97j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>98j</t>
+          <t>97j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (22/07/2026)</t>
+          <t>Valide 83j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (14/10/2026)</t>
+          <t>Valide 167j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>168j</t>
+          <t>167j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (29/06/2026)</t>
+          <t>Valide 60j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 222j (07/12/2026)</t>
+          <t>Valide 221j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (09/10/2026)</t>
+          <t>Valide 162j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>163j</t>
+          <t>162j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 215j (30/11/2026)</t>
+          <t>Valide 214j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 286j (09/02/2027)</t>
+          <t>Valide 285j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>286j</t>
+          <t>285j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 205j (20/11/2026)</t>
+          <t>Valide 204j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 234j (19/12/2026)</t>
+          <t>Valide 233j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>234j</t>
+          <t>233j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 93j (31/07/2026)</t>
+          <t>Valide 92j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (13/10/2026)</t>
+          <t>Valide 166j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>167j</t>
+          <t>166j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (10/10/2026)</t>
+          <t>Valide 163j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>29/04/2026 09:12</t>
+          <t>30/04/2026 09:17</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 01/05/2026 09:08
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (14/07/2026)</t>
+          <t>Valide 73j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 308j (05/03/2027)</t>
+          <t>Valide 307j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 98j (07/08/2026)</t>
+          <t>Valide 97j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (05/07/2026)</t>
+          <t>Valide 64j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 270j (26/01/2027)</t>
+          <t>Valide 269j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 20j (20/05/2026)</t>
+          <t>Expire dans 19j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>20j</t>
+          <t>19j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 186j (02/11/2026)</t>
+          <t>Valide 185j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 285j (09/02/2027)</t>
+          <t>Valide 284j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>285j</t>
+          <t>284j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 304j (28/02/2027)</t>
+          <t>Valide 303j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (14/06/2026)</t>
+          <t>Valide 44j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 97j (05/08/2026)</t>
+          <t>Valide 96j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>97j</t>
+          <t>96j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 83j (22/07/2026)</t>
+          <t>Valide 82j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (14/10/2026)</t>
+          <t>Valide 166j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>167j</t>
+          <t>166j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1810,30 +1810,34 @@
       </c>
       <c r="K26" s="9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (29/06/2026)</t>
+          <t>Valide 59j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 221j (07/12/2026)</t>
+          <t>Valide 220j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr"/>
+          <t>01/05/2026 09:03</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="3" t="inlineStr">
@@ -2001,22 +2005,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (09/10/2026)</t>
+          <t>Valide 161j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>162j</t>
+          <t>161j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 214j (30/11/2026)</t>
+          <t>Valide 213j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2207,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 285j (09/02/2027)</t>
+          <t>Valide 284j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>285j</t>
+          <t>284j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 204j (20/11/2026)</t>
+          <t>Valide 203j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2453,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 233j (19/12/2026)</t>
+          <t>Valide 232j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>233j</t>
+          <t>232j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 92j (31/07/2026)</t>
+          <t>Valide 91j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2695,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (13/10/2026)</t>
+          <t>Valide 165j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>166j</t>
+          <t>165j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (10/10/2026)</t>
+          <t>Valide 162j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>30/04/2026 09:17</t>
+          <t>01/05/2026 09:03</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 02/05/2026 08:27
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (14/07/2026)</t>
+          <t>Valide 72j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 307j (05/03/2027)</t>
+          <t>Valide 306j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 97j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>97j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 97j (07/08/2026)</t>
+          <t>Valide 96j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (05/07/2026)</t>
+          <t>Valide 63j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 269j (26/01/2027)</t>
+          <t>Valide 268j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 19j (20/05/2026)</t>
+          <t>Expire dans 18j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>19j</t>
+          <t>18j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (02/11/2026)</t>
+          <t>Valide 184j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 284j (09/02/2027)</t>
+          <t>Valide 283j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>284j</t>
+          <t>283j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 303j (28/02/2027)</t>
+          <t>Valide 302j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (14/06/2026)</t>
+          <t>[Errno -2] Name or service not known</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 96j (05/08/2026)</t>
+          <t>Valide 95j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>96j</t>
+          <t>95j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (22/07/2026)</t>
+          <t>[Errno -2] Name or service not known</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (14/10/2026)</t>
+          <t>Valide 165j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>166j</t>
+          <t>165j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (29/06/2026)</t>
+          <t>Valide 58j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 220j (07/12/2026)</t>
+          <t>Valide 219j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2005,22 +2005,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (09/10/2026)</t>
+          <t>Valide 160j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>161j</t>
+          <t>160j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 213j (30/11/2026)</t>
+          <t>[Errno -2] Name or service not known</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2207,22 +2207,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 284j (09/02/2027)</t>
+          <t>Valide 283j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>284j</t>
+          <t>283j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 203j (20/11/2026)</t>
+          <t>Valide 202j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2453,22 +2453,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 232j (19/12/2026)</t>
+          <t>Valide 231j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>232j</t>
+          <t>231j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 91j (31/07/2026)</t>
+          <t>Valide 90j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2695,22 +2695,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (13/10/2026)</t>
+          <t>Valide 164j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>165j</t>
+          <t>164j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (10/10/2026)</t>
+          <t>[Errno -2] Name or service not known</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>01/05/2026 09:03</t>
+          <t>02/05/2026 08:22</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 03/05/2026 08:54
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (14/07/2026)</t>
+          <t>Valide 71j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 306j (05/03/2027)</t>
+          <t>Valide 305j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 97j (07/08/2026)</t>
+          <t>Valide 96j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>97j</t>
+          <t>96j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 96j (07/08/2026)</t>
+          <t>Valide 95j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (05/07/2026)</t>
+          <t>Valide 62j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 268j (26/01/2027)</t>
+          <t>Valide 267j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 18j (20/05/2026)</t>
+          <t>Expire dans 17j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>18j</t>
+          <t>17j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 184j (02/11/2026)</t>
+          <t>Valide 183j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 283j (09/02/2027)</t>
+          <t>Valide 282j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>283j</t>
+          <t>282j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 302j (28/02/2027)</t>
+          <t>Valide 301j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>[Errno -2] Name or service not known</t>
+          <t>Valide 42j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 95j (05/08/2026)</t>
+          <t>Valide 94j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>95j</t>
+          <t>94j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>[Errno -2] Name or service not known</t>
+          <t>Valide 80j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (14/10/2026)</t>
+          <t>Valide 164j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>165j</t>
+          <t>164j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1810,34 +1810,30 @@
       </c>
       <c r="K26" s="9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (29/06/2026)</t>
+          <t>Valide 57j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 219j (07/12/2026)</t>
+          <t>Valide 218j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>03/05/2026 08:49</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="3" t="inlineStr">
@@ -2005,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (09/10/2026)</t>
+          <t>Valide 159j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>160j</t>
+          <t>159j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>[Errno -2] Name or service not known</t>
+          <t>Valide 211j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2207,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 283j (09/02/2027)</t>
+          <t>Valide 282j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>283j</t>
+          <t>282j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 202j (20/11/2026)</t>
+          <t>Valide 201j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2453,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 231j (19/12/2026)</t>
+          <t>Valide 230j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>231j</t>
+          <t>230j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 90j (31/07/2026)</t>
+          <t>Valide 89j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2695,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (13/10/2026)</t>
+          <t>Valide 163j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>164j</t>
+          <t>163j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>[Errno -2] Name or service not known</t>
+          <t>Valide 160j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>02/05/2026 08:22</t>
+          <t>03/05/2026 08:49</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 04/05/2026 09:28
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (14/07/2026)</t>
+          <t>Valide 70j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 305j (05/03/2027)</t>
+          <t>Valide 304j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 96j (07/08/2026)</t>
+          <t>Valide 95j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>96j</t>
+          <t>95j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 95j (07/08/2026)</t>
+          <t>Valide 94j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (05/07/2026)</t>
+          <t>Valide 61j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 267j (26/01/2027)</t>
+          <t>Valide 266j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 17j (20/05/2026)</t>
+          <t>Expire dans 16j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>17j</t>
+          <t>16j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (02/11/2026)</t>
+          <t>Valide 182j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 282j (09/02/2027)</t>
+          <t>Valide 281j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>282j</t>
+          <t>281j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 301j (28/02/2027)</t>
+          <t>Valide 300j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (14/06/2026)</t>
+          <t>Valide 41j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 94j (05/08/2026)</t>
+          <t>Valide 93j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>94j</t>
+          <t>93j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 80j (22/07/2026)</t>
+          <t>Valide 79j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (14/10/2026)</t>
+          <t>Valide 163j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>164j</t>
+          <t>163j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (29/06/2026)</t>
+          <t>Valide 56j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 218j (07/12/2026)</t>
+          <t>Valide 217j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (09/10/2026)</t>
+          <t>Valide 158j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>159j</t>
+          <t>158j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 211j (30/11/2026)</t>
+          <t>Valide 210j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 282j (09/02/2027)</t>
+          <t>Valide 281j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>282j</t>
+          <t>281j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 201j (20/11/2026)</t>
+          <t>Valide 200j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 230j (19/12/2026)</t>
+          <t>Valide 229j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>230j</t>
+          <t>229j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (31/07/2026)</t>
+          <t>Valide 88j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (13/10/2026)</t>
+          <t>Valide 162j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>163j</t>
+          <t>162j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (10/10/2026)</t>
+          <t>Valide 159j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>03/05/2026 08:49</t>
+          <t>04/05/2026 09:24</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 05/05/2026 09:16
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (14/07/2026)</t>
+          <t>Valide 69j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 304j (05/03/2027)</t>
+          <t>Valide 303j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 95j (07/08/2026)</t>
+          <t>Valide 94j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>95j</t>
+          <t>94j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 94j (07/08/2026)</t>
+          <t>Valide 93j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (05/07/2026)</t>
+          <t>Valide 60j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 266j (26/01/2027)</t>
+          <t>Valide 265j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 16j (20/05/2026)</t>
+          <t>Expire dans 15j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>16j</t>
+          <t>15j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (02/11/2026)</t>
+          <t>Valide 181j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 281j (09/02/2027)</t>
+          <t>Valide 280j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>281j</t>
+          <t>280j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 300j (28/02/2027)</t>
+          <t>Valide 299j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (14/06/2026)</t>
+          <t>Valide 40j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 93j (05/08/2026)</t>
+          <t>Valide 92j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>93j</t>
+          <t>92j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (22/07/2026)</t>
+          <t>Valide 78j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (14/10/2026)</t>
+          <t>Valide 162j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>163j</t>
+          <t>162j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (29/06/2026)</t>
+          <t>Valide 55j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 217j (07/12/2026)</t>
+          <t>Valide 216j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (09/10/2026)</t>
+          <t>Valide 157j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>158j</t>
+          <t>157j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 210j (30/11/2026)</t>
+          <t>Valide 209j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 281j (09/02/2027)</t>
+          <t>Valide 280j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>281j</t>
+          <t>280j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 200j (20/11/2026)</t>
+          <t>Valide 199j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 229j (19/12/2026)</t>
+          <t>Valide 228j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>229j</t>
+          <t>228j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 88j (31/07/2026)</t>
+          <t>Valide 87j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (13/10/2026)</t>
+          <t>Valide 161j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>162j</t>
+          <t>161j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (10/10/2026)</t>
+          <t>Valide 158j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>04/05/2026 09:24</t>
+          <t>05/05/2026 09:09</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 06/05/2026 09:32
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (14/07/2026)</t>
+          <t>Valide 68j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 303j (05/03/2027)</t>
+          <t>Valide 302j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 94j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>94j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 93j (07/08/2026)</t>
+          <t>Valide 92j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (05/07/2026)</t>
+          <t>Valide 59j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 265j (26/01/2027)</t>
+          <t>Valide 264j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 15j (20/05/2026)</t>
+          <t>Expire dans 14j (20/05/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>15j</t>
+          <t>14j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (02/11/2026)</t>
+          <t>Valide 180j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 280j (09/02/2027)</t>
+          <t>Valide 279j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>280j</t>
+          <t>279j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 299j (28/02/2027)</t>
+          <t>Valide 298j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (14/06/2026)</t>
+          <t>Valide 39j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 92j (05/08/2026)</t>
+          <t>Valide 91j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>92j</t>
+          <t>91j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (22/07/2026)</t>
+          <t>Valide 77j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (14/10/2026)</t>
+          <t>Valide 161j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>162j</t>
+          <t>161j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (29/06/2026)</t>
+          <t>Valide 54j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 216j (07/12/2026)</t>
+          <t>Valide 215j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (09/10/2026)</t>
+          <t>Valide 156j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>157j</t>
+          <t>156j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 209j (30/11/2026)</t>
+          <t>Valide 208j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 280j (09/02/2027)</t>
+          <t>Valide 279j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>280j</t>
+          <t>279j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 199j (20/11/2026)</t>
+          <t>Valide 198j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 228j (19/12/2026)</t>
+          <t>Valide 227j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>228j</t>
+          <t>227j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (31/07/2026)</t>
+          <t>Valide 86j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (13/10/2026)</t>
+          <t>Valide 160j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>161j</t>
+          <t>160j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (10/10/2026)</t>
+          <t>Valide 157j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>05/05/2026 09:09</t>
+          <t>06/05/2026 09:27</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 07/05/2026 09:41
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (14/07/2026)</t>
+          <t>Valide 67j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 302j (05/03/2027)</t>
+          <t>Valide 301j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 92j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>92j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 92j (07/08/2026)</t>
+          <t>Valide 91j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (05/07/2026)</t>
+          <t>Valide 58j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 264j (26/01/2027)</t>
+          <t>Valide 263j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,29 +1152,25 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 14j (20/05/2026)</t>
+          <t>Valide 197j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>14j</t>
+          <t>197j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (02/11/2026)</t>
+          <t>Valide 179j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>07/05/2026 09:36</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1262,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 279j (09/02/2027)</t>
+          <t>Valide 278j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>279j</t>
+          <t>278j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 298j (28/02/2027)</t>
+          <t>Valide 297j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (14/06/2026)</t>
+          <t>Valide 38j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 91j (05/08/2026)</t>
+          <t>Valide 90j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>91j</t>
+          <t>90j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (22/07/2026)</t>
+          <t>Valide 76j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (14/10/2026)</t>
+          <t>Valide 160j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>161j</t>
+          <t>160j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (29/06/2026)</t>
+          <t>Valide 53j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 215j (07/12/2026)</t>
+          <t>Valide 214j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (09/10/2026)</t>
+          <t>Valide 155j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>156j</t>
+          <t>155j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 208j (30/11/2026)</t>
+          <t>Valide 207j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 279j (09/02/2027)</t>
+          <t>Valide 278j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>279j</t>
+          <t>278j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 198j (20/11/2026)</t>
+          <t>Valide 197j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 227j (19/12/2026)</t>
+          <t>Valide 226j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>227j</t>
+          <t>226j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (31/07/2026)</t>
+          <t>Valide 85j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (13/10/2026)</t>
+          <t>Valide 159j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>160j</t>
+          <t>159j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (10/10/2026)</t>
+          <t>Valide 156j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>06/05/2026 09:27</t>
+          <t>07/05/2026 09:36</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 08/05/2026 08:28
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (14/07/2026)</t>
+          <t>Valide 66j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 301j (05/03/2027)</t>
+          <t>Valide 300j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 92j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>92j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 91j (07/08/2026)</t>
+          <t>Valide 90j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (05/07/2026)</t>
+          <t>Valide 57j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 263j (26/01/2027)</t>
+          <t>Valide 262j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (20/11/2026)</t>
+          <t>Valide 196j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>197j</t>
+          <t>196j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (02/11/2026)</t>
+          <t>Valide 178j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 278j (09/02/2027)</t>
+          <t>Valide 277j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>278j</t>
+          <t>277j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 297j (28/02/2027)</t>
+          <t>Valide 296j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (14/06/2026)</t>
+          <t>Valide 37j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 90j (05/08/2026)</t>
+          <t>Valide 89j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>90j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (22/07/2026)</t>
+          <t>Valide 75j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (14/10/2026)</t>
+          <t>Valide 159j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>160j</t>
+          <t>159j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (29/06/2026)</t>
+          <t>Valide 52j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 214j (07/12/2026)</t>
+          <t>Valide 213j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (09/10/2026)</t>
+          <t>Valide 154j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>155j</t>
+          <t>154j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 207j (30/11/2026)</t>
+          <t>Valide 206j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 278j (09/02/2027)</t>
+          <t>Valide 277j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>278j</t>
+          <t>277j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (20/11/2026)</t>
+          <t>Valide 196j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 226j (19/12/2026)</t>
+          <t>Valide 225j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>226j</t>
+          <t>225j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (31/07/2026)</t>
+          <t>Valide 84j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (13/10/2026)</t>
+          <t>Valide 158j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>159j</t>
+          <t>158j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (10/10/2026)</t>
+          <t>Valide 155j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>07/05/2026 09:36</t>
+          <t>08/05/2026 08:22</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 09/05/2026 08:47
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (14/07/2026)</t>
+          <t>Valide 65j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 300j (05/03/2027)</t>
+          <t>Valide 299j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 90j (07/08/2026)</t>
+          <t>Valide 89j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (05/07/2026)</t>
+          <t>Valide 56j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 262j (26/01/2027)</t>
+          <t>Valide 261j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (20/11/2026)</t>
+          <t>Valide 195j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>196j</t>
+          <t>195j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (02/11/2026)</t>
+          <t>Valide 177j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 277j (09/02/2027)</t>
+          <t>Valide 276j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>277j</t>
+          <t>276j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 296j (28/02/2027)</t>
+          <t>Valide 295j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (14/06/2026)</t>
+          <t>Valide 36j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (05/08/2026)</t>
+          <t>Valide 88j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (22/07/2026)</t>
+          <t>Valide 74j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (14/10/2026)</t>
+          <t>Valide 158j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>159j</t>
+          <t>158j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (29/06/2026)</t>
+          <t>Valide 51j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 213j (07/12/2026)</t>
+          <t>Valide 212j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (09/10/2026)</t>
+          <t>Valide 153j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>154j</t>
+          <t>153j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 206j (30/11/2026)</t>
+          <t>Valide 205j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 277j (09/02/2027)</t>
+          <t>Valide 276j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>277j</t>
+          <t>276j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (20/11/2026)</t>
+          <t>Valide 195j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 225j (19/12/2026)</t>
+          <t>Valide 224j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>225j</t>
+          <t>224j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (31/07/2026)</t>
+          <t>Valide 83j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (13/10/2026)</t>
+          <t>Valide 157j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>158j</t>
+          <t>157j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (10/10/2026)</t>
+          <t>Valide 154j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>08/05/2026 08:22</t>
+          <t>09/05/2026 08:43</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 10/05/2026 09:01
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (14/07/2026)</t>
+          <t>Valide 64j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 299j (05/03/2027)</t>
+          <t>Valide 298j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 89j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (07/08/2026)</t>
+          <t>Valide 88j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (05/07/2026)</t>
+          <t>Valide 55j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 261j (26/01/2027)</t>
+          <t>Valide 260j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (20/11/2026)</t>
+          <t>Valide 194j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>195j</t>
+          <t>194j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (02/11/2026)</t>
+          <t>Valide 176j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 276j (09/02/2027)</t>
+          <t>Valide 275j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>276j</t>
+          <t>275j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 295j (28/02/2027)</t>
+          <t>Valide 294j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (14/06/2026)</t>
+          <t>Valide 35j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 88j (05/08/2026)</t>
+          <t>Valide 87j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 74j (22/07/2026)</t>
+          <t>Valide 73j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (14/10/2026)</t>
+          <t>Valide 157j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>158j</t>
+          <t>157j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (29/06/2026)</t>
+          <t>Valide 50j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 212j (07/12/2026)</t>
+          <t>Valide 211j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (09/10/2026)</t>
+          <t>Valide 152j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>153j</t>
+          <t>152j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 205j (30/11/2026)</t>
+          <t>Valide 204j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 276j (09/02/2027)</t>
+          <t>Valide 275j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>276j</t>
+          <t>275j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (20/11/2026)</t>
+          <t>Valide 194j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 224j (19/12/2026)</t>
+          <t>Valide 223j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>224j</t>
+          <t>223j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 83j (31/07/2026)</t>
+          <t>Valide 82j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (13/10/2026)</t>
+          <t>Valide 156j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>157j</t>
+          <t>156j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (10/10/2026)</t>
+          <t>Valide 153j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>09/05/2026 08:43</t>
+          <t>10/05/2026 08:57</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 11/05/2026 10:44
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (14/07/2026)</t>
+          <t>Valide 63j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 298j (05/03/2027)</t>
+          <t>Valide 297j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 88j (07/08/2026)</t>
+          <t>Valide 87j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (05/07/2026)</t>
+          <t>Valide 54j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 260j (26/01/2027)</t>
+          <t>Valide 259j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (20/11/2026)</t>
+          <t>Valide 193j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>194j</t>
+          <t>193j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (02/11/2026)</t>
+          <t>Valide 175j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 275j (09/02/2027)</t>
+          <t>Valide 274j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>275j</t>
+          <t>274j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 294j (28/02/2027)</t>
+          <t>Valide 293j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (14/06/2026)</t>
+          <t>Valide 34j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (05/08/2026)</t>
+          <t>Valide 86j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (22/07/2026)</t>
+          <t>Valide 72j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (14/10/2026)</t>
+          <t>Valide 156j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>157j</t>
+          <t>156j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (29/06/2026)</t>
+          <t>Valide 49j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 211j (07/12/2026)</t>
+          <t>Valide 210j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (09/10/2026)</t>
+          <t>Valide 151j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>152j</t>
+          <t>151j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 204j (30/11/2026)</t>
+          <t>Valide 203j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 275j (09/02/2027)</t>
+          <t>Valide 274j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>275j</t>
+          <t>274j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (20/11/2026)</t>
+          <t>Valide 193j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 223j (19/12/2026)</t>
+          <t>Valide 222j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>223j</t>
+          <t>222j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (31/07/2026)</t>
+          <t>Valide 81j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (13/10/2026)</t>
+          <t>Valide 155j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>156j</t>
+          <t>155j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (10/10/2026)</t>
+          <t>Valide 152j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>10/05/2026 08:57</t>
+          <t>11/05/2026 10:39</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 12/05/2026 09:48
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (14/07/2026)</t>
+          <t>Valide 62j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 297j (05/03/2027)</t>
+          <t>Valide 296j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 87j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (07/08/2026)</t>
+          <t>Valide 86j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (05/07/2026)</t>
+          <t>Valide 53j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 259j (26/01/2027)</t>
+          <t>Valide 258j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (20/11/2026)</t>
+          <t>Valide 192j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>193j</t>
+          <t>192j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (02/11/2026)</t>
+          <t>Valide 174j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 274j (09/02/2027)</t>
+          <t>Valide 273j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>274j</t>
+          <t>273j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 293j (28/02/2027)</t>
+          <t>Valide 292j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (14/06/2026)</t>
+          <t>Valide 33j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (05/08/2026)</t>
+          <t>Valide 85j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (22/07/2026)</t>
+          <t>Valide 71j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (14/10/2026)</t>
+          <t>Valide 155j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>156j</t>
+          <t>155j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (29/06/2026)</t>
+          <t>Valide 48j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 210j (07/12/2026)</t>
+          <t>Valide 209j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (09/10/2026)</t>
+          <t>Valide 150j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>151j</t>
+          <t>150j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 203j (30/11/2026)</t>
+          <t>Valide 202j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 274j (09/02/2027)</t>
+          <t>Valide 273j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>274j</t>
+          <t>273j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (20/11/2026)</t>
+          <t>Valide 192j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 222j (19/12/2026)</t>
+          <t>Valide 221j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>222j</t>
+          <t>221j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 81j (31/07/2026)</t>
+          <t>Valide 80j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (13/10/2026)</t>
+          <t>Valide 154j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>155j</t>
+          <t>154j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (10/10/2026)</t>
+          <t>Valide 151j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>11/05/2026 10:39</t>
+          <t>12/05/2026 09:43</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 13/05/2026 09:52
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (14/07/2026)</t>
+          <t>Valide 61j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 296j (05/03/2027)</t>
+          <t>Valide 295j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (07/08/2026)</t>
+          <t>Valide 86j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (07/08/2026)</t>
+          <t>Valide 85j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (05/07/2026)</t>
+          <t>Valide 52j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 258j (26/01/2027)</t>
+          <t>Valide 257j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (20/11/2026)</t>
+          <t>Valide 191j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>192j</t>
+          <t>191j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (02/11/2026)</t>
+          <t>Valide 173j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 273j (09/02/2027)</t>
+          <t>Valide 272j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>273j</t>
+          <t>272j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 292j (28/02/2027)</t>
+          <t>Valide 291j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (14/06/2026)</t>
+          <t>Valide 32j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (05/08/2026)</t>
+          <t>Valide 84j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (22/07/2026)</t>
+          <t>Valide 70j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (14/10/2026)</t>
+          <t>Valide 154j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>155j</t>
+          <t>154j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (29/06/2026)</t>
+          <t>Valide 47j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 209j (07/12/2026)</t>
+          <t>Valide 208j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (09/10/2026)</t>
+          <t>Valide 149j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>150j</t>
+          <t>149j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 202j (30/11/2026)</t>
+          <t>Valide 201j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 273j (09/02/2027)</t>
+          <t>Valide 272j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>273j</t>
+          <t>272j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (20/11/2026)</t>
+          <t>Valide 191j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 221j (19/12/2026)</t>
+          <t>Valide 220j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>221j</t>
+          <t>220j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 80j (31/07/2026)</t>
+          <t>Valide 79j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (13/10/2026)</t>
+          <t>Valide 153j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>154j</t>
+          <t>153j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (10/10/2026)</t>
+          <t>Valide 150j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>12/05/2026 09:43</t>
+          <t>13/05/2026 09:46</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 14/05/2026 09:41
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (14/07/2026)</t>
+          <t>Valide 60j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 295j (05/03/2027)</t>
+          <t>Valide 294j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (07/08/2026)</t>
+          <t>Valide 85j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (07/08/2026)</t>
+          <t>Valide 84j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (05/07/2026)</t>
+          <t>Valide 51j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 257j (26/01/2027)</t>
+          <t>Valide 256j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (20/11/2026)</t>
+          <t>Valide 190j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>191j</t>
+          <t>190j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (02/11/2026)</t>
+          <t>Valide 172j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 272j (09/02/2027)</t>
+          <t>Valide 271j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>272j</t>
+          <t>271j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 291j (28/02/2027)</t>
+          <t>Valide 290j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (14/06/2026)</t>
+          <t>Valide 31j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (05/08/2026)</t>
+          <t>Valide 83j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (22/07/2026)</t>
+          <t>Valide 69j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (14/10/2026)</t>
+          <t>Valide 153j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>154j</t>
+          <t>153j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (29/06/2026)</t>
+          <t>Valide 46j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 208j (07/12/2026)</t>
+          <t>Valide 207j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (09/10/2026)</t>
+          <t>Valide 148j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>149j</t>
+          <t>148j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 201j (30/11/2026)</t>
+          <t>Valide 200j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 272j (09/02/2027)</t>
+          <t>Valide 271j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>272j</t>
+          <t>271j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (20/11/2026)</t>
+          <t>Valide 190j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 220j (19/12/2026)</t>
+          <t>Valide 219j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>220j</t>
+          <t>219j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (31/07/2026)</t>
+          <t>Valide 78j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (13/10/2026)</t>
+          <t>Valide 152j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>153j</t>
+          <t>152j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (10/10/2026)</t>
+          <t>Valide 149j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>13/05/2026 09:46</t>
+          <t>14/05/2026 09:36</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 15/05/2026 09:55
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (14/07/2026)</t>
+          <t>Valide 59j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 294j (05/03/2027)</t>
+          <t>Valide 293j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (07/08/2026)</t>
+          <t>Valide 84j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (07/08/2026)</t>
+          <t>Valide 83j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (05/07/2026)</t>
+          <t>Valide 50j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 256j (26/01/2027)</t>
+          <t>Valide 255j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (20/11/2026)</t>
+          <t>Valide 189j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>190j</t>
+          <t>189j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (02/11/2026)</t>
+          <t>Valide 171j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 271j (09/02/2027)</t>
+          <t>Valide 270j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>271j</t>
+          <t>270j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 290j (28/02/2027)</t>
+          <t>Valide 289j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,15 +1358,19 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (14/06/2026)</t>
+          <t>Expire dans 30j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr"/>
+          <t>15/05/2026 09:49</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="15" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A15" s="3" t="inlineStr">
@@ -1646,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 83j (05/08/2026)</t>
+          <t>Valide 82j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (22/07/2026)</t>
+          <t>Valide 68j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (14/10/2026)</t>
+          <t>Valide 152j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>153j</t>
+          <t>152j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (29/06/2026)</t>
+          <t>Valide 45j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 207j (07/12/2026)</t>
+          <t>Valide 206j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (09/10/2026)</t>
+          <t>Valide 147j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>148j</t>
+          <t>147j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 200j (30/11/2026)</t>
+          <t>Valide 199j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 271j (09/02/2027)</t>
+          <t>Valide 270j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>271j</t>
+          <t>270j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (20/11/2026)</t>
+          <t>Valide 189j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 219j (19/12/2026)</t>
+          <t>Valide 218j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>219j</t>
+          <t>218j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (31/07/2026)</t>
+          <t>Valide 77j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (13/10/2026)</t>
+          <t>Valide 151j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>152j</t>
+          <t>151j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (10/10/2026)</t>
+          <t>Valide 148j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>14/05/2026 09:36</t>
+          <t>15/05/2026 09:49</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 16/05/2026 08:55
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (14/07/2026)</t>
+          <t>Valide 58j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 293j (05/03/2027)</t>
+          <t>Valide 292j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 83j (07/08/2026)</t>
+          <t>Valide 82j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (05/07/2026)</t>
+          <t>Valide 49j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 255j (26/01/2027)</t>
+          <t>Valide 254j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (20/11/2026)</t>
+          <t>Valide 188j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>189j</t>
+          <t>188j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (02/11/2026)</t>
+          <t>Valide 170j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 270j (09/02/2027)</t>
+          <t>Valide 269j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>270j</t>
+          <t>269j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 289j (28/02/2027)</t>
+          <t>Valide 288j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (14/06/2026)</t>
+          <t>Expire dans 29j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (05/08/2026)</t>
+          <t>Valide 81j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (22/07/2026)</t>
+          <t>Valide 67j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (14/10/2026)</t>
+          <t>Valide 151j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>152j</t>
+          <t>151j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (29/06/2026)</t>
+          <t>Valide 44j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 206j (07/12/2026)</t>
+          <t>Valide 205j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (09/10/2026)</t>
+          <t>Valide 146j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>147j</t>
+          <t>146j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 199j (30/11/2026)</t>
+          <t>Valide 198j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 270j (09/02/2027)</t>
+          <t>Valide 269j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>270j</t>
+          <t>269j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (20/11/2026)</t>
+          <t>Valide 188j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 218j (19/12/2026)</t>
+          <t>Valide 217j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>218j</t>
+          <t>217j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (31/07/2026)</t>
+          <t>Valide 76j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (13/10/2026)</t>
+          <t>Valide 150j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>151j</t>
+          <t>150j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (10/10/2026)</t>
+          <t>Valide 147j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>15/05/2026 09:49</t>
+          <t>16/05/2026 08:50</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 17/05/2026 09:13
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (14/07/2026)</t>
+          <t>Valide 57j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 292j (05/03/2027)</t>
+          <t>Valide 291j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 82j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (07/08/2026)</t>
+          <t>Valide 81j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (05/07/2026)</t>
+          <t>Valide 48j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 254j (26/01/2027)</t>
+          <t>Valide 253j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (20/11/2026)</t>
+          <t>Valide 187j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>188j</t>
+          <t>187j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (02/11/2026)</t>
+          <t>Valide 169j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 269j (09/02/2027)</t>
+          <t>Valide 268j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>269j</t>
+          <t>268j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 288j (28/02/2027)</t>
+          <t>Valide 287j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (14/06/2026)</t>
+          <t>Expire dans 28j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 81j (05/08/2026)</t>
+          <t>Valide 80j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (22/07/2026)</t>
+          <t>Valide 66j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (14/10/2026)</t>
+          <t>Valide 150j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>151j</t>
+          <t>150j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (29/06/2026)</t>
+          <t>Valide 43j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 205j (07/12/2026)</t>
+          <t>Valide 204j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (09/10/2026)</t>
+          <t>Valide 145j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>146j</t>
+          <t>145j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 198j (30/11/2026)</t>
+          <t>Valide 197j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 269j (09/02/2027)</t>
+          <t>Valide 268j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>269j</t>
+          <t>268j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (20/11/2026)</t>
+          <t>Valide 187j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 217j (19/12/2026)</t>
+          <t>Valide 216j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>217j</t>
+          <t>216j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (31/07/2026)</t>
+          <t>Valide 75j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (13/10/2026)</t>
+          <t>Valide 149j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>150j</t>
+          <t>149j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (10/10/2026)</t>
+          <t>Valide 146j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>16/05/2026 08:50</t>
+          <t>17/05/2026 09:08</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 18/05/2026 14:43
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (14/07/2026)</t>
+          <t>Valide 56j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 291j (05/03/2027)</t>
+          <t>Valide 290j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (07/08/2026)</t>
+          <t>Valide 81j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 81j (07/08/2026)</t>
+          <t>Valide 80j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (05/07/2026)</t>
+          <t>Valide 47j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 253j (26/01/2027)</t>
+          <t>Valide 252j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (20/11/2026)</t>
+          <t>Valide 186j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>187j</t>
+          <t>186j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (02/11/2026)</t>
+          <t>Valide 167j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 268j (09/02/2027)</t>
+          <t>Valide 267j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>268j</t>
+          <t>267j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 287j (28/02/2027)</t>
+          <t>Valide 285j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 28j (14/06/2026)</t>
+          <t>Expire dans 26j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 80j (05/08/2026)</t>
+          <t>Valide 79j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (22/07/2026)</t>
+          <t>Valide 64j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (14/10/2026)</t>
+          <t>Valide 149j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>150j</t>
+          <t>149j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (29/06/2026)</t>
+          <t>Valide 42j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 204j (07/12/2026)</t>
+          <t>Valide 203j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (09/10/2026)</t>
+          <t>Valide 144j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>145j</t>
+          <t>144j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (30/11/2026)</t>
+          <t>Valide 196j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 268j (09/02/2027)</t>
+          <t>Valide 267j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>268j</t>
+          <t>267j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (20/11/2026)</t>
+          <t>Valide 186j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 216j (19/12/2026)</t>
+          <t>Valide 215j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>216j</t>
+          <t>215j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (31/07/2026)</t>
+          <t>Valide 73j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (13/10/2026)</t>
+          <t>Valide 148j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>149j</t>
+          <t>148j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (10/10/2026)</t>
+          <t>Valide 144j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>17/05/2026 09:08</t>
+          <t>18/05/2026 14:38</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 19/05/2026 10:43
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (14/07/2026)</t>
+          <t>Valide 55j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 290j (05/03/2027)</t>
+          <t>Valide 289j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 81j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 80j (07/08/2026)</t>
+          <t>Valide 79j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (05/07/2026)</t>
+          <t>Valide 46j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 252j (26/01/2027)</t>
+          <t>Valide 251j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 186j (20/11/2026)</t>
+          <t>Valide 185j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>186j</t>
+          <t>185j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,12 +1258,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 267j (09/02/2027)</t>
+          <t>Valide 266j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>267j</t>
+          <t>266j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1363,14 +1363,10 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>19/05/2026 10:38</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A15" s="3" t="inlineStr">
@@ -1650,12 +1646,12 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (05/08/2026)</t>
+          <t>Valide 78j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
@@ -1665,7 +1661,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (14/10/2026)</t>
+          <t>Valide 148j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>149j</t>
+          <t>148j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (29/06/2026)</t>
+          <t>Valide 41j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 203j (07/12/2026)</t>
+          <t>Valide 202j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (09/10/2026)</t>
+          <t>Valide 143j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>144j</t>
+          <t>143j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (30/11/2026)</t>
+          <t>Valide 195j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 267j (09/02/2027)</t>
+          <t>Valide 266j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>267j</t>
+          <t>266j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 186j (20/11/2026)</t>
+          <t>Valide 185j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,12 +2445,12 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 215j (19/12/2026)</t>
+          <t>Valide 214j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>215j</t>
+          <t>214j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
@@ -2464,7 +2460,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,12 +2687,12 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (13/10/2026)</t>
+          <t>Valide 147j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>148j</t>
+          <t>147j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
@@ -2706,7 +2702,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>18/05/2026 14:38</t>
+          <t>19/05/2026 10:38</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 20/05/2026 10:30
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (14/07/2026)</t>
+          <t>Valide 54j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 289j (05/03/2027)</t>
+          <t>Valide 288j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 79j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (07/08/2026)</t>
+          <t>Valide 78j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (05/07/2026)</t>
+          <t>Valide 45j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 251j (26/01/2027)</t>
+          <t>Valide 250j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (20/11/2026)</t>
+          <t>Valide 184j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>185j</t>
+          <t>184j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (02/11/2026)</t>
+          <t>Valide 166j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 266j (09/02/2027)</t>
+          <t>Valide 265j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>266j</t>
+          <t>265j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 285j (28/02/2027)</t>
+          <t>Valide 284j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 26j (14/06/2026)</t>
+          <t>Expire dans 25j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (05/08/2026)</t>
+          <t>Valide 77j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (22/07/2026)</t>
+          <t>Valide 63j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (14/10/2026)</t>
+          <t>Valide 147j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>148j</t>
+          <t>147j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (29/06/2026)</t>
+          <t>Valide 40j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 202j (07/12/2026)</t>
+          <t>Valide 201j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (09/10/2026)</t>
+          <t>Valide 142j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>143j</t>
+          <t>142j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (30/11/2026)</t>
+          <t>Valide 194j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 266j (09/02/2027)</t>
+          <t>Valide 265j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>266j</t>
+          <t>265j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (20/11/2026)</t>
+          <t>Valide 184j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 214j (19/12/2026)</t>
+          <t>Valide 213j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>214j</t>
+          <t>213j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (31/07/2026)</t>
+          <t>Valide 72j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (13/10/2026)</t>
+          <t>Valide 146j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>147j</t>
+          <t>146j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (10/10/2026)</t>
+          <t>Valide 143j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>19/05/2026 10:38</t>
+          <t>20/05/2026 10:25</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 21/05/2026 10:46
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (14/07/2026)</t>
+          <t>Valide 53j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 288j (05/03/2027)</t>
+          <t>Valide 287j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (07/08/2026)</t>
+          <t>Valide 78j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (07/08/2026)</t>
+          <t>Valide 77j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (05/07/2026)</t>
+          <t>Valide 44j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 250j (26/01/2027)</t>
+          <t>Valide 249j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 184j (20/11/2026)</t>
+          <t>Valide 183j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>184j</t>
+          <t>183j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (02/11/2026)</t>
+          <t>Valide 165j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 265j (09/02/2027)</t>
+          <t>Valide 264j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>265j</t>
+          <t>264j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 284j (28/02/2027)</t>
+          <t>Valide 283j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 25j (14/06/2026)</t>
+          <t>Expire dans 24j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (05/08/2026)</t>
+          <t>Valide 76j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (22/07/2026)</t>
+          <t>Valide 62j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (14/10/2026)</t>
+          <t>Valide 146j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>147j</t>
+          <t>146j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (29/06/2026)</t>
+          <t>Valide 39j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 201j (07/12/2026)</t>
+          <t>Valide 200j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (09/10/2026)</t>
+          <t>Valide 141j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>142j</t>
+          <t>141j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (30/11/2026)</t>
+          <t>Valide 193j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 265j (09/02/2027)</t>
+          <t>Valide 264j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>265j</t>
+          <t>264j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 184j (20/11/2026)</t>
+          <t>Valide 183j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 213j (19/12/2026)</t>
+          <t>Valide 212j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>213j</t>
+          <t>212j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (31/07/2026)</t>
+          <t>Valide 71j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (13/10/2026)</t>
+          <t>Valide 145j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>146j</t>
+          <t>145j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (10/10/2026)</t>
+          <t>Valide 142j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>20/05/2026 10:25</t>
+          <t>21/05/2026 10:41</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 22/05/2026 10:30
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (14/07/2026)</t>
+          <t>Valide 52j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 287j (05/03/2027)</t>
+          <t>Valide 286j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (07/08/2026)</t>
+          <t>Valide 76j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (05/07/2026)</t>
+          <t>Valide 43j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 249j (26/01/2027)</t>
+          <t>Valide 248j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (20/11/2026)</t>
+          <t>Valide 182j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>183j</t>
+          <t>182j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (02/11/2026)</t>
+          <t>Valide 164j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 264j (09/02/2027)</t>
+          <t>Valide 263j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>264j</t>
+          <t>263j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 283j (28/02/2027)</t>
+          <t>Valide 282j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 24j (14/06/2026)</t>
+          <t>Expire dans 23j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (05/08/2026)</t>
+          <t>Valide 75j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (22/07/2026)</t>
+          <t>Valide 61j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (14/10/2026)</t>
+          <t>Valide 145j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>146j</t>
+          <t>145j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (29/06/2026)</t>
+          <t>Valide 38j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 200j (07/12/2026)</t>
+          <t>Valide 199j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (09/10/2026)</t>
+          <t>Valide 140j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>141j</t>
+          <t>140j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (30/11/2026)</t>
+          <t>Valide 192j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 264j (09/02/2027)</t>
+          <t>Valide 263j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>264j</t>
+          <t>263j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (20/11/2026)</t>
+          <t>Valide 182j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 212j (19/12/2026)</t>
+          <t>Valide 211j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>212j</t>
+          <t>211j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (31/07/2026)</t>
+          <t>Valide 70j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (13/10/2026)</t>
+          <t>Valide 144j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>145j</t>
+          <t>144j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (10/10/2026)</t>
+          <t>Valide 141j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>21/05/2026 10:41</t>
+          <t>22/05/2026 10:25</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 23/05/2026 09:08
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (14/07/2026)</t>
+          <t>Valide 51j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 286j (05/03/2027)</t>
+          <t>Valide 285j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 76j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (07/08/2026)</t>
+          <t>Valide 75j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (05/07/2026)</t>
+          <t>Valide 42j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 248j (26/01/2027)</t>
+          <t>Valide 247j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (20/11/2026)</t>
+          <t>Valide 181j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>182j</t>
+          <t>181j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (02/11/2026)</t>
+          <t>Valide 163j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 263j (09/02/2027)</t>
+          <t>Valide 262j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>263j</t>
+          <t>262j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 282j (28/02/2027)</t>
+          <t>Valide 281j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 23j (14/06/2026)</t>
+          <t>Expire dans 22j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (05/08/2026)</t>
+          <t>Valide 74j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (22/07/2026)</t>
+          <t>Valide 60j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (14/10/2026)</t>
+          <t>Valide 144j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>145j</t>
+          <t>144j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (29/06/2026)</t>
+          <t>Valide 37j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 199j (07/12/2026)</t>
+          <t>Valide 198j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (09/10/2026)</t>
+          <t>Valide 139j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>140j</t>
+          <t>139j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (30/11/2026)</t>
+          <t>Valide 191j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 263j (09/02/2027)</t>
+          <t>Valide 262j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>263j</t>
+          <t>262j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (20/11/2026)</t>
+          <t>Valide 181j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 211j (19/12/2026)</t>
+          <t>Valide 210j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>211j</t>
+          <t>210j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (31/07/2026)</t>
+          <t>Valide 69j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (13/10/2026)</t>
+          <t>Valide 143j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>144j</t>
+          <t>143j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (10/10/2026)</t>
+          <t>Valide 140j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>22/05/2026 10:25</t>
+          <t>23/05/2026 09:03</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 24/05/2026 09:27
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (14/07/2026)</t>
+          <t>Valide 50j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 285j (05/03/2027)</t>
+          <t>Valide 284j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (07/08/2026)</t>
+          <t>Valide 74j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (05/07/2026)</t>
+          <t>Valide 41j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 247j (26/01/2027)</t>
+          <t>Valide 246j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (20/11/2026)</t>
+          <t>Valide 180j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>181j</t>
+          <t>180j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (02/11/2026)</t>
+          <t>Valide 162j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 262j (09/02/2027)</t>
+          <t>Valide 261j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>262j</t>
+          <t>261j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 281j (28/02/2027)</t>
+          <t>Valide 280j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 22j (14/06/2026)</t>
+          <t>Expire dans 21j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 74j (05/08/2026)</t>
+          <t>Valide 73j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 60j (22/07/2026)</t>
+          <t>Valide 59j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (14/10/2026)</t>
+          <t>Valide 143j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>144j</t>
+          <t>143j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (29/06/2026)</t>
+          <t>Valide 36j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 198j (07/12/2026)</t>
+          <t>Valide 197j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (09/10/2026)</t>
+          <t>Valide 138j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>139j</t>
+          <t>138j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (30/11/2026)</t>
+          <t>Valide 190j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 262j (09/02/2027)</t>
+          <t>Valide 261j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>262j</t>
+          <t>261j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (20/11/2026)</t>
+          <t>Valide 180j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 210j (19/12/2026)</t>
+          <t>Valide 209j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>210j</t>
+          <t>209j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (31/07/2026)</t>
+          <t>Valide 68j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (13/10/2026)</t>
+          <t>Valide 142j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>143j</t>
+          <t>142j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (10/10/2026)</t>
+          <t>Valide 139j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>23/05/2026 09:03</t>
+          <t>24/05/2026 09:22</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 25/05/2026 11:17
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (14/07/2026)</t>
+          <t>Valide 49j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 284j (05/03/2027)</t>
+          <t>Valide 283j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 74j (07/08/2026)</t>
+          <t>Valide 73j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (05/07/2026)</t>
+          <t>Valide 40j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 246j (26/01/2027)</t>
+          <t>Valide 245j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (20/11/2026)</t>
+          <t>Valide 179j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>179j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (02/11/2026)</t>
+          <t>Valide 161j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 261j (09/02/2027)</t>
+          <t>Valide 260j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>261j</t>
+          <t>260j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 280j (28/02/2027)</t>
+          <t>Valide 278j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 21j (14/06/2026)</t>
+          <t>Expire dans 20j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (05/08/2026)</t>
+          <t>Valide 72j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 59j (22/07/2026)</t>
+          <t>Valide 57j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (14/10/2026)</t>
+          <t>Valide 142j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>143j</t>
+          <t>142j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (29/06/2026)</t>
+          <t>Valide 35j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (07/12/2026)</t>
+          <t>Valide 196j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (09/10/2026)</t>
+          <t>Valide 137j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>138j</t>
+          <t>137j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (30/11/2026)</t>
+          <t>Valide 189j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 261j (09/02/2027)</t>
+          <t>Valide 260j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>261j</t>
+          <t>260j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (20/11/2026)</t>
+          <t>Valide 179j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 209j (19/12/2026)</t>
+          <t>Valide 208j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>209j</t>
+          <t>208j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (31/07/2026)</t>
+          <t>Valide 66j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (13/10/2026)</t>
+          <t>Valide 141j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>142j</t>
+          <t>141j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (10/10/2026)</t>
+          <t>Valide 138j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>24/05/2026 09:22</t>
+          <t>25/05/2026 11:13</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 26/05/2026 09:59
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (14/07/2026)</t>
+          <t>Valide 48j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 283j (05/03/2027)</t>
+          <t>Valide 282j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (07/08/2026)</t>
+          <t>Valide 72j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (05/07/2026)</t>
+          <t>Valide 39j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 245j (26/01/2027)</t>
+          <t>Valide 244j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (20/11/2026)</t>
+          <t>Valide 178j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>179j</t>
+          <t>178j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (02/11/2026)</t>
+          <t>Valide 160j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,12 +1258,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 260j (09/02/2027)</t>
+          <t>Valide 259j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>260j</t>
+          <t>259j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 20j (14/06/2026)</t>
+          <t>Expire dans 19j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,12 +1646,12 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (05/08/2026)</t>
+          <t>Valide 71j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (14/10/2026)</t>
+          <t>Valide 141j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>142j</t>
+          <t>141j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (29/06/2026)</t>
+          <t>Valide 34j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (07/12/2026)</t>
+          <t>Valide 195j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (09/10/2026)</t>
+          <t>Valide 136j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>137j</t>
+          <t>136j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (30/11/2026)</t>
+          <t>Valide 188j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 260j (09/02/2027)</t>
+          <t>Valide 259j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>260j</t>
+          <t>259j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (20/11/2026)</t>
+          <t>Valide 178j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,12 +2445,12 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 208j (19/12/2026)</t>
+          <t>Valide 207j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>208j</t>
+          <t>207j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (13/10/2026)</t>
+          <t>Valide 140j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>141j</t>
+          <t>140j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (10/10/2026)</t>
+          <t>Valide 137j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>25/05/2026 11:13</t>
+          <t>26/05/2026 09:53</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 26/05/2026 10:19
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -857,7 +857,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,12 +976,12 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 73j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>26/05/2026 09:53</t>
+          <t>26/05/2026 10:14</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 26/05/2026 14:21
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -857,7 +857,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -991,7 +991,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1162,12 +1162,12 @@
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (02/11/2026)</t>
+          <t>Valide 159j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1268,12 +1268,12 @@
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 278j (28/02/2027)</t>
+          <t>Valide 277j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 19j (14/06/2026)</t>
+          <t>Expire dans 18j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1656,12 +1656,12 @@
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 57j (22/07/2026)</t>
+          <t>Valide 56j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2455,12 +2455,12 @@
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (31/07/2026)</t>
+          <t>Valide 65j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2697,12 +2697,12 @@
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (10/10/2026)</t>
+          <t>Valide 136j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>26/05/2026 10:14</t>
+          <t>26/05/2026 14:15</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 26/05/2026 14:32
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -857,7 +857,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,12 +976,12 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2460,7 +2460,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2702,7 +2702,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>26/05/2026 14:15</t>
+          <t>26/05/2026 14:26</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 27/05/2026 11:02
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (14/07/2026)</t>
+          <t>Valide 47j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 282j (05/03/2027)</t>
+          <t>Valide 281j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (07/08/2026)</t>
+          <t>Valide 71j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (05/07/2026)</t>
+          <t>Valide 38j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 244j (26/01/2027)</t>
+          <t>Valide 243j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (20/11/2026)</t>
+          <t>Valide 177j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>178j</t>
+          <t>177j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 259j (09/02/2027)</t>
+          <t>Valide 258j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>259j</t>
+          <t>258j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 277j (28/02/2027)</t>
+          <t>Valide 276j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,12 +1646,12 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (05/08/2026)</t>
+          <t>Valide 70j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (14/10/2026)</t>
+          <t>Valide 140j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>141j</t>
+          <t>140j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (29/06/2026)</t>
+          <t>Valide 33j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (07/12/2026)</t>
+          <t>Valide 194j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (09/10/2026)</t>
+          <t>Valide 135j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>136j</t>
+          <t>135j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (30/11/2026)</t>
+          <t>Valide 187j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 259j (09/02/2027)</t>
+          <t>Valide 258j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>259j</t>
+          <t>258j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (20/11/2026)</t>
+          <t>Valide 177j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 207j (19/12/2026)</t>
+          <t>Valide 206j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>207j</t>
+          <t>206j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 65j (31/07/2026)</t>
+          <t>Valide 64j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,12 +2687,12 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (13/10/2026)</t>
+          <t>Valide 139j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>140j</t>
+          <t>139j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>26/05/2026 14:26</t>
+          <t>27/05/2026 10:57</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 28/05/2026 11:03
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (14/07/2026)</t>
+          <t>Valide 46j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 281j (05/03/2027)</t>
+          <t>Valide 280j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 71j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (07/08/2026)</t>
+          <t>Valide 70j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (05/07/2026)</t>
+          <t>Valide 37j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 243j (26/01/2027)</t>
+          <t>Valide 242j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (20/11/2026)</t>
+          <t>Valide 176j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>177j</t>
+          <t>176j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (02/11/2026)</t>
+          <t>Valide 158j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 258j (09/02/2027)</t>
+          <t>Valide 257j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>258j</t>
+          <t>257j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 276j (28/02/2027)</t>
+          <t>Valide 275j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 18j (14/06/2026)</t>
+          <t>Expire dans 17j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (05/08/2026)</t>
+          <t>Valide 69j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 56j (22/07/2026)</t>
+          <t>Valide 55j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (14/10/2026)</t>
+          <t>Valide 139j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>140j</t>
+          <t>139j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (29/06/2026)</t>
+          <t>Valide 32j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (07/12/2026)</t>
+          <t>Valide 193j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (09/10/2026)</t>
+          <t>Valide 134j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>135j</t>
+          <t>134j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (30/11/2026)</t>
+          <t>Valide 186j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 258j (09/02/2027)</t>
+          <t>Valide 257j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>258j</t>
+          <t>257j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (20/11/2026)</t>
+          <t>Valide 176j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 206j (19/12/2026)</t>
+          <t>Valide 205j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>206j</t>
+          <t>205j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (31/07/2026)</t>
+          <t>Valide 63j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (13/10/2026)</t>
+          <t>Valide 138j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>139j</t>
+          <t>138j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (10/10/2026)</t>
+          <t>Valide 135j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>27/05/2026 10:57</t>
+          <t>28/05/2026 10:58</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 29/05/2026 10:55
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (14/07/2026)</t>
+          <t>Valide 45j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 280j (05/03/2027)</t>
+          <t>Valide 279j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (07/08/2026)</t>
+          <t>Valide 70j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (07/08/2026)</t>
+          <t>Valide 69j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (05/07/2026)</t>
+          <t>Valide 36j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 242j (26/01/2027)</t>
+          <t>Valide 241j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (20/11/2026)</t>
+          <t>Valide 175j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>176j</t>
+          <t>175j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (02/11/2026)</t>
+          <t>Valide 157j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,12 +1258,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 257j (09/02/2027)</t>
+          <t>Valide 256j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>257j</t>
+          <t>256j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 17j (14/06/2026)</t>
+          <t>Expire dans 16j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (05/08/2026)</t>
+          <t>Valide 68j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 55j (22/07/2026)</t>
+          <t>Valide 54j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (14/10/2026)</t>
+          <t>Valide 138j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>139j</t>
+          <t>138j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (29/06/2026)</t>
+          <t>Valide 31j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (07/12/2026)</t>
+          <t>Valide 192j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (09/10/2026)</t>
+          <t>Valide 133j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>134j</t>
+          <t>133j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 186j (30/11/2026)</t>
+          <t>Valide 185j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 257j (09/02/2027)</t>
+          <t>Valide 256j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>257j</t>
+          <t>256j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (20/11/2026)</t>
+          <t>Valide 175j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,12 +2445,12 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 205j (19/12/2026)</t>
+          <t>Valide 204j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>205j</t>
+          <t>204j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (13/10/2026)</t>
+          <t>Valide 137j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>138j</t>
+          <t>137j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (10/10/2026)</t>
+          <t>Valide 134j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>28/05/2026 10:58</t>
+          <t>29/05/2026 10:49</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 30/05/2026 09:26
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (14/07/2026)</t>
+          <t>Valide 44j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 279j (05/03/2027)</t>
+          <t>Valide 278j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
+          <t>30/05/2026 09:21</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (07/08/2026)</t>
+          <t>Valide 69j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (07/08/2026)</t>
+          <t>Valide 68j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
+          <t>30/05/2026 09:21</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (05/07/2026)</t>
+          <t>Valide 35j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 241j (26/01/2027)</t>
+          <t>Valide 240j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
+          <t>30/05/2026 09:21</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (20/11/2026)</t>
+          <t>Valide 174j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>174j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (02/11/2026)</t>
+          <t>Valide 156j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
+          <t>30/05/2026 09:21</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 256j (09/02/2027)</t>
+          <t>Valide 255j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>256j</t>
+          <t>255j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 275j (28/02/2027)</t>
+          <t>Valide 274j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
+          <t>30/05/2026 09:21</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,15 +1358,19 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 16j (14/06/2026)</t>
+          <t>Expire dans 15j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr"/>
+          <t>30/05/2026 09:21</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="15" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A15" s="3" t="inlineStr">
@@ -1646,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (05/08/2026)</t>
+          <t>Valide 67j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (22/07/2026)</t>
+          <t>Valide 53j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
+          <t>30/05/2026 09:21</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (14/10/2026)</t>
+          <t>Valide 137j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>138j</t>
+          <t>137j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
+          <t>30/05/2026 09:21</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,25 +1815,29 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (29/06/2026)</t>
+          <t>Expire dans 30j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (07/12/2026)</t>
+          <t>Valide 191j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr"/>
+          <t>30/05/2026 09:21</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="3" t="inlineStr">
@@ -1997,22 +2005,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (09/10/2026)</t>
+          <t>Valide 132j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>133j</t>
+          <t>132j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (30/11/2026)</t>
+          <t>Valide 184j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
+          <t>30/05/2026 09:21</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2207,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 256j (09/02/2027)</t>
+          <t>Valide 255j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>256j</t>
+          <t>255j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (20/11/2026)</t>
+          <t>Valide 174j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
+          <t>30/05/2026 09:21</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2453,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 204j (19/12/2026)</t>
+          <t>Valide 203j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>204j</t>
+          <t>203j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (31/07/2026)</t>
+          <t>Valide 62j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
+          <t>30/05/2026 09:21</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2695,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (13/10/2026)</t>
+          <t>Valide 136j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>137j</t>
+          <t>136j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (10/10/2026)</t>
+          <t>Valide 133j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>29/05/2026 10:49</t>
+          <t>30/05/2026 09:21</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 31/05/2026 09:52
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (14/07/2026)</t>
+          <t>Valide 43j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 278j (05/03/2027)</t>
+          <t>Valide 277j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
+          <t>31/05/2026 09:48</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (07/08/2026)</t>
+          <t>Valide 67j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
+          <t>31/05/2026 09:48</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (05/07/2026)</t>
+          <t>Valide 34j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 240j (26/01/2027)</t>
+          <t>Valide 239j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
+          <t>31/05/2026 09:48</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (20/11/2026)</t>
+          <t>Valide 173j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>174j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (02/11/2026)</t>
+          <t>Valide 155j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
+          <t>31/05/2026 09:48</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 255j (09/02/2027)</t>
+          <t>Valide 254j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>255j</t>
+          <t>254j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 274j (28/02/2027)</t>
+          <t>Valide 273j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
+          <t>31/05/2026 09:48</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,19 +1358,15 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 15j (14/06/2026)</t>
+          <t>Expire dans 14j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>31/05/2026 09:48</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A15" s="3" t="inlineStr">
@@ -1650,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (05/08/2026)</t>
+          <t>Valide 66j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 53j (22/07/2026)</t>
+          <t>Valide 52j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
+          <t>31/05/2026 09:48</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (14/10/2026)</t>
+          <t>Valide 136j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>137j</t>
+          <t>136j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
+          <t>31/05/2026 09:48</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,29 +1811,25 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (29/06/2026)</t>
+          <t>Expire dans 29j (29/06/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (07/12/2026)</t>
+          <t>Valide 190j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>31/05/2026 09:48</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="3" t="inlineStr">
@@ -2005,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (09/10/2026)</t>
+          <t>Valide 131j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>132j</t>
+          <t>131j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 184j (30/11/2026)</t>
+          <t>Valide 183j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
+          <t>31/05/2026 09:48</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2207,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 255j (09/02/2027)</t>
+          <t>Valide 254j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>255j</t>
+          <t>254j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (20/11/2026)</t>
+          <t>Valide 173j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
+          <t>31/05/2026 09:48</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2453,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 203j (19/12/2026)</t>
+          <t>Valide 202j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>203j</t>
+          <t>202j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (31/07/2026)</t>
+          <t>Valide 61j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
+          <t>31/05/2026 09:48</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2695,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (13/10/2026)</t>
+          <t>Valide 135j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>136j</t>
+          <t>135j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (10/10/2026)</t>
+          <t>Valide 132j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>30/05/2026 09:21</t>
+          <t>31/05/2026 09:48</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 01/06/2026 12:45
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (14/07/2026)</t>
+          <t>Valide 42j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 277j (05/03/2027)</t>
+          <t>Valide 276j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 67j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (07/08/2026)</t>
+          <t>Valide 66j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (05/07/2026)</t>
+          <t>Valide 33j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 239j (26/01/2027)</t>
+          <t>Valide 238j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (20/11/2026)</t>
+          <t>Valide 172j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>173j</t>
+          <t>172j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (02/11/2026)</t>
+          <t>Valide 153j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 254j (09/02/2027)</t>
+          <t>Valide 253j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>254j</t>
+          <t>253j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 273j (28/02/2027)</t>
+          <t>Valide 271j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 14j (14/06/2026)</t>
+          <t>Expire dans 12j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (05/08/2026)</t>
+          <t>Valide 65j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 52j (22/07/2026)</t>
+          <t>Valide 50j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (14/10/2026)</t>
+          <t>Valide 135j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>136j</t>
+          <t>135j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (29/06/2026)</t>
+          <t>Valide 89j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (07/12/2026)</t>
+          <t>Valide 189j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (09/10/2026)</t>
+          <t>Valide 130j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>131j</t>
+          <t>130j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (30/11/2026)</t>
+          <t>Valide 182j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 254j (09/02/2027)</t>
+          <t>Valide 253j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>254j</t>
+          <t>253j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (20/11/2026)</t>
+          <t>Valide 172j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 202j (19/12/2026)</t>
+          <t>Valide 201j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>202j</t>
+          <t>201j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (31/07/2026)</t>
+          <t>Valide 59j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (13/10/2026)</t>
+          <t>Valide 134j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>135j</t>
+          <t>134j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (10/10/2026)</t>
+          <t>Valide 131j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>31/05/2026 09:48</t>
+          <t>01/06/2026 12:40</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 02/06/2026 11:25
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (14/07/2026)</t>
+          <t>Valide 41j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 276j (05/03/2027)</t>
+          <t>Valide 275j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (07/08/2026)</t>
+          <t>Valide 66j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (07/08/2026)</t>
+          <t>Valide 65j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (05/07/2026)</t>
+          <t>Valide 32j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 238j (26/01/2027)</t>
+          <t>Valide 237j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (20/11/2026)</t>
+          <t>Valide 171j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>172j</t>
+          <t>171j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 253j (09/02/2027)</t>
+          <t>Valide 252j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>253j</t>
+          <t>252j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 271j (28/02/2027)</t>
+          <t>Valide 270j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 12j (14/06/2026)</t>
+          <t>Expire dans 11j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 65j (05/08/2026)</t>
+          <t>Valide 64j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 50j (22/07/2026)</t>
+          <t>Valide 49j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (14/10/2026)</t>
+          <t>Valide 134j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>135j</t>
+          <t>134j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (29/08/2026)</t>
+          <t>Valide 88j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (07/12/2026)</t>
+          <t>Valide 188j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (09/10/2026)</t>
+          <t>Valide 129j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>130j</t>
+          <t>129j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (30/11/2026)</t>
+          <t>Valide 181j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 253j (09/02/2027)</t>
+          <t>Valide 252j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>253j</t>
+          <t>252j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (20/11/2026)</t>
+          <t>Valide 171j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 201j (19/12/2026)</t>
+          <t>Valide 200j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>201j</t>
+          <t>200j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 59j (31/07/2026)</t>
+          <t>Valide 58j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (13/10/2026)</t>
+          <t>Valide 133j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>134j</t>
+          <t>133j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (10/10/2026)</t>
+          <t>Valide 130j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>01/06/2026 12:40</t>
+          <t>02/06/2026 11:20</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 03/06/2026 12:04
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (14/07/2026)</t>
+          <t>Valide 40j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 275j (05/03/2027)</t>
+          <t>Valide 274j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 65j (07/08/2026)</t>
+          <t>Valide 64j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (05/07/2026)</t>
+          <t>Valide 31j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 237j (26/01/2027)</t>
+          <t>Valide 236j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (20/11/2026)</t>
+          <t>Valide 170j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>171j</t>
+          <t>170j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (02/11/2026)</t>
+          <t>Valide 152j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 252j (09/02/2027)</t>
+          <t>Valide 251j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>252j</t>
+          <t>251j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 270j (28/02/2027)</t>
+          <t>Valide 269j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1343,30 +1343,34 @@
       </c>
       <c r="K14" s="9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L14" s="9" t="inlineStr">
         <is>
-          <t>Pas de certificat SSL</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Pas de certificat SSL</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 11j (14/06/2026)</t>
+          <t>Expire dans 10j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr"/>
+          <t>03/06/2026 11:58</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="15" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A15" s="3" t="inlineStr">
@@ -1646,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (05/08/2026)</t>
+          <t>Valide 63j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 49j (22/07/2026)</t>
+          <t>Valide 48j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (14/10/2026)</t>
+          <t>Valide 133j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>134j</t>
+          <t>133j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (29/08/2026)</t>
+          <t>Valide 87j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (07/12/2026)</t>
+          <t>Valide 187j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (09/10/2026)</t>
+          <t>Valide 128j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>129j</t>
+          <t>128j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (30/11/2026)</t>
+          <t>Valide 180j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 252j (09/02/2027)</t>
+          <t>Valide 251j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>252j</t>
+          <t>251j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (20/11/2026)</t>
+          <t>Valide 170j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 200j (19/12/2026)</t>
+          <t>Valide 199j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>200j</t>
+          <t>199j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 58j (31/07/2026)</t>
+          <t>Valide 57j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (13/10/2026)</t>
+          <t>Valide 132j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>133j</t>
+          <t>132j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (10/10/2026)</t>
+          <t>Valide 129j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>02/06/2026 11:20</t>
+          <t>03/06/2026 11:58</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 04/06/2026 10:44
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (14/07/2026)</t>
+          <t>Valide 39j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 274j (05/03/2027)</t>
+          <t>Valide 273j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
+          <t>04/06/2026 10:39</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 64j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (07/08/2026)</t>
+          <t>Valide 63j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
+          <t>04/06/2026 10:39</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,25 +1046,29 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (05/07/2026)</t>
+          <t>Expire dans 30j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 236j (26/01/2027)</t>
+          <t>Valide 235j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr"/>
+          <t>04/06/2026 10:39</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="9" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A9" s="3" t="inlineStr">
@@ -1152,22 +1156,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (20/11/2026)</t>
+          <t>Valide 169j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>170j</t>
+          <t>169j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (02/11/2026)</t>
+          <t>Valide 151j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
+          <t>04/06/2026 10:39</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,12 +1262,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 251j (09/02/2027)</t>
+          <t>Valide 250j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>251j</t>
+          <t>250j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1273,7 +1277,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
+          <t>04/06/2026 10:39</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1343,17 +1347,17 @@
       </c>
       <c r="K14" s="9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L14" s="9" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Pas de certificat SSL</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Pas de certificat SSL</t>
         </is>
       </c>
       <c r="N14" s="9" t="inlineStr">
@@ -1363,14 +1367,10 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>04/06/2026 10:39</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A15" s="3" t="inlineStr">
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (05/08/2026)</t>
+          <t>Valide 62j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
+          <t>04/06/2026 10:39</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (14/10/2026)</t>
+          <t>Valide 132j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>133j</t>
+          <t>132j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
+          <t>04/06/2026 10:39</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (29/08/2026)</t>
+          <t>Valide 86j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (07/12/2026)</t>
+          <t>Valide 186j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
+          <t>04/06/2026 10:39</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (09/10/2026)</t>
+          <t>Valide 127j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>128j</t>
+          <t>127j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (30/11/2026)</t>
+          <t>Valide 179j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
+          <t>04/06/2026 10:39</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 251j (09/02/2027)</t>
+          <t>Valide 250j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>251j</t>
+          <t>250j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (20/11/2026)</t>
+          <t>Valide 169j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
+          <t>04/06/2026 10:39</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,12 +2449,12 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 199j (19/12/2026)</t>
+          <t>Valide 198j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>199j</t>
+          <t>198j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
+          <t>04/06/2026 10:39</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (13/10/2026)</t>
+          <t>Valide 131j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>132j</t>
+          <t>131j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (10/10/2026)</t>
+          <t>Valide 128j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>03/06/2026 11:58</t>
+          <t>04/06/2026 10:39</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 05/06/2026 10:55
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (14/07/2026)</t>
+          <t>Valide 38j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 273j (05/03/2027)</t>
+          <t>Valide 272j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (07/08/2026)</t>
+          <t>Valide 63j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (07/08/2026)</t>
+          <t>Valide 62j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,29 +1046,25 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (05/07/2026)</t>
+          <t>Expire dans 29j (05/07/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 235j (26/01/2027)</t>
+          <t>Valide 234j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>05/06/2026 10:50</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A9" s="3" t="inlineStr">
@@ -1156,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (20/11/2026)</t>
+          <t>Valide 168j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>169j</t>
+          <t>168j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (02/11/2026)</t>
+          <t>Valide 150j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1262,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 250j (09/02/2027)</t>
+          <t>Valide 249j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>250j</t>
+          <t>249j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 269j (28/02/2027)</t>
+          <t>Valide 268j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1362,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 10j (14/06/2026)</t>
+          <t>Expire dans 9j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1650,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (05/08/2026)</t>
+          <t>Valide 61j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 48j (22/07/2026)</t>
+          <t>Valide 47j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (14/10/2026)</t>
+          <t>Valide 131j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>132j</t>
+          <t>131j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (29/08/2026)</t>
+          <t>Valide 85j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 186j (07/12/2026)</t>
+          <t>Valide 185j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (09/10/2026)</t>
+          <t>Valide 126j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>127j</t>
+          <t>126j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (30/11/2026)</t>
+          <t>Valide 178j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 250j (09/02/2027)</t>
+          <t>Valide 249j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>250j</t>
+          <t>249j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (20/11/2026)</t>
+          <t>Valide 168j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 198j (19/12/2026)</t>
+          <t>Valide 197j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>198j</t>
+          <t>197j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 57j (31/07/2026)</t>
+          <t>Valide 56j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (13/10/2026)</t>
+          <t>Valide 130j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>131j</t>
+          <t>130j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (10/10/2026)</t>
+          <t>Valide 127j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>04/06/2026 10:39</t>
+          <t>05/06/2026 10:50</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 06/06/2026 09:32
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (14/07/2026)</t>
+          <t>Valide 37j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 272j (05/03/2027)</t>
+          <t>Valide 271j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (07/08/2026)</t>
+          <t>Valide 61j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (05/07/2026)</t>
+          <t>Valide 88j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 234j (26/01/2027)</t>
+          <t>Valide 233j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (20/11/2026)</t>
+          <t>Valide 167j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>168j</t>
+          <t>167j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (02/11/2026)</t>
+          <t>Valide 149j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 249j (09/02/2027)</t>
+          <t>Valide 248j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>249j</t>
+          <t>248j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 268j (28/02/2027)</t>
+          <t>Valide 267j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 9j (14/06/2026)</t>
+          <t>Expire dans 8j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (05/08/2026)</t>
+          <t>Valide 60j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 47j (22/07/2026)</t>
+          <t>Valide 46j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (14/10/2026)</t>
+          <t>Valide 130j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>131j</t>
+          <t>130j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (29/08/2026)</t>
+          <t>Valide 84j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (07/12/2026)</t>
+          <t>Valide 184j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +1997,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (09/10/2026)</t>
+          <t>Valide 125j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>126j</t>
+          <t>125j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (30/11/2026)</t>
+          <t>Valide 177j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2199,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 249j (09/02/2027)</t>
+          <t>Valide 248j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>249j</t>
+          <t>248j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (20/11/2026)</t>
+          <t>Valide 167j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2445,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 197j (19/12/2026)</t>
+          <t>Valide 196j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>197j</t>
+          <t>196j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 56j (31/07/2026)</t>
+          <t>Valide 55j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2687,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (13/10/2026)</t>
+          <t>Valide 129j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>130j</t>
+          <t>129j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (10/10/2026)</t>
+          <t>Valide 126j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>05/06/2026 10:50</t>
+          <t>06/06/2026 09:27</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 07/06/2026 10:10
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (14/07/2026)</t>
+          <t>Valide 36j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 271j (05/03/2027)</t>
+          <t>Valide 270j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 61j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (07/08/2026)</t>
+          <t>Valide 60j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (03/09/2026)</t>
+          <t>Valide 87j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 233j (26/01/2027)</t>
+          <t>Valide 232j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (20/11/2026)</t>
+          <t>Valide 166j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>167j</t>
+          <t>166j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (02/11/2026)</t>
+          <t>Valide 148j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 248j (09/02/2027)</t>
+          <t>Valide 247j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>248j</t>
+          <t>247j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 267j (28/02/2027)</t>
+          <t>Valide 266j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,15 +1358,19 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 8j (14/06/2026)</t>
+          <t>Expire dans 7j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr"/>
+          <t>07/06/2026 10:06</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="15" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A15" s="3" t="inlineStr">
@@ -1646,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 60j (05/08/2026)</t>
+          <t>Valide 59j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 46j (22/07/2026)</t>
+          <t>Valide 45j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1716,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (14/10/2026)</t>
+          <t>Valide 129j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>130j</t>
+          <t>129j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1731,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (29/08/2026)</t>
+          <t>Valide 83j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 184j (07/12/2026)</t>
+          <t>Valide 183j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1997,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (09/10/2026)</t>
+          <t>Valide 124j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>125j</t>
+          <t>124j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (30/11/2026)</t>
+          <t>Valide 176j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2199,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 248j (09/02/2027)</t>
+          <t>Valide 247j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>248j</t>
+          <t>247j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (20/11/2026)</t>
+          <t>Valide 166j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2445,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 196j (19/12/2026)</t>
+          <t>Valide 195j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>196j</t>
+          <t>195j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 55j (31/07/2026)</t>
+          <t>Valide 54j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2687,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (13/10/2026)</t>
+          <t>Valide 128j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>129j</t>
+          <t>128j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (10/10/2026)</t>
+          <t>Valide 125j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>06/06/2026 09:27</t>
+          <t>07/06/2026 10:06</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 08/06/2026 12:05
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (14/07/2026)</t>
+          <t>Valide 35j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 270j (05/03/2027)</t>
+          <t>Valide 269j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 60j (07/08/2026)</t>
+          <t>Valide 59j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (03/09/2026)</t>
+          <t>Valide 86j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 232j (26/01/2027)</t>
+          <t>Valide 231j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (20/11/2026)</t>
+          <t>Valide 165j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>166j</t>
+          <t>165j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (02/11/2026)</t>
+          <t>Valide 147j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 247j (09/02/2027)</t>
+          <t>Valide 246j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>247j</t>
+          <t>246j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 266j (28/02/2027)</t>
+          <t>Valide 264j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1358,12 +1358,12 @@
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 7j (14/06/2026)</t>
+          <t>Expire dans 5j (14/06/2026)</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1650,22 +1650,22 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 59j (05/08/2026)</t>
+          <t>Valide 58j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>Valide 45j (22/07/2026)</t>
+          <t>Valide 43j (22/07/2026)</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (14/10/2026)</t>
+          <t>Valide 128j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>129j</t>
+          <t>128j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (29/08/2026)</t>
+          <t>Valide 82j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (07/12/2026)</t>
+          <t>Valide 182j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (09/10/2026)</t>
+          <t>Valide 123j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>124j</t>
+          <t>123j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (30/11/2026)</t>
+          <t>Valide 175j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 247j (09/02/2027)</t>
+          <t>Valide 246j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>247j</t>
+          <t>246j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (20/11/2026)</t>
+          <t>Valide 165j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,22 +2449,22 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 195j (19/12/2026)</t>
+          <t>Valide 194j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>195j</t>
+          <t>194j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (31/07/2026)</t>
+          <t>Valide 52j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (13/10/2026)</t>
+          <t>Valide 127j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>128j</t>
+          <t>127j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (10/10/2026)</t>
+          <t>Valide 124j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>07/06/2026 10:06</t>
+          <t>08/06/2026 12:00</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 09/06/2026 10:40
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (14/07/2026)</t>
+          <t>Valide 34j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 269j (05/03/2027)</t>
+          <t>Valide 268j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 59j (07/08/2026)</t>
+          <t>Valide 58j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (03/09/2026)</t>
+          <t>Valide 85j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 231j (26/01/2027)</t>
+          <t>Valide 230j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (20/11/2026)</t>
+          <t>Valide 164j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>165j</t>
+          <t>164j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (02/11/2026)</t>
+          <t>Valide 146j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,12 +1258,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 246j (09/02/2027)</t>
+          <t>Valide 245j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>246j</t>
+          <t>245j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Valide 58j (05/08/2026)</t>
+          <t>Valide 57j (05/08/2026)</t>
         </is>
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="L24" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (14/10/2026)</t>
+          <t>Valide 127j (14/10/2026)</t>
         </is>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>128j</t>
+          <t>127j</t>
         </is>
       </c>
       <c r="N24" s="9" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (29/08/2026)</t>
+          <t>Valide 81j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (07/12/2026)</t>
+          <t>Valide 181j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2001,22 +2001,22 @@
       </c>
       <c r="L30" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (09/10/2026)</t>
+          <t>Valide 122j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>123j</t>
+          <t>122j</t>
         </is>
       </c>
       <c r="N30" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (30/11/2026)</t>
+          <t>Valide 174j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2203,22 +2203,22 @@
       </c>
       <c r="L36" s="9" t="inlineStr">
         <is>
-          <t>Valide 246j (09/02/2027)</t>
+          <t>Valide 245j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>246j</t>
+          <t>245j</t>
         </is>
       </c>
       <c r="N36" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (20/11/2026)</t>
+          <t>Valide 164j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2449,12 +2449,12 @@
       </c>
       <c r="L43" s="4" t="inlineStr">
         <is>
-          <t>Valide 194j (19/12/2026)</t>
+          <t>Valide 193j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="4" t="inlineStr">
         <is>
-          <t>194j</t>
+          <t>193j</t>
         </is>
       </c>
       <c r="N43" s="4" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2691,22 +2691,22 @@
       </c>
       <c r="L50" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (13/10/2026)</t>
+          <t>Valide 126j (13/10/2026)</t>
         </is>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>127j</t>
+          <t>126j</t>
         </is>
       </c>
       <c r="N50" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (10/10/2026)</t>
+          <t>Valide 123j (10/10/2026)</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>08/06/2026 12:00</t>
+          <t>09/06/2026 10:35</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 10/06/2026 16:51
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventaire" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Inventaire" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Config" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$2:$N$51</definedName>
@@ -842,24 +842,25 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (14/07/2026)</t>
+          <t>Valide 33j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 321j (05/03/2027)</t>
+          <t>Valide 267j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A5" s="3" t="inlineStr">
@@ -975,24 +976,25 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 58j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 111j (07/08/2026)</t>
+          <t>Valide 57j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1" s="34">
       <c r="A8" s="8" t="inlineStr">
@@ -1044,24 +1046,25 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (05/07/2026)</t>
+          <t>Valide 84j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 283j (26/01/2027)</t>
+          <t>Valide 229j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A9" s="3" t="inlineStr">
@@ -1149,24 +1152,25 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (20/05/2026)</t>
+          <t>Valide 163j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>163j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 199j (02/11/2026)</t>
+          <t>Valide 144j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A11" s="3" t="inlineStr">
@@ -1254,24 +1258,25 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 298j (09/02/2027)</t>
+          <t>Valide 244j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>298j</t>
+          <t>244j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 317j (28/02/2027)</t>
+          <t>Valide 262j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A13" s="3" t="inlineStr">
@@ -1575,24 +1580,25 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 110j (05/08/2026)</t>
+          <t>Valide 56j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 96j (22/07/2026)</t>
+          <t>Valide 41j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1" s="34">
       <c r="A23" s="8" t="inlineStr">
@@ -1644,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (14/10/2026)</t>
+          <t>Valide 126j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>126j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1659,9 +1665,10 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>x</t>
@@ -1738,24 +1745,25 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (29/06/2026)</t>
+          <t>Valide 80j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 234j (07/12/2026)</t>
+          <t>Valide 180j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1" s="34">
       <c r="A26" s="3" t="inlineStr">
@@ -1768,7 +1776,11 @@
           <t>albystech.com</t>
         </is>
       </c>
-      <c r="C26" s="5" t="n"/>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>https://albys.com/</t>
+        </is>
+      </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
           <t>AWS</t>
@@ -1923,24 +1935,25 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (09/10/2026)</t>
+          <t>Valide 121j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>121j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 227j (30/11/2026)</t>
+          <t>Valide 172j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1" s="34">
       <c r="A30" s="3" t="inlineStr">
@@ -1953,7 +1966,11 @@
           <t>leadportage.com</t>
         </is>
       </c>
-      <c r="C30" s="5" t="n"/>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>https://lead-portage.com/</t>
+        </is>
+      </c>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
@@ -2124,24 +2141,25 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 298j (09/02/2027)</t>
+          <t>Valide 244j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>298j</t>
+          <t>244j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 217j (20/11/2026)</t>
+          <t>Valide 162j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36" ht="18" customHeight="1" s="34">
       <c r="A36" s="3" t="inlineStr">
@@ -2154,7 +2172,11 @@
           <t>idec91.fr</t>
         </is>
       </c>
-      <c r="C36" s="5" t="n"/>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>https://selnhelp.fr/</t>
+        </is>
+      </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
           <t>GANDI</t>
@@ -2369,24 +2391,25 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 246j (19/12/2026)</t>
+          <t>Valide 192j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>246j</t>
+          <t>192j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 105j (31/07/2026)</t>
+          <t>Valide 50j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr"/>
     </row>
     <row r="43" ht="18" customHeight="1" s="34">
       <c r="A43" s="8" t="inlineStr">
@@ -2399,7 +2422,11 @@
           <t>isytem.fr</t>
         </is>
       </c>
-      <c r="C43" s="10" t="n"/>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>https://isytem.com/</t>
+        </is>
+      </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
           <t>GANDI</t>
@@ -2610,24 +2637,25 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (13/10/2026)</t>
+          <t>Valide 125j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>179j</t>
+          <t>125j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (10/10/2026)</t>
+          <t>Valide 121j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>17/04/2026 08:27</t>
-        </is>
-      </c>
+          <t>10/06/2026 16:48</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1" s="34">
       <c r="A50" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: monitoring 11/06/2026 11:29
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (14/07/2026)</t>
+          <t>Valide 32j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 267j (05/03/2027)</t>
+          <t>Valide 266j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 58j (07/08/2026)</t>
+          <t>Valide 57j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 57j (07/08/2026)</t>
+          <t>Valide 56j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (03/09/2026)</t>
+          <t>Valide 83j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 229j (26/01/2027)</t>
+          <t>Valide 228j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (20/11/2026)</t>
+          <t>Valide 162j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>163j</t>
+          <t>162j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 244j (09/02/2027)</t>
+          <t>Valide 243j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>244j</t>
+          <t>243j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 262j (28/02/2027)</t>
+          <t>Valide 261j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 56j (05/08/2026)</t>
+          <t>Valide 55j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 41j (22/07/2026)</t>
+          <t>Valide 40j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (14/10/2026)</t>
+          <t>Valide 125j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>126j</t>
+          <t>125j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (29/08/2026)</t>
+          <t>Valide 79j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (07/12/2026)</t>
+          <t>Valide 179j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1804,10 +1804,32 @@
         </is>
       </c>
       <c r="J26" s="4" t="n"/>
-      <c r="K26" s="4" t="n"/>
-      <c r="L26" s="4" t="n"/>
-      <c r="M26" s="4" t="n"/>
-      <c r="N26" s="4" t="n"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Valide 79j (29/08/2026)</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>79j</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>Valide 179j (07/12/2026)</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>11/06/2026 11:24</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="8" t="inlineStr">
@@ -1935,12 +1957,12 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (09/10/2026)</t>
+          <t>Valide 120j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>121j</t>
+          <t>120j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
@@ -1950,7 +1972,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -1978,10 +2000,32 @@
       <c r="H30" s="6" t="n"/>
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="4" t="n"/>
-      <c r="K30" s="4" t="n"/>
-      <c r="L30" s="4" t="n"/>
-      <c r="M30" s="4" t="n"/>
-      <c r="N30" s="4" t="n"/>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Valide 120j (09/10/2026)</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>120j</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>Valide 172j (30/11/2026)</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>11/06/2026 11:24</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A31" s="8" t="inlineStr">
@@ -2141,12 +2185,12 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 244j (09/02/2027)</t>
+          <t>Valide 243j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>244j</t>
+          <t>243j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
@@ -2156,7 +2200,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2196,10 +2240,32 @@
         </is>
       </c>
       <c r="J36" s="4" t="n"/>
-      <c r="K36" s="4" t="n"/>
-      <c r="L36" s="4" t="n"/>
-      <c r="M36" s="4" t="n"/>
-      <c r="N36" s="4" t="n"/>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Valide 243j (09/02/2027)</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>243j</t>
+        </is>
+      </c>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>Valide 162j (20/11/2026)</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>11/06/2026 11:24</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A37" s="8" t="inlineStr">
@@ -2391,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 192j (19/12/2026)</t>
+          <t>Valide 191j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>192j</t>
+          <t>191j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 50j (31/07/2026)</t>
+          <t>Valide 49j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2438,10 +2504,32 @@
       <c r="H43" s="11" t="n"/>
       <c r="I43" s="12" t="n"/>
       <c r="J43" s="9" t="n"/>
-      <c r="K43" s="9" t="n"/>
-      <c r="L43" s="9" t="n"/>
-      <c r="M43" s="9" t="n"/>
-      <c r="N43" s="9" t="n"/>
+      <c r="K43" s="9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="L43" s="9" t="inlineStr">
+        <is>
+          <t>Valide 191j (19/12/2026)</t>
+        </is>
+      </c>
+      <c r="M43" s="9" t="inlineStr">
+        <is>
+          <t>191j</t>
+        </is>
+      </c>
+      <c r="N43" s="9" t="inlineStr">
+        <is>
+          <t>Valide 49j (31/07/2026)</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>11/06/2026 11:24</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr"/>
     </row>
     <row r="44" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A44" s="3" t="inlineStr">
@@ -2637,12 +2725,12 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (13/10/2026)</t>
+          <t>Valide 124j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>125j</t>
+          <t>124j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
@@ -2652,7 +2740,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>10/06/2026 16:48</t>
+          <t>11/06/2026 11:24</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 12/06/2026 11:09
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (14/07/2026)</t>
+          <t>Valide 31j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 266j (05/03/2027)</t>
+          <t>Valide 265j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 57j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 56j (07/08/2026)</t>
+          <t>Valide 55j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (03/09/2026)</t>
+          <t>Valide 82j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 228j (26/01/2027)</t>
+          <t>Valide 227j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (20/11/2026)</t>
+          <t>Valide 161j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>162j</t>
+          <t>161j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (02/11/2026)</t>
+          <t>Valide 143j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 243j (09/02/2027)</t>
+          <t>Valide 242j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>243j</t>
+          <t>242j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 261j (28/02/2027)</t>
+          <t>Valide 260j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,12 +1580,12 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 55j (05/08/2026)</t>
+          <t>Valide 54j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (14/10/2026)</t>
+          <t>Valide 124j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>125j</t>
+          <t>124j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (29/08/2026)</t>
+          <t>Valide 78j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (07/12/2026)</t>
+          <t>Valide 178j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (29/08/2026)</t>
+          <t>Valide 78j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 179j (07/12/2026)</t>
+          <t>Valide 178j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (09/10/2026)</t>
+          <t>Valide 119j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>119j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (30/11/2026)</t>
+          <t>Valide 171j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 120j (09/10/2026)</t>
+          <t>Valide 119j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>119j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 172j (30/11/2026)</t>
+          <t>Valide 171j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 243j (09/02/2027)</t>
+          <t>Valide 242j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>243j</t>
+          <t>242j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (20/11/2026)</t>
+          <t>Valide 161j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 243j (09/02/2027)</t>
+          <t>Valide 242j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>243j</t>
+          <t>242j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 162j (20/11/2026)</t>
+          <t>Valide 161j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 191j (19/12/2026)</t>
+          <t>Valide 190j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>191j</t>
+          <t>190j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 49j (31/07/2026)</t>
+          <t>Valide 48j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (19/12/2026)</t>
+          <t>Valide 190j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>191j</t>
+          <t>190j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (31/07/2026)</t>
+          <t>Valide 48j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (13/10/2026)</t>
+          <t>Valide 123j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>124j</t>
+          <t>123j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (10/10/2026)</t>
+          <t>Valide 120j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>11/06/2026 11:24</t>
+          <t>12/06/2026 11:03</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 13/06/2026 10:02
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,25 +842,29 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (14/07/2026)</t>
+          <t>Expire dans 30j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 265j (05/03/2027)</t>
+          <t>Valide 264j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
+          <t>13/06/2026 09:57</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="5" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A5" s="3" t="inlineStr">
@@ -986,12 +990,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 55j (07/08/2026)</t>
+          <t>Valide 54j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1050,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (03/09/2026)</t>
+          <t>Valide 81j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 227j (26/01/2027)</t>
+          <t>Valide 226j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1156,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (20/11/2026)</t>
+          <t>Valide 160j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>161j</t>
+          <t>160j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (02/11/2026)</t>
+          <t>Valide 142j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,12 +1262,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 242j (09/02/2027)</t>
+          <t>Valide 241j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>242j</t>
+          <t>241j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1273,7 +1277,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (05/08/2026)</t>
+          <t>Valide 53j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 40j (22/07/2026)</t>
+          <t>Valide 39j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (14/10/2026)</t>
+          <t>Valide 123j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>124j</t>
+          <t>123j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (29/08/2026)</t>
+          <t>Valide 77j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (07/12/2026)</t>
+          <t>Valide 177j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (29/08/2026)</t>
+          <t>Valide 77j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 178j (07/12/2026)</t>
+          <t>Valide 177j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (09/10/2026)</t>
+          <t>Valide 118j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>119j</t>
+          <t>118j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (30/11/2026)</t>
+          <t>Valide 170j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 119j (09/10/2026)</t>
+          <t>Valide 118j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>119j</t>
+          <t>118j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 171j (30/11/2026)</t>
+          <t>Valide 170j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 242j (09/02/2027)</t>
+          <t>Valide 241j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>242j</t>
+          <t>241j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (20/11/2026)</t>
+          <t>Valide 160j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 242j (09/02/2027)</t>
+          <t>Valide 241j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>242j</t>
+          <t>241j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 161j (20/11/2026)</t>
+          <t>Valide 160j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,12 +2461,12 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 190j (19/12/2026)</t>
+          <t>Valide 189j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>190j</t>
+          <t>189j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
@@ -2472,7 +2476,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,12 +2515,12 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (19/12/2026)</t>
+          <t>Valide 189j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>190j</t>
+          <t>189j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
@@ -2526,7 +2530,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (13/10/2026)</t>
+          <t>Valide 122j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>123j</t>
+          <t>122j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (10/10/2026)</t>
+          <t>Valide 119j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>12/06/2026 11:03</t>
+          <t>13/06/2026 09:57</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 14/06/2026 10:31
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (14/07/2026)</t>
+          <t>Expire dans 29j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 264j (05/03/2027)</t>
+          <t>Valide 263j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -980,22 +980,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 54j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (07/08/2026)</t>
+          <t>Valide 53j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1050,22 +1050,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (03/09/2026)</t>
+          <t>Valide 80j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 226j (26/01/2027)</t>
+          <t>Valide 225j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1156,22 +1156,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (20/11/2026)</t>
+          <t>Valide 159j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>160j</t>
+          <t>159j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (02/11/2026)</t>
+          <t>Valide 141j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 241j (09/02/2027)</t>
+          <t>Valide 240j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>241j</t>
+          <t>240j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 260j (28/02/2027)</t>
+          <t>Valide 259j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 53j (05/08/2026)</t>
+          <t>Valide 52j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 39j (22/07/2026)</t>
+          <t>Valide 38j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (14/10/2026)</t>
+          <t>Valide 122j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>123j</t>
+          <t>122j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (29/08/2026)</t>
+          <t>Valide 76j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (07/12/2026)</t>
+          <t>Valide 176j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (29/08/2026)</t>
+          <t>Valide 76j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 177j (07/12/2026)</t>
+          <t>Valide 176j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (09/10/2026)</t>
+          <t>Valide 117j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>118j</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (30/11/2026)</t>
+          <t>Valide 169j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 118j (09/10/2026)</t>
+          <t>Valide 117j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>118j</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 170j (30/11/2026)</t>
+          <t>Valide 169j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 241j (09/02/2027)</t>
+          <t>Valide 240j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>241j</t>
+          <t>240j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (20/11/2026)</t>
+          <t>Valide 159j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 241j (09/02/2027)</t>
+          <t>Valide 240j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>241j</t>
+          <t>240j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 160j (20/11/2026)</t>
+          <t>Valide 159j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 189j (19/12/2026)</t>
+          <t>Valide 188j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>189j</t>
+          <t>188j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 48j (31/07/2026)</t>
+          <t>Valide 47j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (19/12/2026)</t>
+          <t>Valide 188j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>189j</t>
+          <t>188j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (31/07/2026)</t>
+          <t>Valide 47j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (13/10/2026)</t>
+          <t>Valide 121j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>122j</t>
+          <t>121j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (10/10/2026)</t>
+          <t>Valide 118j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>13/06/2026 09:57</t>
+          <t>14/06/2026 10:26</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 15/06/2026 13:24
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (14/07/2026)</t>
+          <t>Expire dans 28j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>28j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 263j (05/03/2027)</t>
+          <t>Valide 262j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -980,22 +980,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 53j (07/08/2026)</t>
+          <t>Valide 52j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1050,22 +1050,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (03/09/2026)</t>
+          <t>Valide 79j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 225j (26/01/2027)</t>
+          <t>Valide 224j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1156,22 +1156,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (20/11/2026)</t>
+          <t>Valide 158j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>159j</t>
+          <t>158j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (02/11/2026)</t>
+          <t>Valide 139j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 240j (09/02/2027)</t>
+          <t>Valide 239j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>240j</t>
+          <t>239j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 259j (28/02/2027)</t>
+          <t>Valide 257j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 52j (05/08/2026)</t>
+          <t>Valide 51j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 38j (22/07/2026)</t>
+          <t>Valide 36j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (14/10/2026)</t>
+          <t>Valide 121j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>122j</t>
+          <t>121j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (29/08/2026)</t>
+          <t>Valide 75j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (07/12/2026)</t>
+          <t>Valide 175j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (29/08/2026)</t>
+          <t>Valide 75j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 176j (07/12/2026)</t>
+          <t>Valide 175j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (09/10/2026)</t>
+          <t>Valide 116j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (30/11/2026)</t>
+          <t>Valide 168j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 117j (09/10/2026)</t>
+          <t>Valide 116j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 169j (30/11/2026)</t>
+          <t>Valide 168j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 240j (09/02/2027)</t>
+          <t>Valide 239j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>240j</t>
+          <t>239j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (20/11/2026)</t>
+          <t>Valide 158j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 240j (09/02/2027)</t>
+          <t>Valide 239j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>240j</t>
+          <t>239j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 159j (20/11/2026)</t>
+          <t>Valide 158j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 188j (19/12/2026)</t>
+          <t>Valide 187j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>188j</t>
+          <t>187j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 47j (31/07/2026)</t>
+          <t>Valide 45j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (19/12/2026)</t>
+          <t>Valide 187j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>188j</t>
+          <t>187j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (31/07/2026)</t>
+          <t>Valide 45j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (13/10/2026)</t>
+          <t>Valide 120j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>121j</t>
+          <t>120j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (10/10/2026)</t>
+          <t>Valide 116j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>14/06/2026 10:26</t>
+          <t>15/06/2026 13:19</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 16/06/2026 12:19
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 28j (14/07/2026)</t>
+          <t>Expire dans 27j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>28j</t>
+          <t>27j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 262j (05/03/2027)</t>
+          <t>Valide 261j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -980,22 +980,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 52j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 52j (07/08/2026)</t>
+          <t>Valide 51j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1050,22 +1050,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (03/09/2026)</t>
+          <t>Valide 78j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 224j (26/01/2027)</t>
+          <t>Valide 223j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1156,12 +1156,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (20/11/2026)</t>
+          <t>Valide 157j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>158j</t>
+          <t>157j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 239j (09/02/2027)</t>
+          <t>Valide 238j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>239j</t>
+          <t>238j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 257j (28/02/2027)</t>
+          <t>Valide 256j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 51j (05/08/2026)</t>
+          <t>Valide 50j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 36j (22/07/2026)</t>
+          <t>Valide 35j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (14/10/2026)</t>
+          <t>Valide 120j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>121j</t>
+          <t>120j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (29/08/2026)</t>
+          <t>Valide 74j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (07/12/2026)</t>
+          <t>Valide 174j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (29/08/2026)</t>
+          <t>Valide 74j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 175j (07/12/2026)</t>
+          <t>Valide 174j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (09/10/2026)</t>
+          <t>Valide 115j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>115j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (30/11/2026)</t>
+          <t>Valide 167j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 116j (09/10/2026)</t>
+          <t>Valide 115j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>115j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 168j (30/11/2026)</t>
+          <t>Valide 167j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 239j (09/02/2027)</t>
+          <t>Valide 238j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>239j</t>
+          <t>238j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (20/11/2026)</t>
+          <t>Valide 157j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 239j (09/02/2027)</t>
+          <t>Valide 238j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>239j</t>
+          <t>238j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 158j (20/11/2026)</t>
+          <t>Valide 157j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 187j (19/12/2026)</t>
+          <t>Valide 186j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>187j</t>
+          <t>186j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 45j (31/07/2026)</t>
+          <t>Valide 44j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (19/12/2026)</t>
+          <t>Valide 186j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>187j</t>
+          <t>186j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (31/07/2026)</t>
+          <t>Valide 44j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,12 +2729,12 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (13/10/2026)</t>
+          <t>Valide 119j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>119j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>15/06/2026 13:19</t>
+          <t>16/06/2026 12:13</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 16/06/2026 12:36
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -857,14 +857,10 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>16/06/2026 12:30</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A5" s="3" t="inlineStr">
@@ -980,12 +976,12 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 52j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -995,7 +991,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1065,7 +1061,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1166,12 +1162,12 @@
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (02/11/2026)</t>
+          <t>Valide 138j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1277,7 +1273,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1599,7 +1595,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1669,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1764,7 +1760,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1830,7 +1826,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1976,7 +1972,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2026,7 +2022,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2204,7 +2200,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2266,7 +2262,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2476,7 +2472,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2530,7 +2526,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2744,7 +2740,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>16/06/2026 12:13</t>
+          <t>16/06/2026 12:30</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 17/06/2026 11:57
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 27j (14/07/2026)</t>
+          <t>Expire dans 26j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>27j</t>
+          <t>26j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 261j (05/03/2027)</t>
+          <t>Valide 260j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 51j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 51j (07/08/2026)</t>
+          <t>Valide 50j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (03/09/2026)</t>
+          <t>Valide 77j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 223j (26/01/2027)</t>
+          <t>Valide 222j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (20/11/2026)</t>
+          <t>Valide 156j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>157j</t>
+          <t>156j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 238j (09/02/2027)</t>
+          <t>Valide 237j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>238j</t>
+          <t>237j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 256j (28/02/2027)</t>
+          <t>Valide 255j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 50j (05/08/2026)</t>
+          <t>Valide 49j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 35j (22/07/2026)</t>
+          <t>Valide 34j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (14/10/2026)</t>
+          <t>Valide 119j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>119j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (29/08/2026)</t>
+          <t>Valide 73j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (07/12/2026)</t>
+          <t>Valide 173j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 74j (29/08/2026)</t>
+          <t>Valide 73j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 174j (07/12/2026)</t>
+          <t>Valide 173j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (09/10/2026)</t>
+          <t>Valide 114j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>115j</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (30/11/2026)</t>
+          <t>Valide 166j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 115j (09/10/2026)</t>
+          <t>Valide 114j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>115j</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 167j (30/11/2026)</t>
+          <t>Valide 166j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 238j (09/02/2027)</t>
+          <t>Valide 237j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>238j</t>
+          <t>237j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (20/11/2026)</t>
+          <t>Valide 156j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 238j (09/02/2027)</t>
+          <t>Valide 237j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>238j</t>
+          <t>237j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 157j (20/11/2026)</t>
+          <t>Valide 156j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 186j (19/12/2026)</t>
+          <t>Valide 185j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>186j</t>
+          <t>185j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 44j (31/07/2026)</t>
+          <t>Valide 43j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 186j (19/12/2026)</t>
+          <t>Valide 185j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>186j</t>
+          <t>185j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (31/07/2026)</t>
+          <t>Valide 43j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (13/10/2026)</t>
+          <t>Valide 118j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>119j</t>
+          <t>118j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (10/10/2026)</t>
+          <t>Valide 115j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>16/06/2026 12:30</t>
+          <t>17/06/2026 11:52</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 18/06/2026 11:15
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 26j (14/07/2026)</t>
+          <t>Expire dans 25j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>26j</t>
+          <t>25j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 260j (05/03/2027)</t>
+          <t>Valide 259j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 51j (07/08/2026)</t>
+          <t>Valide 50j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 50j (07/08/2026)</t>
+          <t>Valide 49j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (03/09/2026)</t>
+          <t>Valide 76j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 222j (26/01/2027)</t>
+          <t>Valide 221j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (20/11/2026)</t>
+          <t>Valide 155j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>156j</t>
+          <t>155j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (02/11/2026)</t>
+          <t>Valide 137j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 237j (09/02/2027)</t>
+          <t>Valide 236j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>237j</t>
+          <t>236j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 255j (28/02/2027)</t>
+          <t>Valide 254j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,12 +1580,12 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 49j (05/08/2026)</t>
+          <t>Valide 48j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (14/10/2026)</t>
+          <t>Valide 118j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>119j</t>
+          <t>118j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (29/08/2026)</t>
+          <t>Valide 72j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (07/12/2026)</t>
+          <t>Valide 172j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (29/08/2026)</t>
+          <t>Valide 72j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 173j (07/12/2026)</t>
+          <t>Valide 172j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (09/10/2026)</t>
+          <t>Valide 113j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (30/11/2026)</t>
+          <t>Valide 165j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 114j (09/10/2026)</t>
+          <t>Valide 113j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 166j (30/11/2026)</t>
+          <t>Valide 165j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 237j (09/02/2027)</t>
+          <t>Valide 236j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>237j</t>
+          <t>236j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (20/11/2026)</t>
+          <t>Valide 155j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 237j (09/02/2027)</t>
+          <t>Valide 236j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>237j</t>
+          <t>236j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 156j (20/11/2026)</t>
+          <t>Valide 155j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 185j (19/12/2026)</t>
+          <t>Valide 184j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>185j</t>
+          <t>184j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 43j (31/07/2026)</t>
+          <t>Valide 42j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (19/12/2026)</t>
+          <t>Valide 184j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>185j</t>
+          <t>184j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (31/07/2026)</t>
+          <t>Valide 42j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (13/10/2026)</t>
+          <t>Valide 117j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>118j</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (10/10/2026)</t>
+          <t>Valide 114j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>17/06/2026 11:52</t>
+          <t>18/06/2026 11:09</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 19/06/2026 11:31
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 25j (14/07/2026)</t>
+          <t>Expire dans 24j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>25j</t>
+          <t>24j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 259j (05/03/2027)</t>
+          <t>Valide 258j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 50j (07/08/2026)</t>
+          <t>Valide 49j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 49j (07/08/2026)</t>
+          <t>Valide 48j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (03/09/2026)</t>
+          <t>Valide 75j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 221j (26/01/2027)</t>
+          <t>Valide 220j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (20/11/2026)</t>
+          <t>Valide 154j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>155j</t>
+          <t>154j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (02/11/2026)</t>
+          <t>Valide 136j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 236j (09/02/2027)</t>
+          <t>Valide 235j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>236j</t>
+          <t>235j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 254j (28/02/2027)</t>
+          <t>Valide 253j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 48j (05/08/2026)</t>
+          <t>Valide 47j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 34j (22/07/2026)</t>
+          <t>Valide 32j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (14/10/2026)</t>
+          <t>Valide 117j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>118j</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (29/08/2026)</t>
+          <t>Valide 71j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (07/12/2026)</t>
+          <t>Valide 171j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (29/08/2026)</t>
+          <t>Valide 71j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 172j (07/12/2026)</t>
+          <t>Valide 171j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (09/10/2026)</t>
+          <t>Valide 112j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>112j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (30/11/2026)</t>
+          <t>Valide 164j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 113j (09/10/2026)</t>
+          <t>Valide 112j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>112j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 165j (30/11/2026)</t>
+          <t>Valide 164j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 236j (09/02/2027)</t>
+          <t>Valide 235j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>236j</t>
+          <t>235j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (20/11/2026)</t>
+          <t>Valide 154j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 236j (09/02/2027)</t>
+          <t>Valide 235j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>236j</t>
+          <t>235j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 155j (20/11/2026)</t>
+          <t>Valide 154j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 184j (19/12/2026)</t>
+          <t>Valide 183j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>184j</t>
+          <t>183j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 42j (31/07/2026)</t>
+          <t>Valide 41j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 184j (19/12/2026)</t>
+          <t>Valide 183j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>184j</t>
+          <t>183j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (31/07/2026)</t>
+          <t>Valide 41j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (13/10/2026)</t>
+          <t>Valide 116j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (10/10/2026)</t>
+          <t>Valide 113j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>18/06/2026 11:09</t>
+          <t>19/06/2026 11:25</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 20/06/2026 10:15
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 24j (14/07/2026)</t>
+          <t>Expire dans 23j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>24j</t>
+          <t>23j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 258j (05/03/2027)</t>
+          <t>Valide 257j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 49j (07/08/2026)</t>
+          <t>Valide 48j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 48j (07/08/2026)</t>
+          <t>Valide 47j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (03/09/2026)</t>
+          <t>Valide 74j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 220j (26/01/2027)</t>
+          <t>Valide 219j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (20/11/2026)</t>
+          <t>Valide 153j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>154j</t>
+          <t>153j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (02/11/2026)</t>
+          <t>Valide 135j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,12 +1258,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 235j (09/02/2027)</t>
+          <t>Valide 234j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>235j</t>
+          <t>234j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,12 +1580,12 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 47j (05/08/2026)</t>
+          <t>Valide 46j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (14/10/2026)</t>
+          <t>Valide 116j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (29/08/2026)</t>
+          <t>Valide 70j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (07/12/2026)</t>
+          <t>Valide 170j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (29/08/2026)</t>
+          <t>Valide 70j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 171j (07/12/2026)</t>
+          <t>Valide 170j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (09/10/2026)</t>
+          <t>Valide 111j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>112j</t>
+          <t>111j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (30/11/2026)</t>
+          <t>Valide 163j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 112j (09/10/2026)</t>
+          <t>Valide 111j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>112j</t>
+          <t>111j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 164j (30/11/2026)</t>
+          <t>Valide 163j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 235j (09/02/2027)</t>
+          <t>Valide 234j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>235j</t>
+          <t>234j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (20/11/2026)</t>
+          <t>Valide 153j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 235j (09/02/2027)</t>
+          <t>Valide 234j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>235j</t>
+          <t>234j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 154j (20/11/2026)</t>
+          <t>Valide 153j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,12 +2457,12 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 183j (19/12/2026)</t>
+          <t>Valide 182j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>183j</t>
+          <t>182j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,12 +2511,12 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (19/12/2026)</t>
+          <t>Valide 182j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>183j</t>
+          <t>182j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (13/10/2026)</t>
+          <t>Valide 115j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>115j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (10/10/2026)</t>
+          <t>Valide 112j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>19/06/2026 11:25</t>
+          <t>20/06/2026 10:10</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 21/06/2026 10:37
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 23j (14/07/2026)</t>
+          <t>Expire dans 22j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>23j</t>
+          <t>22j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 257j (05/03/2027)</t>
+          <t>Valide 256j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 48j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 47j (07/08/2026)</t>
+          <t>Valide 46j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (03/09/2026)</t>
+          <t>Valide 73j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 219j (26/01/2027)</t>
+          <t>Valide 218j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (20/11/2026)</t>
+          <t>Valide 152j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>153j</t>
+          <t>152j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (02/11/2026)</t>
+          <t>Valide 134j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 234j (09/02/2027)</t>
+          <t>Valide 233j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>234j</t>
+          <t>233j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 253j (28/02/2027)</t>
+          <t>Valide 252j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 46j (05/08/2026)</t>
+          <t>Valide 45j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 32j (22/07/2026)</t>
+          <t>Valide 31j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (14/10/2026)</t>
+          <t>Valide 115j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>115j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (29/08/2026)</t>
+          <t>Valide 69j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (07/12/2026)</t>
+          <t>Valide 169j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (29/08/2026)</t>
+          <t>Valide 69j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 170j (07/12/2026)</t>
+          <t>Valide 169j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (09/10/2026)</t>
+          <t>Valide 110j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>111j</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (30/11/2026)</t>
+          <t>Valide 162j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 111j (09/10/2026)</t>
+          <t>Valide 110j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>111j</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 163j (30/11/2026)</t>
+          <t>Valide 162j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 234j (09/02/2027)</t>
+          <t>Valide 233j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>234j</t>
+          <t>233j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (20/11/2026)</t>
+          <t>Valide 152j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 234j (09/02/2027)</t>
+          <t>Valide 233j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>234j</t>
+          <t>233j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 153j (20/11/2026)</t>
+          <t>Valide 152j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 182j (19/12/2026)</t>
+          <t>Valide 181j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>182j</t>
+          <t>181j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 41j (31/07/2026)</t>
+          <t>Valide 40j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (19/12/2026)</t>
+          <t>Valide 181j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>182j</t>
+          <t>181j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (31/07/2026)</t>
+          <t>Valide 40j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (13/10/2026)</t>
+          <t>Valide 114j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>115j</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (10/10/2026)</t>
+          <t>Valide 111j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>20/06/2026 10:10</t>
+          <t>21/06/2026 10:33</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 22/06/2026 12:56
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 22j (14/07/2026)</t>
+          <t>Expire dans 21j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>22j</t>
+          <t>21j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 256j (05/03/2027)</t>
+          <t>Valide 255j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 46j (07/08/2026)</t>
+          <t>Valide 45j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (03/09/2026)</t>
+          <t>Valide 72j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 218j (26/01/2027)</t>
+          <t>Valide 217j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (20/11/2026)</t>
+          <t>Valide 151j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>152j</t>
+          <t>151j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (02/11/2026)</t>
+          <t>Valide 132j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 233j (09/02/2027)</t>
+          <t>Valide 232j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>233j</t>
+          <t>232j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 252j (28/02/2027)</t>
+          <t>Valide 250j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,25 +1580,29 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 45j (05/08/2026)</t>
+          <t>Valide 44j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 31j (22/07/2026)</t>
+          <t>Expire dans 29j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr"/>
+          <t>22/06/2026 12:51</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="34">
       <c r="A23" s="8" t="inlineStr">
@@ -1650,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (14/10/2026)</t>
+          <t>Valide 114j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>115j</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (29/08/2026)</t>
+          <t>Valide 68j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (07/12/2026)</t>
+          <t>Valide 168j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (29/08/2026)</t>
+          <t>Valide 68j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 169j (07/12/2026)</t>
+          <t>Valide 168j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (09/10/2026)</t>
+          <t>Valide 109j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>109j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (30/11/2026)</t>
+          <t>Valide 161j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 110j (09/10/2026)</t>
+          <t>Valide 109j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>109j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 162j (30/11/2026)</t>
+          <t>Valide 161j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 233j (09/02/2027)</t>
+          <t>Valide 232j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>233j</t>
+          <t>232j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (20/11/2026)</t>
+          <t>Valide 151j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 233j (09/02/2027)</t>
+          <t>Valide 232j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>233j</t>
+          <t>232j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 152j (20/11/2026)</t>
+          <t>Valide 151j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 181j (19/12/2026)</t>
+          <t>Valide 180j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>181j</t>
+          <t>180j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 40j (31/07/2026)</t>
+          <t>Valide 38j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (19/12/2026)</t>
+          <t>Valide 180j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>181j</t>
+          <t>180j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (31/07/2026)</t>
+          <t>Valide 38j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (13/10/2026)</t>
+          <t>Valide 113j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (10/10/2026)</t>
+          <t>Valide 110j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>21/06/2026 10:33</t>
+          <t>22/06/2026 12:51</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 23/06/2026 10:42
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 21j (14/07/2026)</t>
+          <t>Expire dans 20j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>21j</t>
+          <t>20j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 255j (05/03/2027)</t>
+          <t>Valide 254j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 45j (07/08/2026)</t>
+          <t>Valide 44j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (03/09/2026)</t>
+          <t>Valide 71j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 217j (26/01/2027)</t>
+          <t>Valide 216j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (20/11/2026)</t>
+          <t>Valide 150j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>151j</t>
+          <t>150j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,12 +1258,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 232j (09/02/2027)</t>
+          <t>Valide 231j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>232j</t>
+          <t>231j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,12 +1580,12 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 44j (05/08/2026)</t>
+          <t>Valide 43j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
@@ -1595,14 +1595,10 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>23/06/2026 10:37</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1" s="34">
       <c r="A23" s="8" t="inlineStr">
@@ -1654,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (14/10/2026)</t>
+          <t>Valide 113j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (29/08/2026)</t>
+          <t>Valide 67j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (07/12/2026)</t>
+          <t>Valide 167j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (29/08/2026)</t>
+          <t>Valide 67j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 168j (07/12/2026)</t>
+          <t>Valide 167j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (09/10/2026)</t>
+          <t>Valide 108j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>109j</t>
+          <t>108j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (30/11/2026)</t>
+          <t>Valide 160j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 109j (09/10/2026)</t>
+          <t>Valide 108j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>109j</t>
+          <t>108j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 161j (30/11/2026)</t>
+          <t>Valide 160j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 232j (09/02/2027)</t>
+          <t>Valide 231j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>232j</t>
+          <t>231j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (20/11/2026)</t>
+          <t>Valide 150j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 232j (09/02/2027)</t>
+          <t>Valide 231j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>232j</t>
+          <t>231j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 151j (20/11/2026)</t>
+          <t>Valide 150j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,12 +2457,12 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 180j (19/12/2026)</t>
+          <t>Valide 179j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>179j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
@@ -2476,7 +2472,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,12 +2511,12 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (19/12/2026)</t>
+          <t>Valide 179j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>179j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
@@ -2530,7 +2526,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (13/10/2026)</t>
+          <t>Valide 112j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>112j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (10/10/2026)</t>
+          <t>Valide 109j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>22/06/2026 12:51</t>
+          <t>23/06/2026 10:37</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 24/06/2026 10:39
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 20j (14/07/2026)</t>
+          <t>Expire dans 19j (14/07/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>20j</t>
+          <t>19j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 254j (05/03/2027)</t>
+          <t>Valide 253j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 44j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 44j (07/08/2026)</t>
+          <t>Valide 43j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (03/09/2026)</t>
+          <t>Valide 70j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 216j (26/01/2027)</t>
+          <t>Valide 215j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (20/11/2026)</t>
+          <t>Valide 149j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>150j</t>
+          <t>149j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (02/11/2026)</t>
+          <t>Valide 131j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 231j (09/02/2027)</t>
+          <t>Valide 230j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>231j</t>
+          <t>230j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 250j (28/02/2027)</t>
+          <t>Valide 249j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 43j (05/08/2026)</t>
+          <t>Valide 42j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 29j (22/07/2026)</t>
+          <t>Expire dans 28j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (14/10/2026)</t>
+          <t>Valide 112j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>112j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (29/08/2026)</t>
+          <t>Valide 66j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (07/12/2026)</t>
+          <t>Valide 166j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (29/08/2026)</t>
+          <t>Valide 66j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 167j (07/12/2026)</t>
+          <t>Valide 166j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (09/10/2026)</t>
+          <t>Valide 107j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>108j</t>
+          <t>107j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (30/11/2026)</t>
+          <t>Valide 159j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 108j (09/10/2026)</t>
+          <t>Valide 107j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>108j</t>
+          <t>107j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 160j (30/11/2026)</t>
+          <t>Valide 159j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 231j (09/02/2027)</t>
+          <t>Valide 230j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>231j</t>
+          <t>230j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (20/11/2026)</t>
+          <t>Valide 149j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 231j (09/02/2027)</t>
+          <t>Valide 230j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>231j</t>
+          <t>230j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 150j (20/11/2026)</t>
+          <t>Valide 149j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 179j (19/12/2026)</t>
+          <t>Valide 178j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>179j</t>
+          <t>178j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 38j (31/07/2026)</t>
+          <t>Valide 37j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (19/12/2026)</t>
+          <t>Valide 178j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>179j</t>
+          <t>178j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (31/07/2026)</t>
+          <t>Valide 37j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (13/10/2026)</t>
+          <t>Valide 111j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>112j</t>
+          <t>111j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (10/10/2026)</t>
+          <t>Valide 108j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>23/06/2026 10:37</t>
+          <t>24/06/2026 10:24</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 25/06/2026 10:21
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 19j (14/07/2026)</t>
+          <t>Valide 89j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>19j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 253j (05/03/2027)</t>
+          <t>Valide 252j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 44j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 43j (07/08/2026)</t>
+          <t>Valide 42j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (03/09/2026)</t>
+          <t>Valide 69j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 215j (26/01/2027)</t>
+          <t>Valide 214j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (20/11/2026)</t>
+          <t>Valide 148j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>149j</t>
+          <t>148j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (02/11/2026)</t>
+          <t>Valide 130j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 230j (09/02/2027)</t>
+          <t>Valide 229j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>230j</t>
+          <t>229j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 249j (28/02/2027)</t>
+          <t>Valide 248j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 42j (05/08/2026)</t>
+          <t>Valide 41j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 28j (22/07/2026)</t>
+          <t>Expire dans 27j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (14/10/2026)</t>
+          <t>Valide 111j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>112j</t>
+          <t>111j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (29/08/2026)</t>
+          <t>Valide 65j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (07/12/2026)</t>
+          <t>Valide 165j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (29/08/2026)</t>
+          <t>Valide 65j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 166j (07/12/2026)</t>
+          <t>Valide 165j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (09/10/2026)</t>
+          <t>Valide 106j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>107j</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (30/11/2026)</t>
+          <t>Valide 158j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 107j (09/10/2026)</t>
+          <t>Valide 106j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>107j</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 159j (30/11/2026)</t>
+          <t>Valide 158j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 230j (09/02/2027)</t>
+          <t>Valide 229j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>230j</t>
+          <t>229j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (20/11/2026)</t>
+          <t>Valide 148j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 230j (09/02/2027)</t>
+          <t>Valide 229j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>230j</t>
+          <t>229j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 149j (20/11/2026)</t>
+          <t>Valide 148j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 178j (19/12/2026)</t>
+          <t>Valide 177j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>178j</t>
+          <t>177j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 37j (31/07/2026)</t>
+          <t>Valide 36j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (19/12/2026)</t>
+          <t>Valide 177j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>178j</t>
+          <t>177j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (31/07/2026)</t>
+          <t>Valide 36j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (13/10/2026)</t>
+          <t>Valide 110j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>111j</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (10/10/2026)</t>
+          <t>Valide 107j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>24/06/2026 10:24</t>
+          <t>25/06/2026 10:16</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 26/06/2026 10:29
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (23/09/2026)</t>
+          <t>Valide 88j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 252j (05/03/2027)</t>
+          <t>Valide 251j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 42j (07/08/2026)</t>
+          <t>Valide 41j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (03/09/2026)</t>
+          <t>Valide 68j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 214j (26/01/2027)</t>
+          <t>Valide 213j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (20/11/2026)</t>
+          <t>Valide 147j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>148j</t>
+          <t>147j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (02/11/2026)</t>
+          <t>Valide 129j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 229j (09/02/2027)</t>
+          <t>Valide 228j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>229j</t>
+          <t>228j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 248j (28/02/2027)</t>
+          <t>Valide 247j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 41j (05/08/2026)</t>
+          <t>Valide 40j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 27j (22/07/2026)</t>
+          <t>Expire dans 26j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (14/10/2026)</t>
+          <t>Valide 110j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>111j</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (29/08/2026)</t>
+          <t>Valide 64j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (07/12/2026)</t>
+          <t>Valide 164j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 65j (29/08/2026)</t>
+          <t>Valide 64j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 165j (07/12/2026)</t>
+          <t>Valide 164j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (09/10/2026)</t>
+          <t>Valide 105j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (30/11/2026)</t>
+          <t>Valide 157j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 106j (09/10/2026)</t>
+          <t>Valide 105j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 158j (30/11/2026)</t>
+          <t>Valide 157j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 229j (09/02/2027)</t>
+          <t>Valide 228j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>229j</t>
+          <t>228j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (20/11/2026)</t>
+          <t>Valide 147j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 229j (09/02/2027)</t>
+          <t>Valide 228j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>229j</t>
+          <t>228j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 148j (20/11/2026)</t>
+          <t>Valide 147j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 177j (19/12/2026)</t>
+          <t>Valide 176j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>177j</t>
+          <t>176j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 36j (31/07/2026)</t>
+          <t>Valide 35j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (19/12/2026)</t>
+          <t>Valide 176j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>177j</t>
+          <t>176j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (31/07/2026)</t>
+          <t>Valide 35j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (13/10/2026)</t>
+          <t>Valide 109j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>109j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (10/10/2026)</t>
+          <t>Valide 106j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>25/06/2026 10:16</t>
+          <t>26/06/2026 10:24</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 27/06/2026 09:35
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (23/09/2026)</t>
+          <t>Valide 87j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 251j (05/03/2027)</t>
+          <t>Valide 250j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 41j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 41j (07/08/2026)</t>
+          <t>Valide 40j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (03/09/2026)</t>
+          <t>Valide 67j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 213j (26/01/2027)</t>
+          <t>Valide 212j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (20/11/2026)</t>
+          <t>Valide 146j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>147j</t>
+          <t>146j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (02/11/2026)</t>
+          <t>Valide 128j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 228j (09/02/2027)</t>
+          <t>Valide 227j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>228j</t>
+          <t>227j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 247j (28/02/2027)</t>
+          <t>Valide 246j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 40j (05/08/2026)</t>
+          <t>Valide 39j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 26j (22/07/2026)</t>
+          <t>Expire dans 25j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (14/10/2026)</t>
+          <t>Valide 109j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>109j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (29/08/2026)</t>
+          <t>Valide 63j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (07/12/2026)</t>
+          <t>Valide 163j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (29/08/2026)</t>
+          <t>Valide 63j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 164j (07/12/2026)</t>
+          <t>Valide 163j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (09/10/2026)</t>
+          <t>Valide 104j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (30/11/2026)</t>
+          <t>Valide 156j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 105j (09/10/2026)</t>
+          <t>Valide 104j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 157j (30/11/2026)</t>
+          <t>Valide 156j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 228j (09/02/2027)</t>
+          <t>Valide 227j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>228j</t>
+          <t>227j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (20/11/2026)</t>
+          <t>Valide 146j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 228j (09/02/2027)</t>
+          <t>Valide 227j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>228j</t>
+          <t>227j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 147j (20/11/2026)</t>
+          <t>Valide 146j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 176j (19/12/2026)</t>
+          <t>Valide 175j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>176j</t>
+          <t>175j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 35j (31/07/2026)</t>
+          <t>Valide 34j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (19/12/2026)</t>
+          <t>Valide 175j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>176j</t>
+          <t>175j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (31/07/2026)</t>
+          <t>Valide 34j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (13/10/2026)</t>
+          <t>Valide 108j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>109j</t>
+          <t>108j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (10/10/2026)</t>
+          <t>Valide 105j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>26/06/2026 10:24</t>
+          <t>27/06/2026 09:30</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 28/06/2026 10:11
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (23/09/2026)</t>
+          <t>Valide 86j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 250j (05/03/2027)</t>
+          <t>Valide 249j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 41j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 40j (07/08/2026)</t>
+          <t>Valide 39j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (03/09/2026)</t>
+          <t>Valide 66j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 212j (26/01/2027)</t>
+          <t>Valide 211j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (20/11/2026)</t>
+          <t>Valide 145j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>146j</t>
+          <t>145j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (02/11/2026)</t>
+          <t>Valide 127j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 227j (09/02/2027)</t>
+          <t>Valide 226j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>227j</t>
+          <t>226j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 246j (28/02/2027)</t>
+          <t>Valide 245j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 39j (05/08/2026)</t>
+          <t>Valide 38j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 25j (22/07/2026)</t>
+          <t>Expire dans 24j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (14/10/2026)</t>
+          <t>Valide 108j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>109j</t>
+          <t>108j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (29/08/2026)</t>
+          <t>Valide 62j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (07/12/2026)</t>
+          <t>Valide 162j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (29/08/2026)</t>
+          <t>Valide 62j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 163j (07/12/2026)</t>
+          <t>Valide 162j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (09/10/2026)</t>
+          <t>Valide 103j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (30/11/2026)</t>
+          <t>Valide 155j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 104j (09/10/2026)</t>
+          <t>Valide 103j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 156j (30/11/2026)</t>
+          <t>Valide 155j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 227j (09/02/2027)</t>
+          <t>Valide 226j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>227j</t>
+          <t>226j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (20/11/2026)</t>
+          <t>Valide 145j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 227j (09/02/2027)</t>
+          <t>Valide 226j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>227j</t>
+          <t>226j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 146j (20/11/2026)</t>
+          <t>Valide 145j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 175j (19/12/2026)</t>
+          <t>Valide 174j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>174j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 34j (31/07/2026)</t>
+          <t>Valide 33j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (19/12/2026)</t>
+          <t>Valide 174j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>174j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (31/07/2026)</t>
+          <t>Valide 33j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (13/10/2026)</t>
+          <t>Valide 107j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>108j</t>
+          <t>107j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (10/10/2026)</t>
+          <t>Valide 104j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>27/06/2026 09:30</t>
+          <t>28/06/2026 10:05</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 29/06/2026 12:07
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (23/09/2026)</t>
+          <t>Valide 85j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 249j (05/03/2027)</t>
+          <t>Valide 248j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 39j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 39j (07/08/2026)</t>
+          <t>Valide 38j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (03/09/2026)</t>
+          <t>Valide 65j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 211j (26/01/2027)</t>
+          <t>Valide 210j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (20/11/2026)</t>
+          <t>Valide 144j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>145j</t>
+          <t>144j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (02/11/2026)</t>
+          <t>Valide 126j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 226j (09/02/2027)</t>
+          <t>Valide 225j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>226j</t>
+          <t>225j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 245j (28/02/2027)</t>
+          <t>Valide 243j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 38j (05/08/2026)</t>
+          <t>Valide 37j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 24j (22/07/2026)</t>
+          <t>Expire dans 22j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (14/10/2026)</t>
+          <t>Valide 107j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>108j</t>
+          <t>107j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (29/08/2026)</t>
+          <t>Valide 61j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (07/12/2026)</t>
+          <t>Valide 161j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (29/08/2026)</t>
+          <t>Valide 61j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 162j (07/12/2026)</t>
+          <t>Valide 161j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (09/10/2026)</t>
+          <t>Valide 102j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (30/11/2026)</t>
+          <t>Valide 154j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 103j (09/10/2026)</t>
+          <t>Valide 102j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 155j (30/11/2026)</t>
+          <t>Valide 154j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 226j (09/02/2027)</t>
+          <t>Valide 225j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>226j</t>
+          <t>225j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (20/11/2026)</t>
+          <t>Valide 144j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 226j (09/02/2027)</t>
+          <t>Valide 225j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>226j</t>
+          <t>225j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 145j (20/11/2026)</t>
+          <t>Valide 144j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 174j (19/12/2026)</t>
+          <t>Valide 173j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>174j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 33j (31/07/2026)</t>
+          <t>Valide 31j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (19/12/2026)</t>
+          <t>Valide 173j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>174j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (31/07/2026)</t>
+          <t>Valide 31j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (13/10/2026)</t>
+          <t>Valide 106j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>107j</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (10/10/2026)</t>
+          <t>Valide 103j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>28/06/2026 10:05</t>
+          <t>29/06/2026 12:01</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 30/06/2026 10:40
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (23/09/2026)</t>
+          <t>Valide 84j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 248j (05/03/2027)</t>
+          <t>Valide 247j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 39j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 38j (07/08/2026)</t>
+          <t>Valide 37j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (03/09/2026)</t>
+          <t>Valide 64j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 210j (26/01/2027)</t>
+          <t>Valide 209j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (20/11/2026)</t>
+          <t>Valide 143j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>144j</t>
+          <t>143j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (02/11/2026)</t>
+          <t>Valide 125j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,12 +1258,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 225j (09/02/2027)</t>
+          <t>Valide 224j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>225j</t>
+          <t>224j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,12 +1580,12 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 37j (05/08/2026)</t>
+          <t>Valide 36j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (14/10/2026)</t>
+          <t>Valide 106j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>107j</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (29/08/2026)</t>
+          <t>Valide 60j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (07/12/2026)</t>
+          <t>Valide 160j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (29/08/2026)</t>
+          <t>Valide 60j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 161j (07/12/2026)</t>
+          <t>Valide 160j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (09/10/2026)</t>
+          <t>Valide 101j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (30/11/2026)</t>
+          <t>Valide 153j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 102j (09/10/2026)</t>
+          <t>Valide 101j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 154j (30/11/2026)</t>
+          <t>Valide 153j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 225j (09/02/2027)</t>
+          <t>Valide 224j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>225j</t>
+          <t>224j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (20/11/2026)</t>
+          <t>Valide 143j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 225j (09/02/2027)</t>
+          <t>Valide 224j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>225j</t>
+          <t>224j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 144j (20/11/2026)</t>
+          <t>Valide 143j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,12 +2457,12 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 173j (19/12/2026)</t>
+          <t>Valide 172j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>173j</t>
+          <t>172j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,12 +2511,12 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (19/12/2026)</t>
+          <t>Valide 172j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>173j</t>
+          <t>172j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (13/10/2026)</t>
+          <t>Valide 105j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (10/10/2026)</t>
+          <t>Valide 102j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>29/06/2026 12:01</t>
+          <t>30/06/2026 10:32</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 01/07/2026 10:49
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (23/09/2026)</t>
+          <t>Valide 83j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 247j (05/03/2027)</t>
+          <t>Valide 246j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 37j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 37j (07/08/2026)</t>
+          <t>Valide 36j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (03/09/2026)</t>
+          <t>Valide 63j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 209j (26/01/2027)</t>
+          <t>Valide 208j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (20/11/2026)</t>
+          <t>Valide 142j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>143j</t>
+          <t>142j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (02/11/2026)</t>
+          <t>Valide 124j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 224j (09/02/2027)</t>
+          <t>Valide 223j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>224j</t>
+          <t>223j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 243j (28/02/2027)</t>
+          <t>Valide 242j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 36j (05/08/2026)</t>
+          <t>Valide 35j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 22j (22/07/2026)</t>
+          <t>Expire dans 21j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (14/10/2026)</t>
+          <t>Valide 105j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (29/08/2026)</t>
+          <t>Valide 59j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (07/12/2026)</t>
+          <t>Valide 159j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 60j (29/08/2026)</t>
+          <t>Valide 59j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 160j (07/12/2026)</t>
+          <t>Valide 159j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 101j (09/10/2026)</t>
+          <t>Valide 100j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>101j</t>
+          <t>100j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (30/11/2026)</t>
+          <t>Valide 152j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 101j (09/10/2026)</t>
+          <t>Valide 100j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>101j</t>
+          <t>100j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 153j (30/11/2026)</t>
+          <t>Valide 152j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 224j (09/02/2027)</t>
+          <t>Valide 223j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>224j</t>
+          <t>223j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (20/11/2026)</t>
+          <t>Valide 142j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 224j (09/02/2027)</t>
+          <t>Valide 223j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>224j</t>
+          <t>223j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 143j (20/11/2026)</t>
+          <t>Valide 142j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,25 +2457,29 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 172j (19/12/2026)</t>
+          <t>Valide 171j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>172j</t>
+          <t>171j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 31j (31/07/2026)</t>
+          <t>Expire dans 30j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr"/>
+          <t>01/07/2026 10:43</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1" s="34">
       <c r="A43" s="8" t="inlineStr">
@@ -2511,25 +2515,29 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (19/12/2026)</t>
+          <t>Valide 171j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>172j</t>
+          <t>171j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (31/07/2026)</t>
+          <t>Expire dans 30j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr"/>
+          <t>01/07/2026 10:43</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="44" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A44" s="3" t="inlineStr">
@@ -2725,22 +2733,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (13/10/2026)</t>
+          <t>Valide 104j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (10/10/2026)</t>
+          <t>Valide 101j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>30/06/2026 10:32</t>
+          <t>01/07/2026 10:43</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 02/07/2026 10:16
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (23/09/2026)</t>
+          <t>Valide 82j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 246j (05/03/2027)</t>
+          <t>Valide 245j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 37j (07/08/2026)</t>
+          <t>Valide 36j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 36j (07/08/2026)</t>
+          <t>Valide 35j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (03/09/2026)</t>
+          <t>Valide 62j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 208j (26/01/2027)</t>
+          <t>Valide 207j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (20/11/2026)</t>
+          <t>Valide 141j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>142j</t>
+          <t>141j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (02/11/2026)</t>
+          <t>Valide 123j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 223j (09/02/2027)</t>
+          <t>Valide 222j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>223j</t>
+          <t>222j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 242j (28/02/2027)</t>
+          <t>Valide 241j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 35j (05/08/2026)</t>
+          <t>Valide 34j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 21j (22/07/2026)</t>
+          <t>Expire dans 20j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (14/10/2026)</t>
+          <t>Valide 104j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (29/08/2026)</t>
+          <t>Valide 58j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (07/12/2026)</t>
+          <t>Valide 158j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 59j (29/08/2026)</t>
+          <t>Valide 58j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 159j (07/12/2026)</t>
+          <t>Valide 158j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 100j (09/10/2026)</t>
+          <t>Valide 99j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>100j</t>
+          <t>99j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (30/11/2026)</t>
+          <t>Valide 151j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 100j (09/10/2026)</t>
+          <t>Valide 99j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>100j</t>
+          <t>99j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 152j (30/11/2026)</t>
+          <t>Valide 151j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 223j (09/02/2027)</t>
+          <t>Valide 222j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>223j</t>
+          <t>222j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (20/11/2026)</t>
+          <t>Valide 141j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 223j (09/02/2027)</t>
+          <t>Valide 222j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>223j</t>
+          <t>222j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 142j (20/11/2026)</t>
+          <t>Valide 141j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,29 +2457,25 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 171j (19/12/2026)</t>
+          <t>Valide 170j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>171j</t>
+          <t>170j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 30j (31/07/2026)</t>
+          <t>Expire dans 29j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>02/07/2026 10:11</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr"/>
     </row>
     <row r="43" ht="18" customHeight="1" s="34">
       <c r="A43" s="8" t="inlineStr">
@@ -2515,29 +2511,25 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (19/12/2026)</t>
+          <t>Valide 170j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>171j</t>
+          <t>170j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (31/07/2026)</t>
+          <t>Expire dans 29j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>02/07/2026 10:11</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr"/>
     </row>
     <row r="44" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A44" s="3" t="inlineStr">
@@ -2733,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (13/10/2026)</t>
+          <t>Valide 103j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 101j (10/10/2026)</t>
+          <t>Valide 100j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>01/07/2026 10:43</t>
+          <t>02/07/2026 10:11</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 03/07/2026 10:13
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (23/09/2026)</t>
+          <t>Valide 81j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 245j (05/03/2027)</t>
+          <t>Valide 244j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 36j (07/08/2026)</t>
+          <t>Valide 35j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 35j (07/08/2026)</t>
+          <t>Valide 34j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (03/09/2026)</t>
+          <t>Valide 61j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 207j (26/01/2027)</t>
+          <t>Valide 206j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (20/11/2026)</t>
+          <t>Valide 140j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>141j</t>
+          <t>140j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (02/11/2026)</t>
+          <t>Valide 122j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 222j (09/02/2027)</t>
+          <t>Valide 221j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>222j</t>
+          <t>221j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 241j (28/02/2027)</t>
+          <t>Valide 240j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 34j (05/08/2026)</t>
+          <t>Valide 33j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 20j (22/07/2026)</t>
+          <t>Expire dans 19j (22/07/2026)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (14/10/2026)</t>
+          <t>Valide 103j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (29/08/2026)</t>
+          <t>Valide 57j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (07/12/2026)</t>
+          <t>Valide 157j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 58j (29/08/2026)</t>
+          <t>Valide 57j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 158j (07/12/2026)</t>
+          <t>Valide 157j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 99j (09/10/2026)</t>
+          <t>Valide 98j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>99j</t>
+          <t>98j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (30/11/2026)</t>
+          <t>Valide 150j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 99j (09/10/2026)</t>
+          <t>Valide 98j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>99j</t>
+          <t>98j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 151j (30/11/2026)</t>
+          <t>Valide 150j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 222j (09/02/2027)</t>
+          <t>Valide 221j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>222j</t>
+          <t>221j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (20/11/2026)</t>
+          <t>Valide 140j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 222j (09/02/2027)</t>
+          <t>Valide 221j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>222j</t>
+          <t>221j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 141j (20/11/2026)</t>
+          <t>Valide 140j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 170j (19/12/2026)</t>
+          <t>Valide 169j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>170j</t>
+          <t>169j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 29j (31/07/2026)</t>
+          <t>Expire dans 28j (31/07/2026)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (19/12/2026)</t>
+          <t>Valide 169j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>170j</t>
+          <t>169j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (31/07/2026)</t>
+          <t>Expire dans 28j (31/07/2026)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (13/10/2026)</t>
+          <t>Valide 102j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 100j (10/10/2026)</t>
+          <t>Valide 99j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>02/07/2026 10:11</t>
+          <t>03/07/2026 10:07</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 04/07/2026 09:31
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (23/09/2026)</t>
+          <t>Valide 80j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 244j (05/03/2027)</t>
+          <t>Valide 243j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 35j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 34j (07/08/2026)</t>
+          <t>Valide 33j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (03/09/2026)</t>
+          <t>Valide 60j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 206j (26/01/2027)</t>
+          <t>Valide 205j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (20/11/2026)</t>
+          <t>Valide 139j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>140j</t>
+          <t>139j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (02/11/2026)</t>
+          <t>Valide 121j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 221j (09/02/2027)</t>
+          <t>Valide 220j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>221j</t>
+          <t>220j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 240j (28/02/2027)</t>
+          <t>Valide 239j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 33j (05/08/2026)</t>
+          <t>Valide 32j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 19j (22/07/2026)</t>
+          <t>Valide 383j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (14/10/2026)</t>
+          <t>Valide 102j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (29/08/2026)</t>
+          <t>Valide 56j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (07/12/2026)</t>
+          <t>Valide 156j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 57j (29/08/2026)</t>
+          <t>Valide 56j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 157j (07/12/2026)</t>
+          <t>Valide 156j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 98j (09/10/2026)</t>
+          <t>Valide 97j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>98j</t>
+          <t>97j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (30/11/2026)</t>
+          <t>Valide 149j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 98j (09/10/2026)</t>
+          <t>Valide 97j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>98j</t>
+          <t>97j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 150j (30/11/2026)</t>
+          <t>Valide 149j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 221j (09/02/2027)</t>
+          <t>Valide 220j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>221j</t>
+          <t>220j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (20/11/2026)</t>
+          <t>Valide 139j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 221j (09/02/2027)</t>
+          <t>Valide 220j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>221j</t>
+          <t>220j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 140j (20/11/2026)</t>
+          <t>Valide 139j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 169j (19/12/2026)</t>
+          <t>Valide 168j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>169j</t>
+          <t>168j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 28j (31/07/2026)</t>
+          <t>Valide 392j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (19/12/2026)</t>
+          <t>Valide 168j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>169j</t>
+          <t>168j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 28j (31/07/2026)</t>
+          <t>Valide 392j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (13/10/2026)</t>
+          <t>Valide 101j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 99j (10/10/2026)</t>
+          <t>Valide 98j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>03/07/2026 10:07</t>
+          <t>04/07/2026 09:24</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 05/07/2026 09:48
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (23/09/2026)</t>
+          <t>Valide 79j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 243j (05/03/2027)</t>
+          <t>Valide 242j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 33j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 33j (07/08/2026)</t>
+          <t>Valide 32j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (03/09/2026)</t>
+          <t>Valide 59j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 205j (26/01/2027)</t>
+          <t>Valide 204j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (20/11/2026)</t>
+          <t>Valide 138j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>139j</t>
+          <t>138j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (02/11/2026)</t>
+          <t>Valide 120j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 220j (09/02/2027)</t>
+          <t>Valide 219j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>220j</t>
+          <t>219j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 239j (28/02/2027)</t>
+          <t>Valide 238j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 32j (05/08/2026)</t>
+          <t>Valide 31j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 383j (22/07/2027)</t>
+          <t>Valide 382j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (14/10/2026)</t>
+          <t>Valide 101j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (29/08/2026)</t>
+          <t>Valide 55j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (07/12/2026)</t>
+          <t>Valide 155j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 56j (29/08/2026)</t>
+          <t>Valide 55j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 156j (07/12/2026)</t>
+          <t>Valide 155j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 97j (09/10/2026)</t>
+          <t>Valide 96j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>97j</t>
+          <t>96j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (30/11/2026)</t>
+          <t>Valide 148j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 97j (09/10/2026)</t>
+          <t>Valide 96j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>97j</t>
+          <t>96j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 149j (30/11/2026)</t>
+          <t>Valide 148j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 220j (09/02/2027)</t>
+          <t>Valide 219j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>220j</t>
+          <t>219j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (20/11/2026)</t>
+          <t>Valide 138j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 220j (09/02/2027)</t>
+          <t>Valide 219j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>220j</t>
+          <t>219j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 139j (20/11/2026)</t>
+          <t>Valide 138j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 168j (19/12/2026)</t>
+          <t>Valide 167j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>168j</t>
+          <t>167j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 392j (31/07/2027)</t>
+          <t>Valide 391j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (19/12/2026)</t>
+          <t>Valide 167j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>168j</t>
+          <t>167j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 392j (31/07/2027)</t>
+          <t>Valide 391j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 101j (13/10/2026)</t>
+          <t>Valide 100j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>101j</t>
+          <t>100j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 98j (10/10/2026)</t>
+          <t>Valide 97j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>04/07/2026 09:24</t>
+          <t>05/07/2026 09:43</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 06/07/2026 11:44
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (23/09/2026)</t>
+          <t>Valide 78j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 242j (05/03/2027)</t>
+          <t>Valide 241j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 33j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 32j (07/08/2026)</t>
+          <t>Valide 31j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (03/09/2026)</t>
+          <t>Valide 58j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 204j (26/01/2027)</t>
+          <t>Valide 203j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (20/11/2026)</t>
+          <t>Valide 137j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>138j</t>
+          <t>137j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (02/11/2026)</t>
+          <t>Valide 119j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 219j (09/02/2027)</t>
+          <t>Valide 218j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>219j</t>
+          <t>218j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 238j (28/02/2027)</t>
+          <t>Valide 236j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,25 +1580,29 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 31j (05/08/2026)</t>
+          <t>Expire dans 30j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 382j (22/07/2027)</t>
+          <t>Valide 380j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr"/>
+          <t>06/07/2026 11:39</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="34">
       <c r="A23" s="8" t="inlineStr">
@@ -1650,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 101j (14/10/2026)</t>
+          <t>Valide 100j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>101j</t>
+          <t>100j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (29/08/2026)</t>
+          <t>Valide 54j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (07/12/2026)</t>
+          <t>Valide 154j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 55j (29/08/2026)</t>
+          <t>Valide 54j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 155j (07/12/2026)</t>
+          <t>Valide 154j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 96j (09/10/2026)</t>
+          <t>Valide 95j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>96j</t>
+          <t>95j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (30/11/2026)</t>
+          <t>Valide 147j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 96j (09/10/2026)</t>
+          <t>Valide 95j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>96j</t>
+          <t>95j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 148j (30/11/2026)</t>
+          <t>Valide 147j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 219j (09/02/2027)</t>
+          <t>Valide 218j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>219j</t>
+          <t>218j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (20/11/2026)</t>
+          <t>Valide 137j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 219j (09/02/2027)</t>
+          <t>Valide 218j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>219j</t>
+          <t>218j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 138j (20/11/2026)</t>
+          <t>Valide 137j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 167j (19/12/2026)</t>
+          <t>Valide 166j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>167j</t>
+          <t>166j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 391j (31/07/2027)</t>
+          <t>Valide 389j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (19/12/2026)</t>
+          <t>Valide 166j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>167j</t>
+          <t>166j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 391j (31/07/2027)</t>
+          <t>Valide 389j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 100j (13/10/2026)</t>
+          <t>Valide 99j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>100j</t>
+          <t>99j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 97j (10/10/2026)</t>
+          <t>Valide 96j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>05/07/2026 09:43</t>
+          <t>06/07/2026 11:39</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 07/07/2026 10:32
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (23/09/2026)</t>
+          <t>Valide 77j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 241j (05/03/2027)</t>
+          <t>Valide 240j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,15 +986,19 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 31j (07/08/2026)</t>
+          <t>Expire dans 30j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
+          <t>07/07/2026 10:27</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1" s="34">
       <c r="A8" s="8" t="inlineStr">
@@ -1046,22 +1050,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (03/09/2026)</t>
+          <t>Valide 57j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 203j (26/01/2027)</t>
+          <t>Valide 202j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1156,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (20/11/2026)</t>
+          <t>Valide 136j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>137j</t>
+          <t>136j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (02/11/2026)</t>
+          <t>Valide 118j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,12 +1262,12 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 218j (09/02/2027)</t>
+          <t>Valide 217j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>218j</t>
+          <t>217j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
@@ -1273,7 +1277,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,12 +1584,12 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 30j (05/08/2026)</t>
+          <t>Expire dans 29j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
@@ -1595,14 +1599,10 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>07/07/2026 10:27</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1" s="34">
       <c r="A23" s="8" t="inlineStr">
@@ -1654,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 100j (14/10/2026)</t>
+          <t>Valide 99j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>100j</t>
+          <t>99j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (29/08/2026)</t>
+          <t>Valide 53j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (07/12/2026)</t>
+          <t>Valide 153j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (29/08/2026)</t>
+          <t>Valide 53j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 154j (07/12/2026)</t>
+          <t>Valide 153j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 95j (09/10/2026)</t>
+          <t>Valide 94j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>95j</t>
+          <t>94j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (30/11/2026)</t>
+          <t>Valide 146j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 95j (09/10/2026)</t>
+          <t>Valide 94j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>95j</t>
+          <t>94j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 147j (30/11/2026)</t>
+          <t>Valide 146j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 218j (09/02/2027)</t>
+          <t>Valide 217j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>218j</t>
+          <t>217j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (20/11/2026)</t>
+          <t>Valide 136j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 218j (09/02/2027)</t>
+          <t>Valide 217j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>218j</t>
+          <t>217j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 137j (20/11/2026)</t>
+          <t>Valide 136j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,12 +2461,12 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 166j (19/12/2026)</t>
+          <t>Valide 165j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>166j</t>
+          <t>165j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,12 +2515,12 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (19/12/2026)</t>
+          <t>Valide 165j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>166j</t>
+          <t>165j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 99j (13/10/2026)</t>
+          <t>Valide 98j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>99j</t>
+          <t>98j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 96j (10/10/2026)</t>
+          <t>Valide 95j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>06/07/2026 11:39</t>
+          <t>07/07/2026 10:27</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 08/07/2026 09:35
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (23/09/2026)</t>
+          <t>Valide 76j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 240j (05/03/2027)</t>
+          <t>Valide 239j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Expire dans 30j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 30j (07/08/2026)</t>
+          <t>Expire dans 29j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1050,22 +1050,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (03/09/2026)</t>
+          <t>Valide 56j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 202j (26/01/2027)</t>
+          <t>Valide 201j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1156,22 +1156,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (20/11/2026)</t>
+          <t>Valide 135j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>136j</t>
+          <t>135j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (02/11/2026)</t>
+          <t>Valide 117j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1262,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 217j (09/02/2027)</t>
+          <t>Valide 216j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>217j</t>
+          <t>216j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 236j (28/02/2027)</t>
+          <t>Valide 235j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 29j (05/08/2026)</t>
+          <t>Expire dans 28j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>28j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 380j (22/07/2027)</t>
+          <t>Valide 379j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 99j (14/10/2026)</t>
+          <t>Valide 98j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>99j</t>
+          <t>98j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (29/08/2026)</t>
+          <t>Valide 52j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (07/12/2026)</t>
+          <t>Valide 152j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 53j (29/08/2026)</t>
+          <t>Valide 52j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 153j (07/12/2026)</t>
+          <t>Valide 152j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 94j (09/10/2026)</t>
+          <t>Valide 93j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>94j</t>
+          <t>93j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (30/11/2026)</t>
+          <t>Valide 145j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 94j (09/10/2026)</t>
+          <t>Valide 93j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>94j</t>
+          <t>93j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 146j (30/11/2026)</t>
+          <t>Valide 145j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 217j (09/02/2027)</t>
+          <t>Valide 216j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>217j</t>
+          <t>216j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (20/11/2026)</t>
+          <t>Valide 135j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 217j (09/02/2027)</t>
+          <t>Valide 216j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>217j</t>
+          <t>216j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 136j (20/11/2026)</t>
+          <t>Valide 135j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 165j (19/12/2026)</t>
+          <t>Valide 164j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>165j</t>
+          <t>164j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 389j (31/07/2027)</t>
+          <t>Valide 388j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (19/12/2026)</t>
+          <t>Valide 164j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>165j</t>
+          <t>164j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 389j (31/07/2027)</t>
+          <t>Valide 388j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 98j (13/10/2026)</t>
+          <t>Valide 97j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>98j</t>
+          <t>97j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 95j (10/10/2026)</t>
+          <t>Valide 94j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>07/07/2026 10:27</t>
+          <t>08/07/2026 09:27</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 09/07/2026 10:33
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (23/09/2026)</t>
+          <t>Valide 75j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 239j (05/03/2027)</t>
+          <t>Valide 238j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,29 +976,25 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 30j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 29j (07/08/2026)</t>
+          <t>Expire dans 28j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>09/07/2026 10:26</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1" s="34">
       <c r="A8" s="8" t="inlineStr">
@@ -1050,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (03/09/2026)</t>
+          <t>Valide 55j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 201j (26/01/2027)</t>
+          <t>Valide 200j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1156,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (20/11/2026)</t>
+          <t>Valide 134j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>135j</t>
+          <t>134j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (02/11/2026)</t>
+          <t>Valide 116j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1262,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 216j (09/02/2027)</t>
+          <t>Valide 215j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>216j</t>
+          <t>215j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 235j (28/02/2027)</t>
+          <t>Valide 234j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 28j (05/08/2026)</t>
+          <t>Expire dans 27j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>28j</t>
+          <t>27j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 379j (22/07/2027)</t>
+          <t>Valide 378j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 98j (14/10/2026)</t>
+          <t>Valide 97j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>98j</t>
+          <t>97j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (29/08/2026)</t>
+          <t>Valide 51j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (07/12/2026)</t>
+          <t>Valide 151j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 52j (29/08/2026)</t>
+          <t>Valide 51j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 152j (07/12/2026)</t>
+          <t>Valide 151j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 93j (09/10/2026)</t>
+          <t>Valide 92j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>93j</t>
+          <t>92j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (30/11/2026)</t>
+          <t>Valide 144j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 93j (09/10/2026)</t>
+          <t>Valide 92j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>93j</t>
+          <t>92j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 145j (30/11/2026)</t>
+          <t>Valide 144j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 216j (09/02/2027)</t>
+          <t>Valide 215j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>216j</t>
+          <t>215j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (20/11/2026)</t>
+          <t>Valide 134j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 216j (09/02/2027)</t>
+          <t>Valide 215j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>216j</t>
+          <t>215j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 135j (20/11/2026)</t>
+          <t>Valide 134j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 164j (19/12/2026)</t>
+          <t>Valide 163j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>164j</t>
+          <t>163j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 388j (31/07/2027)</t>
+          <t>Valide 387j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (19/12/2026)</t>
+          <t>Valide 163j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>164j</t>
+          <t>163j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 388j (31/07/2027)</t>
+          <t>Valide 387j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 97j (13/10/2026)</t>
+          <t>Valide 96j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>97j</t>
+          <t>96j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 94j (10/10/2026)</t>
+          <t>Valide 93j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>08/07/2026 09:27</t>
+          <t>09/07/2026 10:26</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 10/07/2026 10:31
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (23/09/2026)</t>
+          <t>Valide 74j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 238j (05/03/2027)</t>
+          <t>Valide 237j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Expire dans 28j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>28j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 28j (07/08/2026)</t>
+          <t>Expire dans 27j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (03/09/2026)</t>
+          <t>Valide 54j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 200j (26/01/2027)</t>
+          <t>Valide 199j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (20/11/2026)</t>
+          <t>Valide 133j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>134j</t>
+          <t>133j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (02/11/2026)</t>
+          <t>Valide 115j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 215j (09/02/2027)</t>
+          <t>Valide 214j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>215j</t>
+          <t>214j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 234j (28/02/2027)</t>
+          <t>Valide 233j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 27j (05/08/2026)</t>
+          <t>Expire dans 26j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>27j</t>
+          <t>26j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 378j (22/07/2027)</t>
+          <t>Valide 377j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 97j (14/10/2026)</t>
+          <t>Valide 96j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>97j</t>
+          <t>96j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (29/08/2026)</t>
+          <t>Valide 50j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (07/12/2026)</t>
+          <t>Valide 150j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 51j (29/08/2026)</t>
+          <t>Valide 50j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 151j (07/12/2026)</t>
+          <t>Valide 150j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 92j (09/10/2026)</t>
+          <t>Valide 91j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>92j</t>
+          <t>91j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (30/11/2026)</t>
+          <t>Valide 143j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 92j (09/10/2026)</t>
+          <t>Valide 91j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>92j</t>
+          <t>91j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 144j (30/11/2026)</t>
+          <t>Valide 143j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 215j (09/02/2027)</t>
+          <t>Valide 214j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>215j</t>
+          <t>214j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (20/11/2026)</t>
+          <t>Valide 133j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 215j (09/02/2027)</t>
+          <t>Valide 214j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>215j</t>
+          <t>214j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 134j (20/11/2026)</t>
+          <t>Valide 133j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 163j (19/12/2026)</t>
+          <t>Valide 162j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>163j</t>
+          <t>162j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 387j (31/07/2027)</t>
+          <t>Valide 386j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (19/12/2026)</t>
+          <t>Valide 162j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>163j</t>
+          <t>162j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 387j (31/07/2027)</t>
+          <t>Valide 386j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 96j (13/10/2026)</t>
+          <t>Valide 95j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>96j</t>
+          <t>95j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 93j (10/10/2026)</t>
+          <t>Valide 92j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>09/07/2026 10:26</t>
+          <t>10/07/2026 10:25</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 11/07/2026 08:54
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (23/09/2026)</t>
+          <t>Valide 73j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 237j (05/03/2027)</t>
+          <t>Valide 236j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 28j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>28j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 27j (07/08/2026)</t>
+          <t>Date inconnue</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 199j (26/01/2027)</t>
+          <t>Valide 198j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (20/11/2026)</t>
+          <t>Valide 132j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>133j</t>
+          <t>132j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (02/11/2026)</t>
+          <t>Valide 114j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 214j (09/02/2027)</t>
+          <t>Valide 213j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>214j</t>
+          <t>213j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 233j (28/02/2027)</t>
+          <t>Valide 232j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 26j (05/08/2026)</t>
+          <t>Expire dans 25j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>26j</t>
+          <t>25j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 377j (22/07/2027)</t>
+          <t>Valide 376j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 96j (14/10/2026)</t>
+          <t>Valide 95j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>96j</t>
+          <t>95j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (29/08/2026)</t>
+          <t>Valide 49j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (07/12/2026)</t>
+          <t>Valide 149j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 50j (29/08/2026)</t>
+          <t>Valide 49j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 150j (07/12/2026)</t>
+          <t>Valide 149j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 91j (09/10/2026)</t>
+          <t>Valide 90j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>91j</t>
+          <t>90j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (30/11/2026)</t>
+          <t>Valide 142j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 91j (09/10/2026)</t>
+          <t>Valide 90j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>91j</t>
+          <t>90j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 143j (30/11/2026)</t>
+          <t>Valide 142j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 214j (09/02/2027)</t>
+          <t>Valide 213j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>214j</t>
+          <t>213j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (20/11/2026)</t>
+          <t>Valide 132j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 214j (09/02/2027)</t>
+          <t>Valide 213j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>214j</t>
+          <t>213j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 133j (20/11/2026)</t>
+          <t>Valide 132j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 162j (19/12/2026)</t>
+          <t>Valide 161j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>162j</t>
+          <t>161j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 386j (31/07/2027)</t>
+          <t>Valide 385j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (19/12/2026)</t>
+          <t>Valide 161j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>162j</t>
+          <t>161j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 386j (31/07/2027)</t>
+          <t>Valide 385j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 95j (13/10/2026)</t>
+          <t>Valide 94j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>95j</t>
+          <t>94j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 92j (10/10/2026)</t>
+          <t>Valide 91j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>10/07/2026 10:25</t>
+          <t>11/07/2026 08:49</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 12/07/2026 09:09
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (23/09/2026)</t>
+          <t>Valide 72j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 236j (05/03/2027)</t>
+          <t>Valide 235j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Date inconnue</t>
+          <t>Expire dans 25j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (03/09/2026)</t>
+          <t>Valide 53j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 198j (26/01/2027)</t>
+          <t>Valide 197j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (20/11/2026)</t>
+          <t>Valide 131j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>132j</t>
+          <t>131j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (02/11/2026)</t>
+          <t>Valide 113j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 213j (09/02/2027)</t>
+          <t>Valide 212j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>213j</t>
+          <t>212j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 232j (28/02/2027)</t>
+          <t>Valide 231j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 25j (05/08/2026)</t>
+          <t>Expire dans 24j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>25j</t>
+          <t>24j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 376j (22/07/2027)</t>
+          <t>Valide 375j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 95j (14/10/2026)</t>
+          <t>Valide 94j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>95j</t>
+          <t>94j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (29/08/2026)</t>
+          <t>Valide 48j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (07/12/2026)</t>
+          <t>Valide 148j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 49j (29/08/2026)</t>
+          <t>Valide 48j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 149j (07/12/2026)</t>
+          <t>Valide 148j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 90j (09/10/2026)</t>
+          <t>Valide 89j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>90j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (30/11/2026)</t>
+          <t>Valide 141j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 90j (09/10/2026)</t>
+          <t>Valide 89j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>90j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 142j (30/11/2026)</t>
+          <t>Valide 141j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 213j (09/02/2027)</t>
+          <t>Valide 212j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>213j</t>
+          <t>212j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (20/11/2026)</t>
+          <t>Valide 131j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 213j (09/02/2027)</t>
+          <t>Valide 212j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>213j</t>
+          <t>212j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 132j (20/11/2026)</t>
+          <t>Valide 131j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 161j (19/12/2026)</t>
+          <t>Valide 160j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>161j</t>
+          <t>160j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 385j (31/07/2027)</t>
+          <t>Valide 384j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (19/12/2026)</t>
+          <t>Valide 160j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>161j</t>
+          <t>160j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 385j (31/07/2027)</t>
+          <t>Valide 384j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 94j (13/10/2026)</t>
+          <t>Valide 93j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>94j</t>
+          <t>93j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 91j (10/10/2026)</t>
+          <t>Valide 90j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>11/07/2026 08:49</t>
+          <t>12/07/2026 09:05</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 13/07/2026 10:35
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (23/09/2026)</t>
+          <t>Valide 71j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 235j (05/03/2027)</t>
+          <t>Valide 234j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Expire dans 25j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>25j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 25j (07/08/2026)</t>
+          <t>Expire dans 24j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (03/09/2026)</t>
+          <t>Valide 51j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (26/01/2027)</t>
+          <t>Valide 196j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (20/11/2026)</t>
+          <t>Valide 130j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>131j</t>
+          <t>130j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (02/11/2026)</t>
+          <t>Valide 112j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 212j (09/02/2027)</t>
+          <t>Valide 211j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>212j</t>
+          <t>211j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 231j (28/02/2027)</t>
+          <t>Valide 230j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 24j (05/08/2026)</t>
+          <t>Expire dans 23j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>24j</t>
+          <t>23j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 375j (22/07/2027)</t>
+          <t>Valide 374j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 94j (14/10/2026)</t>
+          <t>Valide 93j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>94j</t>
+          <t>93j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (29/08/2026)</t>
+          <t>Valide 47j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (07/12/2026)</t>
+          <t>Valide 147j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 48j (29/08/2026)</t>
+          <t>Valide 47j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 148j (07/12/2026)</t>
+          <t>Valide 147j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (09/10/2026)</t>
+          <t>Valide 88j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (30/11/2026)</t>
+          <t>Valide 140j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (09/10/2026)</t>
+          <t>Valide 88j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 141j (30/11/2026)</t>
+          <t>Valide 140j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 212j (09/02/2027)</t>
+          <t>Valide 211j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>212j</t>
+          <t>211j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (20/11/2026)</t>
+          <t>Valide 130j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 212j (09/02/2027)</t>
+          <t>Valide 211j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>212j</t>
+          <t>211j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 131j (20/11/2026)</t>
+          <t>Valide 130j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 160j (19/12/2026)</t>
+          <t>Valide 159j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>160j</t>
+          <t>159j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 384j (31/07/2027)</t>
+          <t>Valide 383j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (19/12/2026)</t>
+          <t>Valide 159j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>160j</t>
+          <t>159j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 384j (31/07/2027)</t>
+          <t>Valide 383j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 93j (13/10/2026)</t>
+          <t>Valide 92j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>93j</t>
+          <t>92j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 90j (10/10/2026)</t>
+          <t>Valide 89j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>12/07/2026 09:05</t>
+          <t>13/07/2026 10:30</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 14/07/2026 09:10
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (23/09/2026)</t>
+          <t>Valide 70j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 234j (05/03/2027)</t>
+          <t>Valide 233j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 25j (07/08/2026)</t>
+          <t>Expire dans 24j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>25j</t>
+          <t>24j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 24j (07/08/2026)</t>
+          <t>Expire dans 23j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (03/09/2026)</t>
+          <t>Valide 50j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (26/01/2027)</t>
+          <t>Valide 195j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (20/11/2026)</t>
+          <t>Valide 129j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>130j</t>
+          <t>129j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (02/11/2026)</t>
+          <t>Valide 111j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 211j (09/02/2027)</t>
+          <t>Valide 210j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>211j</t>
+          <t>210j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 230j (28/02/2027)</t>
+          <t>Valide 229j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 23j (05/08/2026)</t>
+          <t>Expire dans 22j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>23j</t>
+          <t>22j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 374j (22/07/2027)</t>
+          <t>Valide 373j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 93j (14/10/2026)</t>
+          <t>Valide 92j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>93j</t>
+          <t>92j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (29/08/2026)</t>
+          <t>Valide 46j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (07/12/2026)</t>
+          <t>Valide 146j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 47j (29/08/2026)</t>
+          <t>Valide 46j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 147j (07/12/2026)</t>
+          <t>Valide 146j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (09/10/2026)</t>
+          <t>Valide 87j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (30/11/2026)</t>
+          <t>Valide 139j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 88j (09/10/2026)</t>
+          <t>Valide 87j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 140j (30/11/2026)</t>
+          <t>Valide 139j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 211j (09/02/2027)</t>
+          <t>Valide 210j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>211j</t>
+          <t>210j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (20/11/2026)</t>
+          <t>Valide 129j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 211j (09/02/2027)</t>
+          <t>Valide 210j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>211j</t>
+          <t>210j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 130j (20/11/2026)</t>
+          <t>Valide 129j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 159j (19/12/2026)</t>
+          <t>Valide 158j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>159j</t>
+          <t>158j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 383j (31/07/2027)</t>
+          <t>Valide 382j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (19/12/2026)</t>
+          <t>Valide 158j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>159j</t>
+          <t>158j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 383j (31/07/2027)</t>
+          <t>Valide 382j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 92j (13/10/2026)</t>
+          <t>Valide 91j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>92j</t>
+          <t>91j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (10/10/2026)</t>
+          <t>Valide 88j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>13/07/2026 10:30</t>
+          <t>14/07/2026 09:06</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 15/07/2026 09:15
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (23/09/2026)</t>
+          <t>Valide 69j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 233j (05/03/2027)</t>
+          <t>Valide 232j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 24j (07/08/2026)</t>
+          <t>Expire dans 23j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>24j</t>
+          <t>23j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 23j (07/08/2026)</t>
+          <t>Expire dans 22j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (03/09/2026)</t>
+          <t>Valide 49j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (26/01/2027)</t>
+          <t>Valide 194j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (20/11/2026)</t>
+          <t>Valide 128j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>129j</t>
+          <t>128j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (02/11/2026)</t>
+          <t>Valide 110j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 210j (09/02/2027)</t>
+          <t>Valide 209j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>210j</t>
+          <t>209j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 229j (28/02/2027)</t>
+          <t>Valide 228j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 22j (05/08/2026)</t>
+          <t>Expire dans 21j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>22j</t>
+          <t>21j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 373j (22/07/2027)</t>
+          <t>Valide 372j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 92j (14/10/2026)</t>
+          <t>Valide 91j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>92j</t>
+          <t>91j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (29/08/2026)</t>
+          <t>Valide 45j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (07/12/2026)</t>
+          <t>Valide 145j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 46j (29/08/2026)</t>
+          <t>Valide 45j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 146j (07/12/2026)</t>
+          <t>Valide 145j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (09/10/2026)</t>
+          <t>Valide 86j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (30/11/2026)</t>
+          <t>Valide 138j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (09/10/2026)</t>
+          <t>Valide 86j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 139j (30/11/2026)</t>
+          <t>Valide 138j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 210j (09/02/2027)</t>
+          <t>Valide 209j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>210j</t>
+          <t>209j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (20/11/2026)</t>
+          <t>Valide 128j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 210j (09/02/2027)</t>
+          <t>Valide 209j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>210j</t>
+          <t>209j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 129j (20/11/2026)</t>
+          <t>Valide 128j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 158j (19/12/2026)</t>
+          <t>Valide 157j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>158j</t>
+          <t>157j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 382j (31/07/2027)</t>
+          <t>Valide 381j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (19/12/2026)</t>
+          <t>Valide 157j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>158j</t>
+          <t>157j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 382j (31/07/2027)</t>
+          <t>Valide 381j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 91j (13/10/2026)</t>
+          <t>Valide 90j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>91j</t>
+          <t>90j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (10/10/2026)</t>
+          <t>Valide 87j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>14/07/2026 09:06</t>
+          <t>15/07/2026 09:10</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 16/07/2026 09:22
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (23/09/2026)</t>
+          <t>Valide 68j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 232j (05/03/2027)</t>
+          <t>Valide 231j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 23j (07/08/2026)</t>
+          <t>Expire dans 22j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>23j</t>
+          <t>22j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 22j (07/08/2026)</t>
+          <t>Expire dans 21j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (03/09/2026)</t>
+          <t>Valide 48j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (26/01/2027)</t>
+          <t>Valide 193j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (20/11/2026)</t>
+          <t>Valide 127j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>128j</t>
+          <t>127j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (02/11/2026)</t>
+          <t>Valide 109j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 209j (09/02/2027)</t>
+          <t>Valide 208j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>209j</t>
+          <t>208j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 228j (28/02/2027)</t>
+          <t>Valide 227j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 21j (05/08/2026)</t>
+          <t>Expire dans 20j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>21j</t>
+          <t>20j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 372j (22/07/2027)</t>
+          <t>Valide 371j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 91j (14/10/2026)</t>
+          <t>Valide 90j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>91j</t>
+          <t>90j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (29/08/2026)</t>
+          <t>Valide 44j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (07/12/2026)</t>
+          <t>Valide 144j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 45j (29/08/2026)</t>
+          <t>Valide 44j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 145j (07/12/2026)</t>
+          <t>Valide 144j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (09/10/2026)</t>
+          <t>Valide 85j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (30/11/2026)</t>
+          <t>Valide 137j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (09/10/2026)</t>
+          <t>Valide 85j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 138j (30/11/2026)</t>
+          <t>Valide 137j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 209j (09/02/2027)</t>
+          <t>Valide 208j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>209j</t>
+          <t>208j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (20/11/2026)</t>
+          <t>Valide 127j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 209j (09/02/2027)</t>
+          <t>Valide 208j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>209j</t>
+          <t>208j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 128j (20/11/2026)</t>
+          <t>Valide 127j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 157j (19/12/2026)</t>
+          <t>Valide 156j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>157j</t>
+          <t>156j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 381j (31/07/2027)</t>
+          <t>Valide 380j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (19/12/2026)</t>
+          <t>Valide 156j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>157j</t>
+          <t>156j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 381j (31/07/2027)</t>
+          <t>Valide 380j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 90j (13/10/2026)</t>
+          <t>Valide 89j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>90j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (10/10/2026)</t>
+          <t>Valide 86j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>15/07/2026 09:10</t>
+          <t>16/07/2026 09:17</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 17/07/2026 09:15
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (23/09/2026)</t>
+          <t>Valide 67j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 231j (05/03/2027)</t>
+          <t>Valide 230j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 22j (07/08/2026)</t>
+          <t>Expire dans 21j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>22j</t>
+          <t>21j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 21j (07/08/2026)</t>
+          <t>Expire dans 20j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (03/09/2026)</t>
+          <t>Valide 47j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (26/01/2027)</t>
+          <t>Valide 192j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (20/11/2026)</t>
+          <t>Valide 126j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>127j</t>
+          <t>126j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (02/11/2026)</t>
+          <t>Valide 108j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 208j (09/02/2027)</t>
+          <t>Valide 207j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>208j</t>
+          <t>207j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 227j (28/02/2027)</t>
+          <t>Valide 226j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 20j (05/08/2026)</t>
+          <t>Expire dans 19j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>20j</t>
+          <t>19j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 371j (22/07/2027)</t>
+          <t>Valide 370j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 90j (14/10/2026)</t>
+          <t>Valide 89j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>90j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (29/08/2026)</t>
+          <t>Valide 43j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (07/12/2026)</t>
+          <t>Valide 143j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 44j (29/08/2026)</t>
+          <t>Valide 43j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 144j (07/12/2026)</t>
+          <t>Valide 143j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (09/10/2026)</t>
+          <t>Valide 84j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (30/11/2026)</t>
+          <t>Valide 136j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (09/10/2026)</t>
+          <t>Valide 84j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 137j (30/11/2026)</t>
+          <t>Valide 136j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 208j (09/02/2027)</t>
+          <t>Valide 207j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>208j</t>
+          <t>207j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (20/11/2026)</t>
+          <t>Valide 126j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 208j (09/02/2027)</t>
+          <t>Valide 207j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>208j</t>
+          <t>207j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 127j (20/11/2026)</t>
+          <t>Valide 126j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 156j (19/12/2026)</t>
+          <t>Valide 155j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>156j</t>
+          <t>155j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 380j (31/07/2027)</t>
+          <t>Valide 379j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (19/12/2026)</t>
+          <t>Valide 155j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>156j</t>
+          <t>155j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 380j (31/07/2027)</t>
+          <t>Valide 379j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (13/10/2026)</t>
+          <t>Valide 88j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (10/10/2026)</t>
+          <t>Valide 85j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>16/07/2026 09:17</t>
+          <t>17/07/2026 09:11</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 18/07/2026 08:54
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (23/09/2026)</t>
+          <t>Valide 66j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 230j (05/03/2027)</t>
+          <t>Valide 229j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 21j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>21j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 20j (07/08/2026)</t>
+          <t>Expire dans 19j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (26/01/2027)</t>
+          <t>Valide 191j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (20/11/2026)</t>
+          <t>Valide 125j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>126j</t>
+          <t>125j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (02/11/2026)</t>
+          <t>Valide 107j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 207j (09/02/2027)</t>
+          <t>Valide 206j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>207j</t>
+          <t>206j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 226j (28/02/2027)</t>
+          <t>Valide 225j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 19j (05/08/2026)</t>
+          <t>Expire dans 18j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>19j</t>
+          <t>18j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 370j (22/07/2027)</t>
+          <t>Valide 369j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (14/10/2026)</t>
+          <t>Valide 88j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (29/08/2026)</t>
+          <t>Valide 42j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (07/12/2026)</t>
+          <t>Valide 142j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 43j (29/08/2026)</t>
+          <t>Valide 42j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 143j (07/12/2026)</t>
+          <t>Valide 142j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (09/10/2026)</t>
+          <t>Valide 83j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (30/11/2026)</t>
+          <t>Valide 135j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (09/10/2026)</t>
+          <t>Valide 83j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 136j (30/11/2026)</t>
+          <t>Valide 135j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 207j (09/02/2027)</t>
+          <t>Valide 206j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>207j</t>
+          <t>206j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (20/11/2026)</t>
+          <t>Valide 125j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 207j (09/02/2027)</t>
+          <t>Valide 206j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>207j</t>
+          <t>206j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 126j (20/11/2026)</t>
+          <t>Valide 125j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 155j (19/12/2026)</t>
+          <t>Valide 154j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>155j</t>
+          <t>154j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 379j (31/07/2027)</t>
+          <t>Valide 378j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (19/12/2026)</t>
+          <t>Valide 154j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>155j</t>
+          <t>154j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 379j (31/07/2027)</t>
+          <t>Valide 378j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (13/10/2026)</t>
+          <t>Valide 87j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (10/10/2026)</t>
+          <t>Valide 84j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>17/07/2026 09:11</t>
+          <t>18/07/2026 08:49</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 19/07/2026 09:10
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (23/09/2026)</t>
+          <t>Valide 65j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 229j (05/03/2027)</t>
+          <t>Valide 228j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Expire dans 19j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>19j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 19j (07/08/2026)</t>
+          <t>Expire dans 18j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (03/09/2026)</t>
+          <t>Valide 45j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (26/01/2027)</t>
+          <t>Valide 190j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (20/11/2026)</t>
+          <t>Valide 124j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>125j</t>
+          <t>124j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (02/11/2026)</t>
+          <t>Valide 106j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 206j (09/02/2027)</t>
+          <t>Valide 205j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>206j</t>
+          <t>205j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 225j (28/02/2027)</t>
+          <t>Valide 224j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 18j (05/08/2026)</t>
+          <t>Expire dans 17j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>18j</t>
+          <t>17j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 369j (22/07/2027)</t>
+          <t>Valide 368j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (14/10/2026)</t>
+          <t>Valide 87j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (29/08/2026)</t>
+          <t>Valide 41j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (07/12/2026)</t>
+          <t>Valide 141j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 42j (29/08/2026)</t>
+          <t>Valide 41j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 142j (07/12/2026)</t>
+          <t>Valide 141j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (09/10/2026)</t>
+          <t>Valide 82j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (30/11/2026)</t>
+          <t>Valide 134j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 83j (09/10/2026)</t>
+          <t>Valide 82j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 135j (30/11/2026)</t>
+          <t>Valide 134j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 206j (09/02/2027)</t>
+          <t>Valide 205j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>206j</t>
+          <t>205j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (20/11/2026)</t>
+          <t>Valide 124j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 206j (09/02/2027)</t>
+          <t>Valide 205j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>206j</t>
+          <t>205j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 125j (20/11/2026)</t>
+          <t>Valide 124j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 154j (19/12/2026)</t>
+          <t>Valide 153j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>154j</t>
+          <t>153j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 378j (31/07/2027)</t>
+          <t>Valide 377j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (19/12/2026)</t>
+          <t>Valide 153j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>154j</t>
+          <t>153j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 378j (31/07/2027)</t>
+          <t>Valide 377j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (13/10/2026)</t>
+          <t>Valide 86j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (10/10/2026)</t>
+          <t>Valide 83j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>18/07/2026 08:49</t>
+          <t>19/07/2026 09:06</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 20/07/2026 10:19
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (23/09/2026)</t>
+          <t>Valide 64j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 228j (05/03/2027)</t>
+          <t>Valide 227j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 19j (07/08/2026)</t>
+          <t>Expire dans 18j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>19j</t>
+          <t>18j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 18j (07/08/2026)</t>
+          <t>Expire dans 17j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (03/09/2026)</t>
+          <t>Valide 44j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (26/01/2027)</t>
+          <t>Valide 189j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (20/11/2026)</t>
+          <t>Valide 123j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>124j</t>
+          <t>123j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (02/11/2026)</t>
+          <t>Valide 105j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 205j (09/02/2027)</t>
+          <t>Valide 204j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>205j</t>
+          <t>204j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 224j (28/02/2027)</t>
+          <t>Valide 223j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 17j (05/08/2026)</t>
+          <t>Expire dans 16j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>17j</t>
+          <t>16j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 368j (22/07/2027)</t>
+          <t>Valide 367j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (14/10/2026)</t>
+          <t>Valide 86j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (29/08/2026)</t>
+          <t>Valide 40j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (07/12/2026)</t>
+          <t>Valide 140j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 41j (29/08/2026)</t>
+          <t>Valide 40j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 141j (07/12/2026)</t>
+          <t>Valide 140j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (09/10/2026)</t>
+          <t>Valide 81j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (30/11/2026)</t>
+          <t>Valide 133j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (09/10/2026)</t>
+          <t>Valide 81j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 134j (30/11/2026)</t>
+          <t>Valide 133j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 205j (09/02/2027)</t>
+          <t>Valide 204j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>205j</t>
+          <t>204j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (20/11/2026)</t>
+          <t>Valide 123j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 205j (09/02/2027)</t>
+          <t>Valide 204j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>205j</t>
+          <t>204j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 124j (20/11/2026)</t>
+          <t>Valide 123j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 153j (19/12/2026)</t>
+          <t>Valide 152j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>153j</t>
+          <t>152j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 377j (31/07/2027)</t>
+          <t>Valide 376j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (19/12/2026)</t>
+          <t>Valide 152j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>153j</t>
+          <t>152j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 377j (31/07/2027)</t>
+          <t>Valide 376j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (13/10/2026)</t>
+          <t>Valide 85j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (10/10/2026)</t>
+          <t>Valide 82j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>19/07/2026 09:06</t>
+          <t>20/07/2026 10:14</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 21/07/2026 09:35
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (23/09/2026)</t>
+          <t>Valide 63j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 227j (05/03/2027)</t>
+          <t>Valide 226j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 18j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>18j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 17j (07/08/2026)</t>
+          <t>Expire dans 16j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (03/09/2026)</t>
+          <t>Valide 43j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (26/01/2027)</t>
+          <t>Valide 188j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (20/11/2026)</t>
+          <t>Valide 122j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>123j</t>
+          <t>122j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (02/11/2026)</t>
+          <t>Valide 104j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 204j (09/02/2027)</t>
+          <t>Valide 203j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>204j</t>
+          <t>203j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 223j (28/02/2027)</t>
+          <t>Valide 222j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,25 +1580,29 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 16j (05/08/2026)</t>
+          <t>Expire dans 15j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>16j</t>
+          <t>15j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 367j (22/07/2027)</t>
+          <t>Valide 366j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr"/>
+          <t>21/07/2026 09:29</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1" s="34">
       <c r="A23" s="8" t="inlineStr">
@@ -1650,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (14/10/2026)</t>
+          <t>Valide 85j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (29/08/2026)</t>
+          <t>Valide 39j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (07/12/2026)</t>
+          <t>Valide 139j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 40j (29/08/2026)</t>
+          <t>Valide 39j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 140j (07/12/2026)</t>
+          <t>Valide 139j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (09/10/2026)</t>
+          <t>Valide 80j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (30/11/2026)</t>
+          <t>Valide 132j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 81j (09/10/2026)</t>
+          <t>Valide 80j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 133j (30/11/2026)</t>
+          <t>Valide 132j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 204j (09/02/2027)</t>
+          <t>Valide 203j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>204j</t>
+          <t>203j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (20/11/2026)</t>
+          <t>Valide 122j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 204j (09/02/2027)</t>
+          <t>Valide 203j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>204j</t>
+          <t>203j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 123j (20/11/2026)</t>
+          <t>Valide 122j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 152j (19/12/2026)</t>
+          <t>Valide 151j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>152j</t>
+          <t>151j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 376j (31/07/2027)</t>
+          <t>Valide 375j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (19/12/2026)</t>
+          <t>Valide 151j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>152j</t>
+          <t>151j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 376j (31/07/2027)</t>
+          <t>Valide 375j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (13/10/2026)</t>
+          <t>Valide 84j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (10/10/2026)</t>
+          <t>Valide 81j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>20/07/2026 10:14</t>
+          <t>21/07/2026 09:29</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 22/07/2026 09:33
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (23/09/2026)</t>
+          <t>Valide 62j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 226j (05/03/2027)</t>
+          <t>Valide 225j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,15 +986,19 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 16j (07/08/2026)</t>
+          <t>Expire dans 15j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
+          <t>22/07/2026 09:28</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1" s="34">
       <c r="A8" s="8" t="inlineStr">
@@ -1046,22 +1050,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (03/09/2026)</t>
+          <t>Valide 42j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (26/01/2027)</t>
+          <t>Valide 187j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1156,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (20/11/2026)</t>
+          <t>Valide 121j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>122j</t>
+          <t>121j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (02/11/2026)</t>
+          <t>Valide 103j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 203j (09/02/2027)</t>
+          <t>Valide 202j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>203j</t>
+          <t>202j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 222j (28/02/2027)</t>
+          <t>Valide 221j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,29 +1584,25 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 15j (05/08/2026)</t>
+          <t>Expire dans 14j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>15j</t>
+          <t>14j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 366j (22/07/2027)</t>
+          <t>Valide 365j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>22/07/2026 09:28</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23" ht="18" customHeight="1" s="34">
       <c r="A23" s="8" t="inlineStr">
@@ -1654,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (14/10/2026)</t>
+          <t>Valide 84j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (29/08/2026)</t>
+          <t>Valide 38j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (07/12/2026)</t>
+          <t>Valide 138j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 39j (29/08/2026)</t>
+          <t>Valide 38j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 139j (07/12/2026)</t>
+          <t>Valide 138j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (09/10/2026)</t>
+          <t>Valide 79j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (30/11/2026)</t>
+          <t>Valide 131j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 80j (09/10/2026)</t>
+          <t>Valide 79j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 132j (30/11/2026)</t>
+          <t>Valide 131j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 203j (09/02/2027)</t>
+          <t>Valide 202j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>203j</t>
+          <t>202j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (20/11/2026)</t>
+          <t>Valide 121j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 203j (09/02/2027)</t>
+          <t>Valide 202j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>203j</t>
+          <t>202j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 122j (20/11/2026)</t>
+          <t>Valide 121j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 151j (19/12/2026)</t>
+          <t>Valide 150j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>151j</t>
+          <t>150j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 375j (31/07/2027)</t>
+          <t>Valide 374j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (19/12/2026)</t>
+          <t>Valide 150j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>151j</t>
+          <t>150j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 375j (31/07/2027)</t>
+          <t>Valide 374j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (13/10/2026)</t>
+          <t>Valide 83j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (10/10/2026)</t>
+          <t>Valide 80j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>21/07/2026 09:29</t>
+          <t>22/07/2026 09:28</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 23/07/2026 09:31
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (23/09/2026)</t>
+          <t>Valide 61j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 225j (05/03/2027)</t>
+          <t>Valide 224j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,19 +986,15 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 15j (07/08/2026)</t>
+          <t>Expire dans 14j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>23/07/2026 09:26</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1" s="34">
       <c r="A8" s="8" t="inlineStr">
@@ -1050,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (03/09/2026)</t>
+          <t>Valide 41j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (26/01/2027)</t>
+          <t>Valide 186j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1156,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (20/11/2026)</t>
+          <t>Valide 120j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>121j</t>
+          <t>120j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (02/11/2026)</t>
+          <t>Valide 102j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1262,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 202j (09/02/2027)</t>
+          <t>Valide 201j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>202j</t>
+          <t>201j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 221j (28/02/2027)</t>
+          <t>Valide 220j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 14j (05/08/2026)</t>
+          <t>Expire dans 13j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>14j</t>
+          <t>13j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 365j (22/07/2027)</t>
+          <t>Valide 364j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (14/10/2026)</t>
+          <t>Valide 83j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (29/08/2026)</t>
+          <t>Valide 37j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (07/12/2026)</t>
+          <t>Valide 137j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 38j (29/08/2026)</t>
+          <t>Valide 37j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 138j (07/12/2026)</t>
+          <t>Valide 137j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (09/10/2026)</t>
+          <t>Valide 78j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (30/11/2026)</t>
+          <t>Valide 130j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (09/10/2026)</t>
+          <t>Valide 78j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 131j (30/11/2026)</t>
+          <t>Valide 130j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 202j (09/02/2027)</t>
+          <t>Valide 201j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>202j</t>
+          <t>201j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (20/11/2026)</t>
+          <t>Valide 120j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 202j (09/02/2027)</t>
+          <t>Valide 201j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>202j</t>
+          <t>201j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 121j (20/11/2026)</t>
+          <t>Valide 120j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 150j (19/12/2026)</t>
+          <t>Valide 149j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>150j</t>
+          <t>149j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 374j (31/07/2027)</t>
+          <t>Valide 373j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (19/12/2026)</t>
+          <t>Valide 149j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>150j</t>
+          <t>149j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 374j (31/07/2027)</t>
+          <t>Valide 373j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (13/10/2026)</t>
+          <t>Valide 82j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (10/10/2026)</t>
+          <t>Valide 79j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>22/07/2026 09:28</t>
+          <t>23/07/2026 09:26</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 24/07/2026 09:27
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (23/09/2026)</t>
+          <t>Valide 60j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 224j (05/03/2027)</t>
+          <t>Valide 223j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,25 +976,29 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Expire dans 14j (07/08/2026)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>14j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 14j (07/08/2026)</t>
+          <t>Expire dans 13j (07/08/2026)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
+          <t>24/07/2026 09:22</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1" s="34">
       <c r="A8" s="8" t="inlineStr">
@@ -1046,22 +1050,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (03/09/2026)</t>
+          <t>Valide 40j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 186j (26/01/2027)</t>
+          <t>Valide 185j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1156,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (20/11/2026)</t>
+          <t>Valide 119j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>119j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (02/11/2026)</t>
+          <t>Valide 101j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 201j (09/02/2027)</t>
+          <t>Valide 200j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>201j</t>
+          <t>200j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 220j (28/02/2027)</t>
+          <t>Valide 219j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 13j (05/08/2026)</t>
+          <t>Expire dans 12j (05/08/2026)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>13j</t>
+          <t>12j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 364j (22/07/2027)</t>
+          <t>Valide 363j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (14/10/2026)</t>
+          <t>Valide 82j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (29/08/2026)</t>
+          <t>Valide 36j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (07/12/2026)</t>
+          <t>Valide 136j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 37j (29/08/2026)</t>
+          <t>Valide 36j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 137j (07/12/2026)</t>
+          <t>Valide 136j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (09/10/2026)</t>
+          <t>Valide 77j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (30/11/2026)</t>
+          <t>Valide 129j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (09/10/2026)</t>
+          <t>Valide 77j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 130j (30/11/2026)</t>
+          <t>Valide 129j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 201j (09/02/2027)</t>
+          <t>Valide 200j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>201j</t>
+          <t>200j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (20/11/2026)</t>
+          <t>Valide 119j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 201j (09/02/2027)</t>
+          <t>Valide 200j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>201j</t>
+          <t>200j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 120j (20/11/2026)</t>
+          <t>Valide 119j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 149j (19/12/2026)</t>
+          <t>Valide 148j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>149j</t>
+          <t>148j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 373j (31/07/2027)</t>
+          <t>Valide 372j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (19/12/2026)</t>
+          <t>Valide 148j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>149j</t>
+          <t>148j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 373j (31/07/2027)</t>
+          <t>Valide 372j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (13/10/2026)</t>
+          <t>Valide 81j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (10/10/2026)</t>
+          <t>Valide 78j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>23/07/2026 09:26</t>
+          <t>24/07/2026 09:22</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 25/07/2026 09:08
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (23/09/2026)</t>
+          <t>Valide 59j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 223j (05/03/2027)</t>
+          <t>Valide 222j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,29 +976,25 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 14j (07/08/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>14j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 13j (07/08/2026)</t>
+          <t>Valide 377j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>25/07/2026 09:01</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1" s="34">
       <c r="A8" s="8" t="inlineStr">
@@ -1060,12 +1056,12 @@
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (26/01/2027)</t>
+          <t>Valide 184j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1156,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (20/11/2026)</t>
+          <t>Valide 118j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>119j</t>
+          <t>118j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 101j (02/11/2026)</t>
+          <t>Valide 100j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1262,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 200j (09/02/2027)</t>
+          <t>Valide 199j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>200j</t>
+          <t>199j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 219j (28/02/2027)</t>
+          <t>Valide 218j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 12j (05/08/2026)</t>
+          <t>Valide 197j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>12j</t>
+          <t>197j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 363j (22/07/2027)</t>
+          <t>Valide 362j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (14/10/2026)</t>
+          <t>Valide 81j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (29/08/2026)</t>
+          <t>Valide 35j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (07/12/2026)</t>
+          <t>Valide 135j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 36j (29/08/2026)</t>
+          <t>Valide 35j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 136j (07/12/2026)</t>
+          <t>Valide 135j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (09/10/2026)</t>
+          <t>Valide 76j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (30/11/2026)</t>
+          <t>Valide 128j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (09/10/2026)</t>
+          <t>Valide 76j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 129j (30/11/2026)</t>
+          <t>Valide 128j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 200j (09/02/2027)</t>
+          <t>Valide 199j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>200j</t>
+          <t>199j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (20/11/2026)</t>
+          <t>Valide 118j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 200j (09/02/2027)</t>
+          <t>Valide 199j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>200j</t>
+          <t>199j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 119j (20/11/2026)</t>
+          <t>Valide 118j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 148j (19/12/2026)</t>
+          <t>Valide 147j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>148j</t>
+          <t>147j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 372j (31/07/2027)</t>
+          <t>Valide 371j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (19/12/2026)</t>
+          <t>Valide 147j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>148j</t>
+          <t>147j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 372j (31/07/2027)</t>
+          <t>Valide 371j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (13/10/2026)</t>
+          <t>Valide 80j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (10/10/2026)</t>
+          <t>Valide 77j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>24/07/2026 09:22</t>
+          <t>25/07/2026 09:01</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 26/07/2026 09:22
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (23/09/2026)</t>
+          <t>Valide 58j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 222j (05/03/2027)</t>
+          <t>Valide 221j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 377j (07/08/2027)</t>
+          <t>Valide 376j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (03/09/2026)</t>
+          <t>Valide 38j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 184j (26/01/2027)</t>
+          <t>Valide 183j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (20/11/2026)</t>
+          <t>Valide 117j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>118j</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 100j (02/11/2026)</t>
+          <t>Valide 99j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 199j (09/02/2027)</t>
+          <t>Valide 198j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>199j</t>
+          <t>198j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 218j (28/02/2027)</t>
+          <t>Valide 217j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 197j (07/02/2027)</t>
+          <t>Valide 196j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>197j</t>
+          <t>196j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 362j (22/07/2027)</t>
+          <t>Valide 361j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (14/10/2026)</t>
+          <t>Valide 80j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (29/08/2026)</t>
+          <t>Valide 34j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (07/12/2026)</t>
+          <t>Valide 134j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 35j (29/08/2026)</t>
+          <t>Valide 34j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 135j (07/12/2026)</t>
+          <t>Valide 134j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (09/10/2026)</t>
+          <t>Valide 75j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (30/11/2026)</t>
+          <t>Valide 127j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (09/10/2026)</t>
+          <t>Valide 75j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 128j (30/11/2026)</t>
+          <t>Valide 127j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 199j (09/02/2027)</t>
+          <t>Valide 198j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>199j</t>
+          <t>198j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (20/11/2026)</t>
+          <t>Valide 117j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 199j (09/02/2027)</t>
+          <t>Valide 198j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>199j</t>
+          <t>198j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 118j (20/11/2026)</t>
+          <t>Valide 117j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 147j (19/12/2026)</t>
+          <t>Valide 146j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>147j</t>
+          <t>146j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 371j (31/07/2027)</t>
+          <t>Valide 370j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (19/12/2026)</t>
+          <t>Valide 146j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>147j</t>
+          <t>146j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 371j (31/07/2027)</t>
+          <t>Valide 370j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (13/10/2026)</t>
+          <t>Valide 79j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (10/10/2026)</t>
+          <t>Valide 76j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>25/07/2026 09:01</t>
+          <t>26/07/2026 09:17</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 27/07/2026 10:50
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (23/09/2026)</t>
+          <t>Valide 57j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 221j (05/03/2027)</t>
+          <t>Valide 220j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 376j (07/08/2027)</t>
+          <t>Valide 375j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (03/09/2026)</t>
+          <t>Valide 37j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (26/01/2027)</t>
+          <t>Valide 182j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (20/11/2026)</t>
+          <t>Valide 116j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 99j (02/11/2026)</t>
+          <t>Valide 98j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 198j (09/02/2027)</t>
+          <t>Valide 197j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>198j</t>
+          <t>197j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 217j (28/02/2027)</t>
+          <t>Valide 216j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 196j (07/02/2027)</t>
+          <t>Valide 195j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>196j</t>
+          <t>195j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 361j (22/07/2027)</t>
+          <t>Valide 360j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (14/10/2026)</t>
+          <t>Valide 79j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (29/08/2026)</t>
+          <t>Valide 33j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (07/12/2026)</t>
+          <t>Valide 133j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 34j (29/08/2026)</t>
+          <t>Valide 33j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 134j (07/12/2026)</t>
+          <t>Valide 133j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (09/10/2026)</t>
+          <t>Valide 74j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (30/11/2026)</t>
+          <t>Valide 126j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (09/10/2026)</t>
+          <t>Valide 74j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 127j (30/11/2026)</t>
+          <t>Valide 126j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 198j (09/02/2027)</t>
+          <t>Valide 197j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>198j</t>
+          <t>197j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (20/11/2026)</t>
+          <t>Valide 116j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 198j (09/02/2027)</t>
+          <t>Valide 197j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>198j</t>
+          <t>197j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 117j (20/11/2026)</t>
+          <t>Valide 116j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 146j (19/12/2026)</t>
+          <t>Valide 145j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>146j</t>
+          <t>145j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 370j (31/07/2027)</t>
+          <t>Valide 369j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (19/12/2026)</t>
+          <t>Valide 145j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>146j</t>
+          <t>145j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 370j (31/07/2027)</t>
+          <t>Valide 369j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (13/10/2026)</t>
+          <t>Valide 78j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (10/10/2026)</t>
+          <t>Valide 75j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>26/07/2026 09:17</t>
+          <t>27/07/2026 10:45</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 28/07/2026 09:44
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (23/09/2026)</t>
+          <t>Valide 56j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 220j (05/03/2027)</t>
+          <t>Valide 219j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 375j (07/08/2027)</t>
+          <t>Valide 374j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (03/09/2026)</t>
+          <t>Valide 36j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (26/01/2027)</t>
+          <t>Valide 181j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (20/11/2026)</t>
+          <t>Valide 115j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>115j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 98j (02/11/2026)</t>
+          <t>Valide 97j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (09/02/2027)</t>
+          <t>Valide 196j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>197j</t>
+          <t>196j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 216j (28/02/2027)</t>
+          <t>Valide 215j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 195j (07/02/2027)</t>
+          <t>Valide 194j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>195j</t>
+          <t>194j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 360j (22/07/2027)</t>
+          <t>Valide 359j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (14/10/2026)</t>
+          <t>Valide 78j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (29/08/2026)</t>
+          <t>Valide 32j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (07/12/2026)</t>
+          <t>Valide 132j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 33j (29/08/2026)</t>
+          <t>Valide 32j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 133j (07/12/2026)</t>
+          <t>Valide 132j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (09/10/2026)</t>
+          <t>Valide 73j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (30/11/2026)</t>
+          <t>Valide 125j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 74j (09/10/2026)</t>
+          <t>Valide 73j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 126j (30/11/2026)</t>
+          <t>Valide 125j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (09/02/2027)</t>
+          <t>Valide 196j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>197j</t>
+          <t>196j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (20/11/2026)</t>
+          <t>Valide 115j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 197j (09/02/2027)</t>
+          <t>Valide 196j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>197j</t>
+          <t>196j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 116j (20/11/2026)</t>
+          <t>Valide 115j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 145j (19/12/2026)</t>
+          <t>Valide 144j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>145j</t>
+          <t>144j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 369j (31/07/2027)</t>
+          <t>Valide 368j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (19/12/2026)</t>
+          <t>Valide 144j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>145j</t>
+          <t>144j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 369j (31/07/2027)</t>
+          <t>Valide 368j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (13/10/2026)</t>
+          <t>Valide 77j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (10/10/2026)</t>
+          <t>Valide 74j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>27/07/2026 10:45</t>
+          <t>28/07/2026 09:37</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 29/07/2026 09:45
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (23/09/2026)</t>
+          <t>Valide 55j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 219j (05/03/2027)</t>
+          <t>Valide 218j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 193j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>193j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 374j (07/08/2027)</t>
+          <t>Valide 373j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (03/09/2026)</t>
+          <t>Valide 35j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (26/01/2027)</t>
+          <t>Valide 180j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (20/11/2026)</t>
+          <t>Valide 114j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>115j</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 97j (02/11/2026)</t>
+          <t>Valide 96j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (09/02/2027)</t>
+          <t>Valide 195j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>196j</t>
+          <t>195j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 215j (28/02/2027)</t>
+          <t>Valide 214j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 194j (07/02/2027)</t>
+          <t>Valide 193j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>194j</t>
+          <t>193j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 359j (22/07/2027)</t>
+          <t>Valide 358j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (14/10/2026)</t>
+          <t>Valide 77j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (29/08/2026)</t>
+          <t>Valide 31j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (07/12/2026)</t>
+          <t>Valide 131j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 32j (29/08/2026)</t>
+          <t>Valide 31j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 132j (07/12/2026)</t>
+          <t>Valide 131j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (09/10/2026)</t>
+          <t>Valide 72j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (30/11/2026)</t>
+          <t>Valide 124j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (09/10/2026)</t>
+          <t>Valide 72j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 125j (30/11/2026)</t>
+          <t>Valide 124j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (09/02/2027)</t>
+          <t>Valide 195j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>196j</t>
+          <t>195j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (20/11/2026)</t>
+          <t>Valide 114j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 196j (09/02/2027)</t>
+          <t>Valide 195j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>196j</t>
+          <t>195j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 115j (20/11/2026)</t>
+          <t>Valide 114j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 144j (19/12/2026)</t>
+          <t>Valide 143j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>144j</t>
+          <t>143j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 368j (31/07/2027)</t>
+          <t>Valide 367j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (19/12/2026)</t>
+          <t>Valide 143j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>144j</t>
+          <t>143j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 368j (31/07/2027)</t>
+          <t>Valide 367j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (13/10/2026)</t>
+          <t>Valide 76j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (10/10/2026)</t>
+          <t>Valide 73j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>28/07/2026 09:37</t>
+          <t>29/07/2026 09:40</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 30/07/2026 09:38
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (23/09/2026)</t>
+          <t>Valide 54j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 218j (05/03/2027)</t>
+          <t>Valide 217j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 193j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>193j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 373j (07/08/2027)</t>
+          <t>Valide 372j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (03/09/2026)</t>
+          <t>Valide 34j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (26/01/2027)</t>
+          <t>Valide 179j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (20/11/2026)</t>
+          <t>Valide 113j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 96j (02/11/2026)</t>
+          <t>Valide 95j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (09/02/2027)</t>
+          <t>Valide 194j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>195j</t>
+          <t>194j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 214j (28/02/2027)</t>
+          <t>Valide 213j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 193j (07/02/2027)</t>
+          <t>Valide 192j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>193j</t>
+          <t>192j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 358j (22/07/2027)</t>
+          <t>Valide 357j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (14/10/2026)</t>
+          <t>Valide 76j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,25 +1745,29 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (29/08/2026)</t>
+          <t>Expire dans 30j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (07/12/2026)</t>
+          <t>Valide 130j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr"/>
+          <t>30/07/2026 09:33</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="34">
       <c r="A26" s="3" t="inlineStr">
@@ -1811,25 +1815,29 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 31j (29/08/2026)</t>
+          <t>Expire dans 30j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 131j (07/12/2026)</t>
+          <t>Valide 130j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr"/>
+          <t>30/07/2026 09:33</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="8" t="inlineStr">
@@ -1957,22 +1965,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (09/10/2026)</t>
+          <t>Valide 71j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (30/11/2026)</t>
+          <t>Valide 123j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2015,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (09/10/2026)</t>
+          <t>Valide 71j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 124j (30/11/2026)</t>
+          <t>Valide 123j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2193,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (09/02/2027)</t>
+          <t>Valide 194j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>195j</t>
+          <t>194j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (20/11/2026)</t>
+          <t>Valide 113j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2255,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 195j (09/02/2027)</t>
+          <t>Valide 194j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>195j</t>
+          <t>194j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 114j (20/11/2026)</t>
+          <t>Valide 113j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2465,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 143j (19/12/2026)</t>
+          <t>Valide 142j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>143j</t>
+          <t>142j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 367j (31/07/2027)</t>
+          <t>Valide 366j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2519,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (19/12/2026)</t>
+          <t>Valide 142j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>143j</t>
+          <t>142j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 367j (31/07/2027)</t>
+          <t>Valide 366j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2733,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (13/10/2026)</t>
+          <t>Valide 75j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (10/10/2026)</t>
+          <t>Valide 72j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>29/07/2026 09:40</t>
+          <t>30/07/2026 09:33</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 31/07/2026 09:53
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (23/09/2026)</t>
+          <t>Valide 53j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 217j (05/03/2027)</t>
+          <t>Valide 216j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 191j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>191j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 372j (07/08/2027)</t>
+          <t>Valide 371j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (03/09/2026)</t>
+          <t>Valide 33j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (26/01/2027)</t>
+          <t>Valide 178j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (20/11/2026)</t>
+          <t>Valide 112j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>112j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 95j (02/11/2026)</t>
+          <t>Valide 94j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (09/02/2027)</t>
+          <t>Valide 193j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>194j</t>
+          <t>193j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 213j (28/02/2027)</t>
+          <t>Valide 212j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 192j (07/02/2027)</t>
+          <t>Valide 191j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>192j</t>
+          <t>191j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 357j (22/07/2027)</t>
+          <t>Valide 356j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (14/10/2026)</t>
+          <t>Valide 75j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,29 +1745,25 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (29/08/2026)</t>
+          <t>Expire dans 29j (29/08/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (07/12/2026)</t>
+          <t>Valide 129j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>31/07/2026 09:47</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1" s="34">
       <c r="A26" s="3" t="inlineStr">
@@ -1815,29 +1811,25 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 30j (29/08/2026)</t>
+          <t>Expire dans 29j (29/08/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 130j (07/12/2026)</t>
+          <t>Valide 129j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>31/07/2026 09:47</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="8" t="inlineStr">
@@ -1965,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (09/10/2026)</t>
+          <t>Valide 70j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (30/11/2026)</t>
+          <t>Valide 122j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2015,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (09/10/2026)</t>
+          <t>Valide 70j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 123j (30/11/2026)</t>
+          <t>Valide 122j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2193,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (09/02/2027)</t>
+          <t>Valide 193j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>194j</t>
+          <t>193j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (20/11/2026)</t>
+          <t>Valide 112j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2255,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 194j (09/02/2027)</t>
+          <t>Valide 193j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>194j</t>
+          <t>193j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 113j (20/11/2026)</t>
+          <t>Valide 112j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2465,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 142j (19/12/2026)</t>
+          <t>Valide 141j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>142j</t>
+          <t>141j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 366j (31/07/2027)</t>
+          <t>Valide 365j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2519,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (19/12/2026)</t>
+          <t>Valide 141j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>142j</t>
+          <t>141j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 366j (31/07/2027)</t>
+          <t>Valide 365j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2733,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (13/10/2026)</t>
+          <t>Valide 74j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (10/10/2026)</t>
+          <t>Valide 71j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>30/07/2026 09:33</t>
+          <t>31/07/2026 09:47</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 01/08/2026 09:15
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (23/09/2026)</t>
+          <t>Valide 52j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 216j (05/03/2027)</t>
+          <t>Valide 215j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 191j (07/02/2027)</t>
+          <t>Valide 190j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>191j</t>
+          <t>190j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 371j (07/08/2027)</t>
+          <t>Valide 370j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (03/09/2026)</t>
+          <t>Valide 32j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (26/01/2027)</t>
+          <t>Valide 177j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (20/11/2026)</t>
+          <t>Valide 111j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>112j</t>
+          <t>111j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 94j (02/11/2026)</t>
+          <t>Valide 93j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (09/02/2027)</t>
+          <t>Valide 192j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>193j</t>
+          <t>192j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 212j (28/02/2027)</t>
+          <t>Valide 211j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 191j (07/02/2027)</t>
+          <t>Valide 190j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>191j</t>
+          <t>190j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 356j (22/07/2027)</t>
+          <t>Valide 355j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (14/10/2026)</t>
+          <t>Valide 74j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (29/08/2026)</t>
+          <t>Valide 89j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (07/12/2026)</t>
+          <t>Valide 128j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 29j (29/08/2026)</t>
+          <t>Valide 89j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 129j (07/12/2026)</t>
+          <t>Valide 128j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (09/10/2026)</t>
+          <t>Valide 69j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (30/11/2026)</t>
+          <t>Valide 121j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (09/10/2026)</t>
+          <t>Valide 69j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 122j (30/11/2026)</t>
+          <t>Valide 121j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (09/02/2027)</t>
+          <t>Valide 192j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>193j</t>
+          <t>192j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (20/11/2026)</t>
+          <t>Valide 111j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 193j (09/02/2027)</t>
+          <t>Valide 192j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>193j</t>
+          <t>192j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 112j (20/11/2026)</t>
+          <t>Valide 111j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 141j (19/12/2026)</t>
+          <t>Valide 140j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>141j</t>
+          <t>140j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 365j (31/07/2027)</t>
+          <t>Valide 364j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (19/12/2026)</t>
+          <t>Valide 140j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>141j</t>
+          <t>140j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 365j (31/07/2027)</t>
+          <t>Valide 364j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (13/10/2026)</t>
+          <t>Valide 73j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (10/10/2026)</t>
+          <t>Valide 70j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>31/07/2026 09:47</t>
+          <t>01/08/2026 09:08</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 02/08/2026 09:16
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (23/09/2026)</t>
+          <t>Valide 51j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 215j (05/03/2027)</t>
+          <t>Valide 214j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 190j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>190j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 370j (07/08/2027)</t>
+          <t>Valide 369j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (03/09/2026)</t>
+          <t>Valide 31j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (26/01/2027)</t>
+          <t>Valide 176j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (20/11/2026)</t>
+          <t>Valide 110j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>111j</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 93j (02/11/2026)</t>
+          <t>Valide 92j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (09/02/2027)</t>
+          <t>Valide 191j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>192j</t>
+          <t>191j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 211j (28/02/2027)</t>
+          <t>Valide 210j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 190j (07/02/2027)</t>
+          <t>Valide 189j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>190j</t>
+          <t>189j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 355j (22/07/2027)</t>
+          <t>Valide 354j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (14/10/2026)</t>
+          <t>Valide 73j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (29/10/2026)</t>
+          <t>Valide 88j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (07/12/2026)</t>
+          <t>Valide 127j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (29/10/2026)</t>
+          <t>Valide 88j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 128j (07/12/2026)</t>
+          <t>Valide 127j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (09/10/2026)</t>
+          <t>Valide 68j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (30/11/2026)</t>
+          <t>Valide 120j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (09/10/2026)</t>
+          <t>Valide 68j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 121j (30/11/2026)</t>
+          <t>Valide 120j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (09/02/2027)</t>
+          <t>Valide 191j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>192j</t>
+          <t>191j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (20/11/2026)</t>
+          <t>Valide 110j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 192j (09/02/2027)</t>
+          <t>Valide 191j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>192j</t>
+          <t>191j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 111j (20/11/2026)</t>
+          <t>Valide 110j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 140j (19/12/2026)</t>
+          <t>Valide 139j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>140j</t>
+          <t>139j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 364j (31/07/2027)</t>
+          <t>Valide 363j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (19/12/2026)</t>
+          <t>Valide 139j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>140j</t>
+          <t>139j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 364j (31/07/2027)</t>
+          <t>Valide 363j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (13/10/2026)</t>
+          <t>Valide 72j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (10/10/2026)</t>
+          <t>Valide 69j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>01/08/2026 09:08</t>
+          <t>02/08/2026 09:11</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 03/08/2026 10:51
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (23/09/2026)</t>
+          <t>Valide 50j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 214j (05/03/2027)</t>
+          <t>Valide 213j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 369j (07/08/2027)</t>
+          <t>Valide 368j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,25 +1046,29 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (03/09/2026)</t>
+          <t>Expire dans 30j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (26/01/2027)</t>
+          <t>Valide 175j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr"/>
+          <t>03/08/2026 10:45</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="9" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A9" s="3" t="inlineStr">
@@ -1152,22 +1156,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (20/11/2026)</t>
+          <t>Valide 109j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>109j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 92j (02/11/2026)</t>
+          <t>Valide 91j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (09/02/2027)</t>
+          <t>Valide 190j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>191j</t>
+          <t>190j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 210j (28/02/2027)</t>
+          <t>Valide 209j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 189j (07/02/2027)</t>
+          <t>Valide 188j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>189j</t>
+          <t>188j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 354j (22/07/2027)</t>
+          <t>Valide 353j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (14/10/2026)</t>
+          <t>Valide 72j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (29/10/2026)</t>
+          <t>Valide 87j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (07/12/2026)</t>
+          <t>Valide 126j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 88j (29/10/2026)</t>
+          <t>Valide 87j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 127j (07/12/2026)</t>
+          <t>Valide 126j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (09/10/2026)</t>
+          <t>Valide 67j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (30/11/2026)</t>
+          <t>Valide 119j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (09/10/2026)</t>
+          <t>Valide 67j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 120j (30/11/2026)</t>
+          <t>Valide 119j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (09/02/2027)</t>
+          <t>Valide 190j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>191j</t>
+          <t>190j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (20/11/2026)</t>
+          <t>Valide 109j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 191j (09/02/2027)</t>
+          <t>Valide 190j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>191j</t>
+          <t>190j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 110j (20/11/2026)</t>
+          <t>Valide 109j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 139j (19/12/2026)</t>
+          <t>Valide 138j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>139j</t>
+          <t>138j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 363j (31/07/2027)</t>
+          <t>Valide 362j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (19/12/2026)</t>
+          <t>Valide 138j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>139j</t>
+          <t>138j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 363j (31/07/2027)</t>
+          <t>Valide 362j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (13/10/2026)</t>
+          <t>Valide 71j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (10/10/2026)</t>
+          <t>Valide 68j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>02/08/2026 09:11</t>
+          <t>03/08/2026 10:45</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 04/08/2026 09:45
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (23/09/2026)</t>
+          <t>Valide 49j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 213j (05/03/2027)</t>
+          <t>Valide 212j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 368j (07/08/2027)</t>
+          <t>Valide 367j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,29 +1046,25 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (03/09/2026)</t>
+          <t>Expire dans 29j (03/09/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (26/01/2027)</t>
+          <t>Valide 174j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>04/08/2026 09:39</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A9" s="3" t="inlineStr">
@@ -1156,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (20/11/2026)</t>
+          <t>Valide 108j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>109j</t>
+          <t>108j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 91j (02/11/2026)</t>
+          <t>Valide 90j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1262,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (09/02/2027)</t>
+          <t>Valide 189j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>190j</t>
+          <t>189j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 209j (28/02/2027)</t>
+          <t>Valide 208j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 188j (07/02/2027)</t>
+          <t>Valide 187j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>188j</t>
+          <t>187j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 353j (22/07/2027)</t>
+          <t>Valide 352j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (14/10/2026)</t>
+          <t>Valide 71j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (29/10/2026)</t>
+          <t>Valide 86j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (07/12/2026)</t>
+          <t>Valide 125j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (29/10/2026)</t>
+          <t>Valide 86j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 126j (07/12/2026)</t>
+          <t>Valide 125j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (09/10/2026)</t>
+          <t>Valide 66j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (30/11/2026)</t>
+          <t>Valide 118j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (09/10/2026)</t>
+          <t>Valide 66j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 119j (30/11/2026)</t>
+          <t>Valide 118j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (09/02/2027)</t>
+          <t>Valide 189j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>190j</t>
+          <t>189j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (20/11/2026)</t>
+          <t>Valide 108j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 190j (09/02/2027)</t>
+          <t>Valide 189j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>190j</t>
+          <t>189j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 109j (20/11/2026)</t>
+          <t>Valide 108j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 138j (19/12/2026)</t>
+          <t>Valide 137j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>138j</t>
+          <t>137j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 362j (31/07/2027)</t>
+          <t>Valide 361j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (19/12/2026)</t>
+          <t>Valide 137j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>138j</t>
+          <t>137j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 362j (31/07/2027)</t>
+          <t>Valide 361j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (13/10/2026)</t>
+          <t>Valide 70j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (10/10/2026)</t>
+          <t>Valide 67j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>03/08/2026 10:45</t>
+          <t>04/08/2026 09:39</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 05/08/2026 09:43
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (23/09/2026)</t>
+          <t>Valide 48j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 212j (05/03/2027)</t>
+          <t>Valide 211j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 367j (07/08/2027)</t>
+          <t>Valide 366j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (03/09/2026)</t>
+          <t>Valide 89j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (26/01/2027)</t>
+          <t>Valide 173j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (20/11/2026)</t>
+          <t>Valide 107j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>108j</t>
+          <t>107j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 90j (02/11/2026)</t>
+          <t>Valide 89j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (09/02/2027)</t>
+          <t>Valide 188j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>189j</t>
+          <t>188j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 208j (28/02/2027)</t>
+          <t>Valide 207j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 187j (07/02/2027)</t>
+          <t>Valide 186j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>187j</t>
+          <t>186j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 352j (22/07/2027)</t>
+          <t>Valide 351j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (14/10/2026)</t>
+          <t>Valide 70j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (29/10/2026)</t>
+          <t>Valide 85j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (07/12/2026)</t>
+          <t>Valide 124j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (29/10/2026)</t>
+          <t>Valide 85j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 125j (07/12/2026)</t>
+          <t>Valide 124j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (09/10/2026)</t>
+          <t>Valide 65j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (30/11/2026)</t>
+          <t>Valide 117j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (09/10/2026)</t>
+          <t>Valide 65j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 118j (30/11/2026)</t>
+          <t>Valide 117j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (09/02/2027)</t>
+          <t>Valide 188j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>189j</t>
+          <t>188j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (20/11/2026)</t>
+          <t>Valide 107j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 189j (09/02/2027)</t>
+          <t>Valide 188j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>189j</t>
+          <t>188j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 108j (20/11/2026)</t>
+          <t>Valide 107j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 137j (19/12/2026)</t>
+          <t>Valide 136j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>137j</t>
+          <t>136j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 361j (31/07/2027)</t>
+          <t>Valide 360j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (19/12/2026)</t>
+          <t>Valide 136j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>137j</t>
+          <t>136j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 361j (31/07/2027)</t>
+          <t>Valide 360j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (13/10/2026)</t>
+          <t>Valide 69j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (10/10/2026)</t>
+          <t>Valide 66j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>04/08/2026 09:39</t>
+          <t>05/08/2026 09:38</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 06/08/2026 09:46
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (23/09/2026)</t>
+          <t>Valide 47j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 211j (05/03/2027)</t>
+          <t>Valide 210j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 366j (07/08/2027)</t>
+          <t>Valide 365j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (02/11/2026)</t>
+          <t>Valide 88j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (26/01/2027)</t>
+          <t>Valide 172j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (20/11/2026)</t>
+          <t>Valide 106j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>107j</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (02/11/2026)</t>
+          <t>Valide 88j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (09/02/2027)</t>
+          <t>Valide 187j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>188j</t>
+          <t>187j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 207j (28/02/2027)</t>
+          <t>Valide 206j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 186j (07/02/2027)</t>
+          <t>Valide 185j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>186j</t>
+          <t>185j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 351j (22/07/2027)</t>
+          <t>Valide 350j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (14/10/2026)</t>
+          <t>Valide 69j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (29/10/2026)</t>
+          <t>Valide 84j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (07/12/2026)</t>
+          <t>Valide 123j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (29/10/2026)</t>
+          <t>Valide 84j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 124j (07/12/2026)</t>
+          <t>Valide 123j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (09/10/2026)</t>
+          <t>Valide 64j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (30/11/2026)</t>
+          <t>Valide 116j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 65j (09/10/2026)</t>
+          <t>Valide 64j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 117j (30/11/2026)</t>
+          <t>Valide 116j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (09/02/2027)</t>
+          <t>Valide 187j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>188j</t>
+          <t>187j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (20/11/2026)</t>
+          <t>Valide 106j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 188j (09/02/2027)</t>
+          <t>Valide 187j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>188j</t>
+          <t>187j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 107j (20/11/2026)</t>
+          <t>Valide 106j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 136j (19/12/2026)</t>
+          <t>Valide 135j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>136j</t>
+          <t>135j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 360j (31/07/2027)</t>
+          <t>Valide 359j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (19/12/2026)</t>
+          <t>Valide 135j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>136j</t>
+          <t>135j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 360j (31/07/2027)</t>
+          <t>Valide 359j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (13/10/2026)</t>
+          <t>Valide 68j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (10/10/2026)</t>
+          <t>Valide 65j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>05/08/2026 09:38</t>
+          <t>06/08/2026 09:41</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 07/08/2026 08:21
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (23/09/2026)</t>
+          <t>Valide 46j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 210j (05/03/2027)</t>
+          <t>Valide 209j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 365j (07/08/2027)</t>
+          <t>Valide 364j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (02/11/2026)</t>
+          <t>Valide 87j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (26/01/2027)</t>
+          <t>Valide 171j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (20/11/2026)</t>
+          <t>Valide 105j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (02/11/2026)</t>
+          <t>Valide 87j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (09/02/2027)</t>
+          <t>Valide 186j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>187j</t>
+          <t>186j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 206j (28/02/2027)</t>
+          <t>Valide 205j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 185j (07/02/2027)</t>
+          <t>Valide 184j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>185j</t>
+          <t>184j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 350j (22/07/2027)</t>
+          <t>Valide 349j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (14/10/2026)</t>
+          <t>Valide 68j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (29/10/2026)</t>
+          <t>Valide 83j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (07/12/2026)</t>
+          <t>Valide 122j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (29/10/2026)</t>
+          <t>Valide 83j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 123j (07/12/2026)</t>
+          <t>Valide 122j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (09/10/2026)</t>
+          <t>Valide 63j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (30/11/2026)</t>
+          <t>Valide 115j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (09/10/2026)</t>
+          <t>Valide 63j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 116j (30/11/2026)</t>
+          <t>Valide 115j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (09/02/2027)</t>
+          <t>Valide 186j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>187j</t>
+          <t>186j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (20/11/2026)</t>
+          <t>Valide 105j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 187j (09/02/2027)</t>
+          <t>Valide 186j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>187j</t>
+          <t>186j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 106j (20/11/2026)</t>
+          <t>Valide 105j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 135j (19/12/2026)</t>
+          <t>Valide 134j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>135j</t>
+          <t>134j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 359j (31/07/2027)</t>
+          <t>Valide 358j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 135j (19/12/2026)</t>
+          <t>Valide 134j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>135j</t>
+          <t>134j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 359j (31/07/2027)</t>
+          <t>Valide 358j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (13/10/2026)</t>
+          <t>Valide 67j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (10/10/2026)</t>
+          <t>Valide 64j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>06/08/2026 09:41</t>
+          <t>07/08/2026 08:16</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 08/08/2026 07:56
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (23/09/2026)</t>
+          <t>Valide 45j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 209j (05/03/2027)</t>
+          <t>Valide 208j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,12 +976,12 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 183j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>183j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (02/11/2026)</t>
+          <t>Valide 86j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (26/01/2027)</t>
+          <t>Valide 170j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (20/11/2026)</t>
+          <t>Valide 104j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (02/11/2026)</t>
+          <t>Valide 86j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 186j (09/02/2027)</t>
+          <t>Valide 185j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>186j</t>
+          <t>185j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 205j (28/02/2027)</t>
+          <t>Valide 204j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 184j (07/02/2027)</t>
+          <t>Valide 183j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>184j</t>
+          <t>183j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 349j (22/07/2027)</t>
+          <t>Valide 348j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (14/10/2026)</t>
+          <t>Valide 67j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (29/10/2026)</t>
+          <t>Valide 82j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (07/12/2026)</t>
+          <t>Valide 121j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 83j (29/10/2026)</t>
+          <t>Valide 82j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 122j (07/12/2026)</t>
+          <t>Valide 121j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (09/10/2026)</t>
+          <t>Valide 62j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (30/11/2026)</t>
+          <t>Valide 114j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (09/10/2026)</t>
+          <t>Valide 62j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 115j (30/11/2026)</t>
+          <t>Valide 114j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 186j (09/02/2027)</t>
+          <t>Valide 185j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>186j</t>
+          <t>185j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (20/11/2026)</t>
+          <t>Valide 104j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 186j (09/02/2027)</t>
+          <t>Valide 185j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>186j</t>
+          <t>185j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 105j (20/11/2026)</t>
+          <t>Valide 104j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 134j (19/12/2026)</t>
+          <t>Valide 133j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>134j</t>
+          <t>133j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 358j (31/07/2027)</t>
+          <t>Valide 357j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 134j (19/12/2026)</t>
+          <t>Valide 133j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>134j</t>
+          <t>133j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 358j (31/07/2027)</t>
+          <t>Valide 357j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (13/10/2026)</t>
+          <t>Valide 66j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (10/10/2026)</t>
+          <t>Valide 63j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>07/08/2026 08:16</t>
+          <t>08/08/2026 07:51</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 09/08/2026 07:59
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (23/09/2026)</t>
+          <t>Valide 44j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 208j (05/03/2027)</t>
+          <t>Valide 207j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 183j (07/02/2027)</t>
+          <t>Valide 182j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>183j</t>
+          <t>182j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 364j (07/08/2027)</t>
+          <t>Valide 363j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (02/11/2026)</t>
+          <t>Valide 85j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (26/01/2027)</t>
+          <t>Valide 169j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (20/11/2026)</t>
+          <t>Valide 103j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (02/11/2026)</t>
+          <t>Valide 85j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (09/02/2027)</t>
+          <t>Valide 184j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>185j</t>
+          <t>184j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 204j (28/02/2027)</t>
+          <t>Valide 203j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 183j (07/02/2027)</t>
+          <t>Valide 182j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>183j</t>
+          <t>182j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 348j (22/07/2027)</t>
+          <t>Valide 347j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (14/10/2026)</t>
+          <t>Valide 66j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (29/10/2026)</t>
+          <t>Valide 81j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (07/12/2026)</t>
+          <t>Valide 120j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (29/10/2026)</t>
+          <t>Valide 81j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 121j (07/12/2026)</t>
+          <t>Valide 120j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (09/10/2026)</t>
+          <t>Valide 61j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (30/11/2026)</t>
+          <t>Valide 113j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (09/10/2026)</t>
+          <t>Valide 61j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 114j (30/11/2026)</t>
+          <t>Valide 113j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (09/02/2027)</t>
+          <t>Valide 184j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>185j</t>
+          <t>184j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (20/11/2026)</t>
+          <t>Valide 103j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 185j (09/02/2027)</t>
+          <t>Valide 184j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>185j</t>
+          <t>184j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 104j (20/11/2026)</t>
+          <t>Valide 103j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 133j (19/12/2026)</t>
+          <t>Valide 132j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>133j</t>
+          <t>132j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 357j (31/07/2027)</t>
+          <t>Valide 356j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 133j (19/12/2026)</t>
+          <t>Valide 132j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>133j</t>
+          <t>132j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 357j (31/07/2027)</t>
+          <t>Valide 356j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (13/10/2026)</t>
+          <t>Valide 65j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (10/10/2026)</t>
+          <t>Valide 62j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>08/08/2026 07:51</t>
+          <t>09/08/2026 07:54</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 10/08/2026 08:45
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (23/09/2026)</t>
+          <t>Valide 43j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 207j (05/03/2027)</t>
+          <t>Valide 206j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 182j (07/02/2027)</t>
+          <t>Valide 181j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>182j</t>
+          <t>181j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 363j (07/08/2027)</t>
+          <t>Valide 361j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (02/11/2026)</t>
+          <t>Valide 84j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (26/01/2027)</t>
+          <t>Valide 168j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (20/11/2026)</t>
+          <t>Valide 102j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (02/11/2026)</t>
+          <t>Valide 84j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 184j (09/02/2027)</t>
+          <t>Valide 183j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>184j</t>
+          <t>183j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 203j (28/02/2027)</t>
+          <t>Valide 202j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 182j (07/02/2027)</t>
+          <t>Valide 181j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>182j</t>
+          <t>181j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 347j (22/07/2027)</t>
+          <t>Valide 346j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (14/10/2026)</t>
+          <t>Valide 65j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (29/10/2026)</t>
+          <t>Valide 80j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (07/12/2026)</t>
+          <t>Valide 119j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 81j (29/10/2026)</t>
+          <t>Valide 80j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 120j (07/12/2026)</t>
+          <t>Valide 119j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (09/10/2026)</t>
+          <t>Valide 60j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (30/11/2026)</t>
+          <t>Valide 112j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (09/10/2026)</t>
+          <t>Valide 60j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 113j (30/11/2026)</t>
+          <t>Valide 112j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 184j (09/02/2027)</t>
+          <t>Valide 183j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>184j</t>
+          <t>183j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (20/11/2026)</t>
+          <t>Valide 102j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 184j (09/02/2027)</t>
+          <t>Valide 183j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>184j</t>
+          <t>183j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 103j (20/11/2026)</t>
+          <t>Valide 102j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 132j (19/12/2026)</t>
+          <t>Valide 131j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>132j</t>
+          <t>131j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 356j (31/07/2027)</t>
+          <t>Valide 355j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 132j (19/12/2026)</t>
+          <t>Valide 131j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>132j</t>
+          <t>131j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 356j (31/07/2027)</t>
+          <t>Valide 355j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (13/10/2026)</t>
+          <t>Valide 64j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (10/10/2026)</t>
+          <t>Valide 61j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>09/08/2026 07:54</t>
+          <t>10/08/2026 08:41</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 11/08/2026 08:16
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (23/09/2026)</t>
+          <t>Valide 42j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 206j (05/03/2027)</t>
+          <t>Valide 205j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 181j (07/02/2027)</t>
+          <t>Valide 180j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>181j</t>
+          <t>180j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 361j (07/08/2027)</t>
+          <t>Valide 360j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (02/11/2026)</t>
+          <t>Valide 83j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (26/01/2027)</t>
+          <t>Valide 167j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (20/11/2026)</t>
+          <t>Valide 101j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (02/11/2026)</t>
+          <t>Valide 83j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (09/02/2027)</t>
+          <t>Valide 182j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>183j</t>
+          <t>182j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 202j (28/02/2027)</t>
+          <t>Valide 201j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 181j (07/02/2027)</t>
+          <t>Valide 180j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>181j</t>
+          <t>180j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 346j (22/07/2027)</t>
+          <t>Valide 345j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (14/10/2026)</t>
+          <t>Valide 64j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (29/10/2026)</t>
+          <t>Valide 79j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (07/12/2026)</t>
+          <t>Valide 118j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 80j (29/10/2026)</t>
+          <t>Valide 79j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 119j (07/12/2026)</t>
+          <t>Valide 118j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (09/10/2026)</t>
+          <t>Valide 59j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (30/11/2026)</t>
+          <t>Valide 111j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 60j (09/10/2026)</t>
+          <t>Valide 59j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 112j (30/11/2026)</t>
+          <t>Valide 111j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (09/02/2027)</t>
+          <t>Valide 182j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>183j</t>
+          <t>182j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (20/11/2026)</t>
+          <t>Valide 101j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 183j (09/02/2027)</t>
+          <t>Valide 182j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>183j</t>
+          <t>182j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 102j (20/11/2026)</t>
+          <t>Valide 101j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 131j (19/12/2026)</t>
+          <t>Valide 130j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>131j</t>
+          <t>130j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 355j (31/07/2027)</t>
+          <t>Valide 354j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 131j (19/12/2026)</t>
+          <t>Valide 130j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>131j</t>
+          <t>130j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 355j (31/07/2027)</t>
+          <t>Valide 354j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (13/10/2026)</t>
+          <t>Valide 63j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (10/10/2026)</t>
+          <t>Valide 60j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>10/08/2026 08:41</t>
+          <t>11/08/2026 08:10</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 12/08/2026 08:27
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (23/09/2026)</t>
+          <t>Valide 41j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 205j (05/03/2027)</t>
+          <t>Valide 204j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 180j (07/02/2027)</t>
+          <t>Valide 179j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>179j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 360j (07/08/2027)</t>
+          <t>Valide 359j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (02/11/2026)</t>
+          <t>Valide 82j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (26/01/2027)</t>
+          <t>Valide 166j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 101j (20/11/2026)</t>
+          <t>Valide 100j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>101j</t>
+          <t>100j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (02/11/2026)</t>
+          <t>Valide 82j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (09/02/2027)</t>
+          <t>Valide 181j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>182j</t>
+          <t>181j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 201j (28/02/2027)</t>
+          <t>Valide 200j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 180j (07/02/2027)</t>
+          <t>Valide 179j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>179j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 345j (22/07/2027)</t>
+          <t>Valide 344j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (14/10/2026)</t>
+          <t>Valide 63j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (29/10/2026)</t>
+          <t>Valide 78j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (07/12/2026)</t>
+          <t>Valide 117j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (29/10/2026)</t>
+          <t>Valide 78j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 118j (07/12/2026)</t>
+          <t>Valide 117j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (09/10/2026)</t>
+          <t>Valide 58j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (30/11/2026)</t>
+          <t>Valide 110j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 59j (09/10/2026)</t>
+          <t>Valide 58j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 111j (30/11/2026)</t>
+          <t>Valide 110j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (09/02/2027)</t>
+          <t>Valide 181j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>182j</t>
+          <t>181j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 101j (20/11/2026)</t>
+          <t>Valide 100j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 182j (09/02/2027)</t>
+          <t>Valide 181j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>182j</t>
+          <t>181j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 101j (20/11/2026)</t>
+          <t>Valide 100j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 130j (19/12/2026)</t>
+          <t>Valide 129j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>130j</t>
+          <t>129j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 354j (31/07/2027)</t>
+          <t>Valide 353j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 130j (19/12/2026)</t>
+          <t>Valide 129j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>130j</t>
+          <t>129j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 354j (31/07/2027)</t>
+          <t>Valide 353j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (13/10/2026)</t>
+          <t>Valide 62j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (10/10/2026)</t>
+          <t>Valide 59j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>11/08/2026 08:10</t>
+          <t>12/08/2026 08:20</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 13/08/2026 08:30
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (23/09/2026)</t>
+          <t>Valide 40j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 204j (05/03/2027)</t>
+          <t>Valide 203j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 179j (07/02/2027)</t>
+          <t>Valide 178j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>179j</t>
+          <t>178j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 359j (07/08/2027)</t>
+          <t>Valide 358j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (02/11/2026)</t>
+          <t>Valide 81j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (26/01/2027)</t>
+          <t>Valide 165j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 100j (20/11/2026)</t>
+          <t>Valide 99j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>100j</t>
+          <t>99j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (02/11/2026)</t>
+          <t>Date inconnue</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (09/02/2027)</t>
+          <t>Valide 180j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>181j</t>
+          <t>180j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 200j (28/02/2027)</t>
+          <t>Valide 199j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 179j (07/02/2027)</t>
+          <t>Valide 178j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>179j</t>
+          <t>178j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 344j (22/07/2027)</t>
+          <t>Whois command returned no output</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (14/10/2026)</t>
+          <t>Valide 62j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (29/10/2026)</t>
+          <t>Valide 77j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (07/12/2026)</t>
+          <t>Valide 116j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (29/10/2026)</t>
+          <t>Valide 77j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 117j (07/12/2026)</t>
+          <t>Valide 116j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (09/10/2026)</t>
+          <t>Valide 57j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (30/11/2026)</t>
+          <t>Valide 109j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 58j (09/10/2026)</t>
+          <t>Valide 57j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 110j (30/11/2026)</t>
+          <t>Valide 109j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (09/02/2027)</t>
+          <t>Valide 180j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>181j</t>
+          <t>180j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 100j (20/11/2026)</t>
+          <t>Date inconnue</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 181j (09/02/2027)</t>
+          <t>Valide 180j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>181j</t>
+          <t>180j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 100j (20/11/2026)</t>
+          <t>Date inconnue</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 129j (19/12/2026)</t>
+          <t>Valide 128j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>129j</t>
+          <t>128j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 353j (31/07/2027)</t>
+          <t>Valide 352j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 129j (19/12/2026)</t>
+          <t>Valide 128j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>129j</t>
+          <t>128j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 353j (31/07/2027)</t>
+          <t>Valide 352j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (13/10/2026)</t>
+          <t>Valide 61j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (10/10/2026)</t>
+          <t>Date inconnue</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>12/08/2026 08:20</t>
+          <t>13/08/2026 08:23</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 14/08/2026 08:24
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (23/09/2026)</t>
+          <t>Valide 39j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 203j (05/03/2027)</t>
+          <t>Valide 202j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 178j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>178j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 358j (07/08/2027)</t>
+          <t>Valide 357j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (02/11/2026)</t>
+          <t>Valide 80j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (26/01/2027)</t>
+          <t>Valide 164j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 99j (20/11/2026)</t>
+          <t>Valide 98j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>99j</t>
+          <t>98j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Date inconnue</t>
+          <t>Valide 80j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (09/02/2027)</t>
+          <t>Valide 179j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>179j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 199j (28/02/2027)</t>
+          <t>Valide 198j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 178j (07/02/2027)</t>
+          <t>Valide 177j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>178j</t>
+          <t>177j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Whois command returned no output</t>
+          <t>Valide 342j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1645,17 +1645,17 @@
       </c>
       <c r="K23" s="9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (14/10/2026)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,10 +1665,14 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr"/>
+          <t>14/08/2026 08:18</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
       <c r="R23" t="inlineStr">
         <is>
           <t>x</t>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (29/10/2026)</t>
+          <t>Valide 76j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (07/12/2026)</t>
+          <t>Valide 115j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (29/10/2026)</t>
+          <t>Valide 76j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 116j (07/12/2026)</t>
+          <t>Valide 115j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (09/10/2026)</t>
+          <t>Valide 56j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (30/11/2026)</t>
+          <t>Valide 108j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 57j (09/10/2026)</t>
+          <t>Valide 56j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 109j (30/11/2026)</t>
+          <t>Valide 108j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (09/02/2027)</t>
+          <t>Valide 179j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>179j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Date inconnue</t>
+          <t>Valide 98j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 180j (09/02/2027)</t>
+          <t>Valide 179j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>180j</t>
+          <t>179j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Date inconnue</t>
+          <t>Valide 98j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 128j (19/12/2026)</t>
+          <t>Valide 127j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>128j</t>
+          <t>127j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 352j (31/07/2027)</t>
+          <t>Valide 351j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 128j (19/12/2026)</t>
+          <t>Valide 127j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>128j</t>
+          <t>127j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 352j (31/07/2027)</t>
+          <t>Valide 351j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (13/10/2026)</t>
+          <t>Valide 60j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Date inconnue</t>
+          <t>Valide 57j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>13/08/2026 08:23</t>
+          <t>14/08/2026 08:18</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 15/08/2026 07:38
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (23/09/2026)</t>
+          <t>Valide 38j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 202j (05/03/2027)</t>
+          <t>Valide 201j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -991,7 +991,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (02/11/2026)</t>
+          <t>Valide 79j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (26/01/2027)</t>
+          <t>Valide 163j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 98j (20/11/2026)</t>
+          <t>Valide 97j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>98j</t>
+          <t>97j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (02/11/2026)</t>
+          <t>Valide 79j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (09/02/2027)</t>
+          <t>Valide 178j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>179j</t>
+          <t>178j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 198j (28/02/2027)</t>
+          <t>Valide 197j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 177j (07/02/2027)</t>
+          <t>Valide 176j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>177j</t>
+          <t>176j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 342j (22/07/2027)</t>
+          <t>Valide 341j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1645,17 +1645,17 @@
       </c>
       <c r="K23" s="9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 60j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,14 +1665,10 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>15/08/2026 07:33</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
       <c r="R23" t="inlineStr">
         <is>
           <t>x</t>
@@ -1749,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (29/10/2026)</t>
+          <t>Valide 75j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (07/12/2026)</t>
+          <t>Valide 114j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (29/10/2026)</t>
+          <t>Valide 75j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 115j (07/12/2026)</t>
+          <t>Valide 114j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (09/10/2026)</t>
+          <t>Valide 55j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (30/11/2026)</t>
+          <t>Valide 107j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 56j (09/10/2026)</t>
+          <t>Valide 55j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 108j (30/11/2026)</t>
+          <t>Valide 107j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (09/02/2027)</t>
+          <t>Valide 178j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>179j</t>
+          <t>178j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 98j (20/11/2026)</t>
+          <t>Valide 97j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 179j (09/02/2027)</t>
+          <t>Valide 178j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>179j</t>
+          <t>178j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 98j (20/11/2026)</t>
+          <t>Valide 97j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 127j (19/12/2026)</t>
+          <t>Valide 126j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>127j</t>
+          <t>126j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 351j (31/07/2027)</t>
+          <t>Valide 350j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 127j (19/12/2026)</t>
+          <t>Valide 126j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>127j</t>
+          <t>126j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 351j (31/07/2027)</t>
+          <t>Valide 350j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (13/10/2026)</t>
+          <t>Valide 59j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (10/10/2026)</t>
+          <t>Valide 56j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>14/08/2026 08:18</t>
+          <t>15/08/2026 07:33</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 16/08/2026 07:38
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (23/09/2026)</t>
+          <t>Valide 37j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 201j (05/03/2027)</t>
+          <t>Valide 200j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 175j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>175j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 357j (07/08/2027)</t>
+          <t>Valide 356j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (02/11/2026)</t>
+          <t>Valide 78j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (26/01/2027)</t>
+          <t>Valide 162j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 97j (20/11/2026)</t>
+          <t>Valide 96j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>97j</t>
+          <t>96j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (02/11/2026)</t>
+          <t>Valide 78j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (09/02/2027)</t>
+          <t>Valide 177j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>178j</t>
+          <t>177j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (28/02/2027)</t>
+          <t>Valide 196j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 176j (07/02/2027)</t>
+          <t>Valide 175j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>176j</t>
+          <t>175j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 341j (22/07/2027)</t>
+          <t>Valide 340j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (14/10/2026)</t>
+          <t>Valide 59j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (29/10/2026)</t>
+          <t>Valide 74j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (07/12/2026)</t>
+          <t>Valide 113j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (29/10/2026)</t>
+          <t>Valide 74j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 114j (07/12/2026)</t>
+          <t>Valide 113j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (09/10/2026)</t>
+          <t>Valide 54j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (30/11/2026)</t>
+          <t>Valide 106j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 55j (09/10/2026)</t>
+          <t>Valide 54j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 107j (30/11/2026)</t>
+          <t>Valide 106j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (09/02/2027)</t>
+          <t>Valide 177j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>178j</t>
+          <t>177j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 97j (20/11/2026)</t>
+          <t>Valide 96j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 178j (09/02/2027)</t>
+          <t>Valide 177j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>178j</t>
+          <t>177j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 97j (20/11/2026)</t>
+          <t>Valide 96j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 126j (19/12/2026)</t>
+          <t>Valide 125j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>126j</t>
+          <t>125j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 350j (31/07/2027)</t>
+          <t>Valide 349j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 126j (19/12/2026)</t>
+          <t>Valide 125j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>126j</t>
+          <t>125j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 350j (31/07/2027)</t>
+          <t>Valide 349j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (13/10/2026)</t>
+          <t>Valide 58j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (10/10/2026)</t>
+          <t>Valide 55j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>15/08/2026 07:33</t>
+          <t>16/08/2026 07:33</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 17/08/2026 07:59
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (23/09/2026)</t>
+          <t>Valide 36j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 200j (05/03/2027)</t>
+          <t>Valide 199j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 175j (07/02/2027)</t>
+          <t>Valide 174j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>174j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 356j (07/08/2027)</t>
+          <t>Valide 355j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (02/11/2026)</t>
+          <t>Valide 77j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (26/01/2027)</t>
+          <t>Valide 161j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 96j (20/11/2026)</t>
+          <t>Valide 95j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>96j</t>
+          <t>95j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (02/11/2026)</t>
+          <t>Valide 77j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (09/02/2027)</t>
+          <t>Valide 176j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>177j</t>
+          <t>176j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (28/02/2027)</t>
+          <t>Valide 195j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 175j (07/02/2027)</t>
+          <t>Valide 174j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>174j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 340j (22/07/2027)</t>
+          <t>Valide 339j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (14/10/2026)</t>
+          <t>Valide 58j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (29/10/2026)</t>
+          <t>Valide 73j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (07/12/2026)</t>
+          <t>Valide 112j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 74j (29/10/2026)</t>
+          <t>Valide 73j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 113j (07/12/2026)</t>
+          <t>Valide 112j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (09/10/2026)</t>
+          <t>Valide 53j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (30/11/2026)</t>
+          <t>Valide 105j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (09/10/2026)</t>
+          <t>Valide 53j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 106j (30/11/2026)</t>
+          <t>Valide 105j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (09/02/2027)</t>
+          <t>Valide 176j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>177j</t>
+          <t>176j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 96j (20/11/2026)</t>
+          <t>Valide 95j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 177j (09/02/2027)</t>
+          <t>Valide 176j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>177j</t>
+          <t>176j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 96j (20/11/2026)</t>
+          <t>Valide 95j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 125j (19/12/2026)</t>
+          <t>Valide 124j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>125j</t>
+          <t>124j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 349j (31/07/2027)</t>
+          <t>Valide 348j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 125j (19/12/2026)</t>
+          <t>Valide 124j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>125j</t>
+          <t>124j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 349j (31/07/2027)</t>
+          <t>Valide 348j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (13/10/2026)</t>
+          <t>Valide 57j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (10/10/2026)</t>
+          <t>Valide 54j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>16/08/2026 07:33</t>
+          <t>17/08/2026 07:54</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 18/08/2026 07:45
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (23/09/2026)</t>
+          <t>Valide 35j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 199j (05/03/2027)</t>
+          <t>Valide 198j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 174j (07/02/2027)</t>
+          <t>Valide 173j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>174j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 355j (07/08/2027)</t>
+          <t>Valide 354j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (02/11/2026)</t>
+          <t>Valide 76j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (26/01/2027)</t>
+          <t>Valide 160j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 95j (20/11/2026)</t>
+          <t>Valide 94j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>95j</t>
+          <t>94j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (02/11/2026)</t>
+          <t>Valide 76j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (09/02/2027)</t>
+          <t>Valide 175j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>176j</t>
+          <t>175j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (28/02/2027)</t>
+          <t>Valide 194j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 174j (07/02/2027)</t>
+          <t>Valide 173j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>174j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 339j (22/07/2027)</t>
+          <t>Valide 338j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (14/10/2026)</t>
+          <t>Valide 57j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (29/10/2026)</t>
+          <t>Valide 72j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (07/12/2026)</t>
+          <t>Valide 111j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (29/10/2026)</t>
+          <t>Valide 72j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 112j (07/12/2026)</t>
+          <t>Valide 111j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (09/10/2026)</t>
+          <t>Valide 52j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (30/11/2026)</t>
+          <t>Valide 104j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 53j (09/10/2026)</t>
+          <t>Valide 52j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 105j (30/11/2026)</t>
+          <t>Valide 104j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (09/02/2027)</t>
+          <t>Valide 175j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>176j</t>
+          <t>175j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 95j (20/11/2026)</t>
+          <t>Valide 94j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 176j (09/02/2027)</t>
+          <t>Valide 175j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>176j</t>
+          <t>175j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 95j (20/11/2026)</t>
+          <t>Valide 94j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 124j (19/12/2026)</t>
+          <t>Valide 123j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>124j</t>
+          <t>123j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 348j (31/07/2027)</t>
+          <t>Valide 347j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 124j (19/12/2026)</t>
+          <t>Valide 123j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>124j</t>
+          <t>123j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 348j (31/07/2027)</t>
+          <t>Valide 347j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (13/10/2026)</t>
+          <t>Valide 56j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (10/10/2026)</t>
+          <t>Valide 53j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>17/08/2026 07:54</t>
+          <t>18/08/2026 07:40</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 19/08/2026 07:48
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (23/09/2026)</t>
+          <t>Valide 34j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 198j (05/03/2027)</t>
+          <t>Valide 197j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 173j (07/02/2027)</t>
+          <t>Valide 172j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>173j</t>
+          <t>172j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 354j (07/08/2027)</t>
+          <t>Valide 353j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (02/11/2026)</t>
+          <t>Valide 75j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (26/01/2027)</t>
+          <t>Valide 159j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 94j (20/11/2026)</t>
+          <t>Valide 93j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>94j</t>
+          <t>93j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (02/11/2026)</t>
+          <t>Valide 75j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (09/02/2027)</t>
+          <t>Valide 174j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>174j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (28/02/2027)</t>
+          <t>Valide 193j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 173j (07/02/2027)</t>
+          <t>Valide 172j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>173j</t>
+          <t>172j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 338j (22/07/2027)</t>
+          <t>Valide 337j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (14/10/2026)</t>
+          <t>Valide 56j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (29/10/2026)</t>
+          <t>Valide 71j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (07/12/2026)</t>
+          <t>Valide 110j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (29/10/2026)</t>
+          <t>Valide 71j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 111j (07/12/2026)</t>
+          <t>Valide 110j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (09/10/2026)</t>
+          <t>Valide 51j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (30/11/2026)</t>
+          <t>Valide 103j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 52j (09/10/2026)</t>
+          <t>Valide 51j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 104j (30/11/2026)</t>
+          <t>Valide 103j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (09/02/2027)</t>
+          <t>Valide 174j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>174j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 94j (20/11/2026)</t>
+          <t>Valide 93j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 175j (09/02/2027)</t>
+          <t>Valide 174j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>175j</t>
+          <t>174j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 94j (20/11/2026)</t>
+          <t>Valide 93j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 123j (19/12/2026)</t>
+          <t>Valide 122j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>123j</t>
+          <t>122j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 347j (31/07/2027)</t>
+          <t>Valide 346j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 123j (19/12/2026)</t>
+          <t>Valide 122j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>123j</t>
+          <t>122j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 347j (31/07/2027)</t>
+          <t>Valide 346j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (13/10/2026)</t>
+          <t>Valide 55j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (10/10/2026)</t>
+          <t>Valide 52j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>18/08/2026 07:40</t>
+          <t>19/08/2026 07:40</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 20/08/2026 07:47
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (23/09/2026)</t>
+          <t>Valide 33j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 197j (05/03/2027)</t>
+          <t>Valide 196j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 172j (07/02/2027)</t>
+          <t>Valide 171j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>172j</t>
+          <t>171j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 353j (07/08/2027)</t>
+          <t>Valide 352j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (02/11/2026)</t>
+          <t>Valide 74j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (26/01/2027)</t>
+          <t>Valide 158j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 93j (20/11/2026)</t>
+          <t>Valide 92j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>93j</t>
+          <t>92j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (02/11/2026)</t>
+          <t>Valide 74j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (09/02/2027)</t>
+          <t>Valide 173j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>174j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (28/02/2027)</t>
+          <t>Valide 192j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 172j (07/02/2027)</t>
+          <t>Valide 171j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>172j</t>
+          <t>171j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 337j (22/07/2027)</t>
+          <t>Valide 336j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (14/10/2026)</t>
+          <t>Valide 55j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (29/10/2026)</t>
+          <t>Valide 70j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (07/12/2026)</t>
+          <t>Valide 109j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (29/10/2026)</t>
+          <t>Valide 70j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 110j (07/12/2026)</t>
+          <t>Valide 109j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (09/10/2026)</t>
+          <t>Valide 50j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (30/11/2026)</t>
+          <t>Valide 102j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 51j (09/10/2026)</t>
+          <t>Valide 50j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 103j (30/11/2026)</t>
+          <t>Valide 102j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (09/02/2027)</t>
+          <t>Valide 173j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>174j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 93j (20/11/2026)</t>
+          <t>Valide 92j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 174j (09/02/2027)</t>
+          <t>Valide 173j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>174j</t>
+          <t>173j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 93j (20/11/2026)</t>
+          <t>Valide 92j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 122j (19/12/2026)</t>
+          <t>Valide 121j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>122j</t>
+          <t>121j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 346j (31/07/2027)</t>
+          <t>Valide 345j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 122j (19/12/2026)</t>
+          <t>Valide 121j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>122j</t>
+          <t>121j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 346j (31/07/2027)</t>
+          <t>Valide 345j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (13/10/2026)</t>
+          <t>Valide 54j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (10/10/2026)</t>
+          <t>Valide 51j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>19/08/2026 07:40</t>
+          <t>20/08/2026 07:43</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 21/08/2026 07:51
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (23/09/2026)</t>
+          <t>Valide 32j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 196j (05/03/2027)</t>
+          <t>Valide 195j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 171j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>171j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 352j (07/08/2027)</t>
+          <t>Valide 351j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (02/11/2026)</t>
+          <t>Valide 73j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (26/01/2027)</t>
+          <t>Valide 157j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 92j (20/11/2026)</t>
+          <t>Valide 91j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>92j</t>
+          <t>91j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (02/11/2026)</t>
+          <t>Valide 73j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (09/02/2027)</t>
+          <t>Valide 172j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>173j</t>
+          <t>172j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (28/02/2027)</t>
+          <t>Valide 191j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 171j (07/02/2027)</t>
+          <t>Valide 170j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>171j</t>
+          <t>170j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 336j (22/07/2027)</t>
+          <t>Valide 335j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (14/10/2026)</t>
+          <t>Valide 54j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (29/10/2026)</t>
+          <t>Valide 69j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (07/12/2026)</t>
+          <t>Valide 108j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (29/10/2026)</t>
+          <t>Valide 69j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 109j (07/12/2026)</t>
+          <t>Valide 108j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (09/10/2026)</t>
+          <t>Valide 49j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (30/11/2026)</t>
+          <t>Valide 101j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 50j (09/10/2026)</t>
+          <t>Valide 49j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 102j (30/11/2026)</t>
+          <t>Valide 101j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (09/02/2027)</t>
+          <t>Valide 172j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>173j</t>
+          <t>172j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 92j (20/11/2026)</t>
+          <t>Valide 91j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 173j (09/02/2027)</t>
+          <t>Valide 172j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>173j</t>
+          <t>172j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 92j (20/11/2026)</t>
+          <t>Valide 91j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 121j (19/12/2026)</t>
+          <t>Valide 120j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>121j</t>
+          <t>120j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 345j (31/07/2027)</t>
+          <t>Valide 344j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 121j (19/12/2026)</t>
+          <t>Valide 120j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>121j</t>
+          <t>120j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 345j (31/07/2027)</t>
+          <t>Valide 344j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (13/10/2026)</t>
+          <t>Valide 53j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (10/10/2026)</t>
+          <t>Valide 50j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>20/08/2026 07:43</t>
+          <t>21/08/2026 07:46</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 22/08/2026 07:39
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (23/09/2026)</t>
+          <t>Valide 31j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 195j (05/03/2027)</t>
+          <t>Valide 194j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 169j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>169j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 351j (07/08/2027)</t>
+          <t>Valide 350j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (02/11/2026)</t>
+          <t>Valide 72j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (26/01/2027)</t>
+          <t>Valide 156j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 91j (20/11/2026)</t>
+          <t>Valide 90j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>91j</t>
+          <t>90j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (02/11/2026)</t>
+          <t>Valide 72j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (09/02/2027)</t>
+          <t>Valide 171j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>172j</t>
+          <t>171j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (28/02/2027)</t>
+          <t>Valide 190j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 170j (07/02/2027)</t>
+          <t>Valide 169j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>170j</t>
+          <t>169j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 335j (22/07/2027)</t>
+          <t>Valide 334j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (14/10/2026)</t>
+          <t>Valide 53j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (29/10/2026)</t>
+          <t>Valide 68j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (07/12/2026)</t>
+          <t>Valide 107j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 69j (29/10/2026)</t>
+          <t>Valide 68j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 108j (07/12/2026)</t>
+          <t>Valide 107j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (09/10/2026)</t>
+          <t>Valide 48j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 101j (30/11/2026)</t>
+          <t>Valide 100j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 49j (09/10/2026)</t>
+          <t>Valide 48j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 101j (30/11/2026)</t>
+          <t>Valide 100j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (09/02/2027)</t>
+          <t>Valide 171j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>172j</t>
+          <t>171j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 91j (20/11/2026)</t>
+          <t>Valide 90j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 172j (09/02/2027)</t>
+          <t>Valide 171j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>172j</t>
+          <t>171j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 91j (20/11/2026)</t>
+          <t>Valide 90j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 120j (19/12/2026)</t>
+          <t>Valide 119j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>119j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 344j (31/07/2027)</t>
+          <t>Valide 343j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 120j (19/12/2026)</t>
+          <t>Valide 119j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>120j</t>
+          <t>119j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 344j (31/07/2027)</t>
+          <t>Valide 343j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (13/10/2026)</t>
+          <t>Valide 52j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (10/10/2026)</t>
+          <t>Valide 49j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>21/08/2026 07:46</t>
+          <t>22/08/2026 07:34</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 23/08/2026 07:39
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,25 +842,29 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (23/09/2026)</t>
+          <t>Expire dans 30j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 194j (05/03/2027)</t>
+          <t>Valide 193j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
+          <t>23/08/2026 07:35</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="5" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A5" s="3" t="inlineStr">
@@ -976,22 +980,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 169j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>169j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 350j (07/08/2027)</t>
+          <t>Valide 349j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1050,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (02/11/2026)</t>
+          <t>Valide 71j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (26/01/2027)</t>
+          <t>Valide 155j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1156,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 90j (20/11/2026)</t>
+          <t>Valide 89j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>90j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (02/11/2026)</t>
+          <t>Valide 71j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1262,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (09/02/2027)</t>
+          <t>Valide 170j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>171j</t>
+          <t>170j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (28/02/2027)</t>
+          <t>Valide 189j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1584,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 169j (07/02/2027)</t>
+          <t>Valide 168j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>169j</t>
+          <t>168j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 334j (22/07/2027)</t>
+          <t>Valide 333j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1654,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (14/10/2026)</t>
+          <t>Valide 52j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1669,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1749,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (29/10/2026)</t>
+          <t>Valide 67j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (07/12/2026)</t>
+          <t>Valide 106j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1815,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 68j (29/10/2026)</t>
+          <t>Valide 67j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>67j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 107j (07/12/2026)</t>
+          <t>Valide 106j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1961,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (09/10/2026)</t>
+          <t>Valide 47j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 100j (30/11/2026)</t>
+          <t>Valide 99j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2011,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 48j (09/10/2026)</t>
+          <t>Valide 47j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 100j (30/11/2026)</t>
+          <t>Valide 99j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2189,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (09/02/2027)</t>
+          <t>Valide 170j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>171j</t>
+          <t>170j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 90j (20/11/2026)</t>
+          <t>Valide 89j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2251,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 171j (09/02/2027)</t>
+          <t>Valide 170j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>171j</t>
+          <t>170j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 90j (20/11/2026)</t>
+          <t>Valide 89j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2461,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 119j (19/12/2026)</t>
+          <t>Valide 118j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>119j</t>
+          <t>118j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 343j (31/07/2027)</t>
+          <t>Valide 342j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2515,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 119j (19/12/2026)</t>
+          <t>Valide 118j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>119j</t>
+          <t>118j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 343j (31/07/2027)</t>
+          <t>Valide 342j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2729,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (13/10/2026)</t>
+          <t>Valide 51j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (10/10/2026)</t>
+          <t>Valide 48j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>22/08/2026 07:34</t>
+          <t>23/08/2026 07:35</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 24/08/2026 08:03
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,29 +842,25 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (23/09/2026)</t>
+          <t>Expire dans 29j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 193j (05/03/2027)</t>
+          <t>Valide 192j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>24/08/2026 07:58</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A5" s="3" t="inlineStr">
@@ -990,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 349j (07/08/2027)</t>
+          <t>Valide 348j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1050,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (02/11/2026)</t>
+          <t>Valide 70j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (26/01/2027)</t>
+          <t>Valide 154j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1156,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (20/11/2026)</t>
+          <t>Valide 88j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (02/11/2026)</t>
+          <t>Valide 70j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1262,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (09/02/2027)</t>
+          <t>Valide 169j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>170j</t>
+          <t>169j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (28/02/2027)</t>
+          <t>Valide 188j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1584,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 168j (07/02/2027)</t>
+          <t>Valide 167j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>168j</t>
+          <t>167j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 333j (22/07/2027)</t>
+          <t>Valide 332j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1654,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (14/10/2026)</t>
+          <t>Valide 51j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1669,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1749,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 67j (29/10/2026)</t>
+          <t>Valide 66j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (07/12/2026)</t>
+          <t>Valide 105j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1815,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 67j (29/10/2026)</t>
+          <t>Valide 66j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>67j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 106j (07/12/2026)</t>
+          <t>Valide 105j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1961,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (09/10/2026)</t>
+          <t>Valide 46j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 99j (30/11/2026)</t>
+          <t>Valide 98j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2011,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 47j (09/10/2026)</t>
+          <t>Valide 46j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 99j (30/11/2026)</t>
+          <t>Valide 98j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2189,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (09/02/2027)</t>
+          <t>Valide 169j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>170j</t>
+          <t>169j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (20/11/2026)</t>
+          <t>Valide 88j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2251,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 170j (09/02/2027)</t>
+          <t>Valide 169j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>170j</t>
+          <t>169j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (20/11/2026)</t>
+          <t>Valide 88j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2461,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 118j (19/12/2026)</t>
+          <t>Valide 117j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>118j</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 342j (31/07/2027)</t>
+          <t>Valide 341j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2515,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 118j (19/12/2026)</t>
+          <t>Valide 117j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>118j</t>
+          <t>117j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 342j (31/07/2027)</t>
+          <t>Valide 341j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2729,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (13/10/2026)</t>
+          <t>Valide 50j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (10/10/2026)</t>
+          <t>Valide 47j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>23/08/2026 07:35</t>
+          <t>24/08/2026 07:58</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 25/08/2026 07:59
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (23/09/2026)</t>
+          <t>Expire dans 28j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>28j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 192j (05/03/2027)</t>
+          <t>Valide 191j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 348j (07/08/2027)</t>
+          <t>Valide 347j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (02/11/2026)</t>
+          <t>Valide 69j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (26/01/2027)</t>
+          <t>Valide 153j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (20/11/2026)</t>
+          <t>Valide 87j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (02/11/2026)</t>
+          <t>Valide 69j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (09/02/2027)</t>
+          <t>Valide 168j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>169j</t>
+          <t>168j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (28/02/2027)</t>
+          <t>Valide 187j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 167j (07/02/2027)</t>
+          <t>Valide 166j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>167j</t>
+          <t>166j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 332j (22/07/2027)</t>
+          <t>Valide 331j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (14/10/2026)</t>
+          <t>Valide 50j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (29/10/2026)</t>
+          <t>Valide 65j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (07/12/2026)</t>
+          <t>Valide 104j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 66j (29/10/2026)</t>
+          <t>Valide 65j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 105j (07/12/2026)</t>
+          <t>Valide 104j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (09/10/2026)</t>
+          <t>Valide 45j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 98j (30/11/2026)</t>
+          <t>Valide 97j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 46j (09/10/2026)</t>
+          <t>Valide 45j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 98j (30/11/2026)</t>
+          <t>Valide 97j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (09/02/2027)</t>
+          <t>Valide 168j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>169j</t>
+          <t>168j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (20/11/2026)</t>
+          <t>Valide 87j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 169j (09/02/2027)</t>
+          <t>Valide 168j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>169j</t>
+          <t>168j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 88j (20/11/2026)</t>
+          <t>Valide 87j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 117j (19/12/2026)</t>
+          <t>Valide 116j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 341j (31/07/2027)</t>
+          <t>Valide 340j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 117j (19/12/2026)</t>
+          <t>Valide 116j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>117j</t>
+          <t>116j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 341j (31/07/2027)</t>
+          <t>Valide 340j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (13/10/2026)</t>
+          <t>Valide 49j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (10/10/2026)</t>
+          <t>Valide 46j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>24/08/2026 07:58</t>
+          <t>25/08/2026 07:47</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 26/08/2026 07:54
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 28j (23/09/2026)</t>
+          <t>Expire dans 27j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>28j</t>
+          <t>27j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 191j (05/03/2027)</t>
+          <t>Valide 190j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 165j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>165j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 347j (07/08/2027)</t>
+          <t>Valide 346j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (02/11/2026)</t>
+          <t>Valide 68j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>69j</t>
+          <t>68j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (26/01/2027)</t>
+          <t>Valide 152j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (20/11/2026)</t>
+          <t>Valide 86j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 69j (02/11/2026)</t>
+          <t>Valide 68j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (09/02/2027)</t>
+          <t>Valide 167j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>168j</t>
+          <t>167j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (28/02/2027)</t>
+          <t>Valide 186j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 166j (07/02/2027)</t>
+          <t>Valide 165j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>166j</t>
+          <t>165j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 331j (22/07/2027)</t>
+          <t>Valide 330j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (14/10/2026)</t>
+          <t>Valide 49j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (29/10/2026)</t>
+          <t>Valide 64j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (07/12/2026)</t>
+          <t>Valide 103j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 65j (29/10/2026)</t>
+          <t>Valide 64j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 104j (07/12/2026)</t>
+          <t>Valide 103j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (09/10/2026)</t>
+          <t>Valide 44j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 97j (30/11/2026)</t>
+          <t>Valide 96j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 45j (09/10/2026)</t>
+          <t>Valide 44j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 97j (30/11/2026)</t>
+          <t>Valide 96j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 168j (09/02/2027)</t>
+          <t>Valide 167j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>168j</t>
+          <t>167j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (20/11/2026)</t>
+          <t>Valide 86j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 168j (09/02/2027)</t>
+          <t>Valide 167j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>168j</t>
+          <t>167j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (20/11/2026)</t>
+          <t>Valide 86j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 116j (19/12/2026)</t>
+          <t>Valide 115j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>115j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 340j (31/07/2027)</t>
+          <t>Valide 339j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 116j (19/12/2026)</t>
+          <t>Valide 115j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>116j</t>
+          <t>115j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 340j (31/07/2027)</t>
+          <t>Valide 339j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (13/10/2026)</t>
+          <t>Valide 48j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (10/10/2026)</t>
+          <t>Valide 45j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>25/08/2026 07:47</t>
+          <t>26/08/2026 07:49</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 27/08/2026 18:14
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 27j (23/09/2026)</t>
+          <t>Expire dans 26j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>27j</t>
+          <t>26j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 190j (05/03/2027)</t>
+          <t>Valide 189j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 165j (07/02/2027)</t>
+          <t>Valide 163j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>165j</t>
+          <t>163j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 346j (07/08/2027)</t>
+          <t>Valide 344j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (02/11/2026)</t>
+          <t>Valide 66j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>68j</t>
+          <t>66j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (26/01/2027)</t>
+          <t>Valide 151j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (20/11/2026)</t>
+          <t>Valide 85j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 68j (02/11/2026)</t>
+          <t>Valide 66j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (09/02/2027)</t>
+          <t>Valide 166j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>167j</t>
+          <t>166j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 186j (28/02/2027)</t>
+          <t>Valide 184j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 165j (07/02/2027)</t>
+          <t>Valide 163j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>165j</t>
+          <t>163j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 330j (22/07/2027)</t>
+          <t>Valide 328j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (14/10/2026)</t>
+          <t>Valide 48j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (29/10/2026)</t>
+          <t>Valide 63j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (07/12/2026)</t>
+          <t>Valide 102j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 64j (29/10/2026)</t>
+          <t>Valide 63j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 103j (07/12/2026)</t>
+          <t>Valide 102j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (09/10/2026)</t>
+          <t>Valide 43j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 96j (30/11/2026)</t>
+          <t>Valide 94j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 44j (09/10/2026)</t>
+          <t>Valide 43j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 96j (30/11/2026)</t>
+          <t>Valide 94j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 167j (09/02/2027)</t>
+          <t>Valide 166j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>167j</t>
+          <t>166j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (20/11/2026)</t>
+          <t>Valide 84j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 167j (09/02/2027)</t>
+          <t>Valide 166j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>167j</t>
+          <t>166j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (20/11/2026)</t>
+          <t>Valide 84j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 115j (19/12/2026)</t>
+          <t>Valide 114j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>115j</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 339j (31/07/2027)</t>
+          <t>Valide 337j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 115j (19/12/2026)</t>
+          <t>Valide 114j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>115j</t>
+          <t>114j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 339j (31/07/2027)</t>
+          <t>Valide 337j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (13/10/2026)</t>
+          <t>Valide 47j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (10/10/2026)</t>
+          <t>Valide 43j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>26/08/2026 07:49</t>
+          <t>27/08/2026 18:09</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 28/08/2026 19:25
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 26j (23/09/2026)</t>
+          <t>Expire dans 25j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>26j</t>
+          <t>25j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 189j (05/03/2027)</t>
+          <t>Valide 188j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 163j (07/02/2027)</t>
+          <t>Valide 162j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>163j</t>
+          <t>162j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 344j (07/08/2027)</t>
+          <t>Valide 343j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (02/11/2026)</t>
+          <t>Valide 65j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>66j</t>
+          <t>65j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (26/01/2027)</t>
+          <t>Valide 150j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (20/11/2026)</t>
+          <t>Valide 84j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 66j (02/11/2026)</t>
+          <t>Valide 65j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (09/02/2027)</t>
+          <t>Valide 165j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>166j</t>
+          <t>165j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 184j (28/02/2027)</t>
+          <t>Valide 183j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 163j (07/02/2027)</t>
+          <t>Valide 162j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>163j</t>
+          <t>162j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 328j (22/07/2027)</t>
+          <t>Valide 327j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (14/10/2026)</t>
+          <t>Valide 47j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (29/10/2026)</t>
+          <t>Valide 62j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (07/12/2026)</t>
+          <t>Valide 100j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 63j (29/10/2026)</t>
+          <t>Valide 62j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 102j (07/12/2026)</t>
+          <t>Valide 100j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (09/10/2026)</t>
+          <t>Valide 42j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 94j (30/11/2026)</t>
+          <t>Valide 93j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 43j (09/10/2026)</t>
+          <t>Valide 42j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 94j (30/11/2026)</t>
+          <t>Valide 93j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 166j (09/02/2027)</t>
+          <t>Valide 165j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>166j</t>
+          <t>165j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (20/11/2026)</t>
+          <t>Valide 83j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 166j (09/02/2027)</t>
+          <t>Valide 165j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>166j</t>
+          <t>165j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (20/11/2026)</t>
+          <t>Valide 83j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 114j (19/12/2026)</t>
+          <t>Valide 113j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 337j (31/07/2027)</t>
+          <t>Valide 336j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 114j (19/12/2026)</t>
+          <t>Valide 113j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>114j</t>
+          <t>113j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 337j (31/07/2027)</t>
+          <t>Valide 336j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (13/10/2026)</t>
+          <t>Valide 46j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (10/10/2026)</t>
+          <t>Valide 42j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>27/08/2026 18:09</t>
+          <t>28/08/2026 19:19</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 29/08/2026 13:08
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 25j (23/09/2026)</t>
+          <t>Expire dans 24j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>25j</t>
+          <t>24j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 188j (05/03/2027)</t>
+          <t>Valide 187j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 343j (07/08/2027)</t>
+          <t>Valide 342j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (02/11/2026)</t>
+          <t>Valide 64j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>65j</t>
+          <t>64j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 150j (26/01/2027)</t>
+          <t>Valide 149j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (20/11/2026)</t>
+          <t>Valide 83j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 65j (02/11/2026)</t>
+          <t>Valide 64j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (09/02/2027)</t>
+          <t>Valide 164j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>165j</t>
+          <t>164j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (28/02/2027)</t>
+          <t>Valide 182j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 327j (22/07/2027)</t>
+          <t>Valide 326j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 47j (14/10/2026)</t>
+          <t>Valide 46j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>47j</t>
+          <t>46j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,12 +1745,12 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (29/10/2026)</t>
+          <t>Valide 61j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 62j (29/10/2026)</t>
+          <t>Valide 61j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,12 +1957,12 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (09/10/2026)</t>
+          <t>Valide 41j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,12 +2007,12 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 42j (09/10/2026)</t>
+          <t>Valide 41j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,12 +2185,12 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 165j (09/02/2027)</t>
+          <t>Valide 164j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>165j</t>
+          <t>164j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,12 +2247,12 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 165j (09/02/2027)</t>
+          <t>Valide 164j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>165j</t>
+          <t>164j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 113j (19/12/2026)</t>
+          <t>Valide 112j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>112j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 336j (31/07/2027)</t>
+          <t>Valide 335j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 113j (19/12/2026)</t>
+          <t>Valide 112j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>113j</t>
+          <t>112j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 336j (31/07/2027)</t>
+          <t>Valide 335j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,12 +2725,12 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (13/10/2026)</t>
+          <t>Valide 45j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>28/08/2026 19:19</t>
+          <t>29/08/2026 13:03</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 30/08/2026 12:44
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 24j (23/09/2026)</t>
+          <t>Expire dans 23j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>24j</t>
+          <t>23j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 187j (05/03/2027)</t>
+          <t>Valide 186j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 162j (07/02/2027)</t>
+          <t>Valide 161j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>162j</t>
+          <t>161j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 342j (07/08/2027)</t>
+          <t>Valide 341j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (02/11/2026)</t>
+          <t>Valide 63j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>64j</t>
+          <t>63j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 149j (26/01/2027)</t>
+          <t>Valide 148j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (20/11/2026)</t>
+          <t>Valide 82j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 64j (02/11/2026)</t>
+          <t>Valide 63j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (09/02/2027)</t>
+          <t>Valide 163j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>164j</t>
+          <t>163j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (28/02/2027)</t>
+          <t>Valide 181j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 162j (07/02/2027)</t>
+          <t>Valide 161j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>162j</t>
+          <t>161j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 326j (22/07/2027)</t>
+          <t>Valide 325j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 46j (14/10/2026)</t>
+          <t>Valide 45j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>46j</t>
+          <t>45j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (29/10/2026)</t>
+          <t>Valide 60j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 100j (07/12/2026)</t>
+          <t>Valide 99j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 61j (29/10/2026)</t>
+          <t>Valide 60j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 100j (07/12/2026)</t>
+          <t>Valide 99j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (09/10/2026)</t>
+          <t>Valide 40j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 93j (30/11/2026)</t>
+          <t>Valide 92j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 41j (09/10/2026)</t>
+          <t>Valide 40j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 93j (30/11/2026)</t>
+          <t>Valide 92j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 164j (09/02/2027)</t>
+          <t>Valide 163j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>164j</t>
+          <t>163j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (20/11/2026)</t>
+          <t>Valide 82j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 164j (09/02/2027)</t>
+          <t>Valide 163j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>164j</t>
+          <t>163j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 83j (20/11/2026)</t>
+          <t>Valide 82j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 112j (19/12/2026)</t>
+          <t>Valide 111j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>112j</t>
+          <t>111j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 335j (31/07/2027)</t>
+          <t>Valide 334j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 112j (19/12/2026)</t>
+          <t>Valide 111j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>112j</t>
+          <t>111j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 335j (31/07/2027)</t>
+          <t>Valide 334j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (13/10/2026)</t>
+          <t>Valide 44j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (10/10/2026)</t>
+          <t>Valide 41j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>29/08/2026 13:03</t>
+          <t>30/08/2026 12:40</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 31/08/2026 15:01
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 23j (23/09/2026)</t>
+          <t>Expire dans 22j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>23j</t>
+          <t>22j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 186j (05/03/2027)</t>
+          <t>Valide 185j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 161j (07/02/2027)</t>
+          <t>Valide 159j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>161j</t>
+          <t>159j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 341j (07/08/2027)</t>
+          <t>Valide 340j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (02/11/2026)</t>
+          <t>Valide 62j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>63j</t>
+          <t>62j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 148j (26/01/2027)</t>
+          <t>Valide 147j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (20/11/2026)</t>
+          <t>Valide 81j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>82j</t>
+          <t>81j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 63j (02/11/2026)</t>
+          <t>Valide 62j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (09/02/2027)</t>
+          <t>Valide 162j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>163j</t>
+          <t>162j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (28/02/2027)</t>
+          <t>Valide 180j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 161j (07/02/2027)</t>
+          <t>Valide 159j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>161j</t>
+          <t>159j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 325j (22/07/2027)</t>
+          <t>Valide 324j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 45j (14/10/2026)</t>
+          <t>Valide 44j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>45j</t>
+          <t>44j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1740,30 +1740,34 @@
       </c>
       <c r="K25" s="9" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (29/10/2026)</t>
+          <t>Valide 59j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 99j (07/12/2026)</t>
+          <t>Valide 98j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr"/>
+          <t>31/08/2026 14:56</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1" s="34">
       <c r="A26" s="3" t="inlineStr">
@@ -1806,30 +1810,34 @@
       <c r="J26" s="4" t="n"/>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>DOWN</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 60j (29/10/2026)</t>
+          <t>Valide 59j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 99j (07/12/2026)</t>
+          <t>Valide 98j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr"/>
+          <t>31/08/2026 14:56</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="8" t="inlineStr">
@@ -1957,22 +1965,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (09/10/2026)</t>
+          <t>Valide 39j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 92j (30/11/2026)</t>
+          <t>Valide 91j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2015,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 40j (09/10/2026)</t>
+          <t>Valide 39j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 92j (30/11/2026)</t>
+          <t>Valide 91j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2193,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 163j (09/02/2027)</t>
+          <t>Valide 162j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>163j</t>
+          <t>162j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (20/11/2026)</t>
+          <t>Valide 80j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2255,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 163j (09/02/2027)</t>
+          <t>Valide 162j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>163j</t>
+          <t>162j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (20/11/2026)</t>
+          <t>Valide 80j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2465,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 111j (19/12/2026)</t>
+          <t>Valide 110j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>111j</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 334j (31/07/2027)</t>
+          <t>Valide 333j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2519,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 111j (19/12/2026)</t>
+          <t>Valide 110j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>111j</t>
+          <t>110j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 334j (31/07/2027)</t>
+          <t>Valide 333j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2733,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (13/10/2026)</t>
+          <t>Valide 43j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (10/10/2026)</t>
+          <t>Valide 39j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>30/08/2026 12:40</t>
+          <t>31/08/2026 14:56</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 01/09/2026 12:33
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 22j (23/09/2026)</t>
+          <t>Expire dans 21j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>22j</t>
+          <t>21j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 185j (05/03/2027)</t>
+          <t>Valide 184j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 340j (07/08/2027)</t>
+          <t>Valide 339j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (02/11/2026)</t>
+          <t>Valide 61j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>62j</t>
+          <t>61j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 147j (26/01/2027)</t>
+          <t>Valide 146j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (20/11/2026)</t>
+          <t>Valide 80j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>81j</t>
+          <t>80j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 62j (02/11/2026)</t>
+          <t>Valide 61j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (09/02/2027)</t>
+          <t>Valide 161j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>162j</t>
+          <t>161j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (28/02/2027)</t>
+          <t>Valide 179j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1590,12 +1590,12 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 324j (22/07/2027)</t>
+          <t>Valide 323j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 44j (14/10/2026)</t>
+          <t>Valide 43j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>44j</t>
+          <t>43j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1740,34 +1740,30 @@
       </c>
       <c r="K25" s="9" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (29/10/2026)</t>
+          <t>Valide 58j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 98j (07/12/2026)</t>
+          <t>Valide 97j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>01/09/2026 12:26</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26" ht="18" customHeight="1" s="34">
       <c r="A26" s="3" t="inlineStr">
@@ -1810,34 +1806,30 @@
       <c r="J26" s="4" t="n"/>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>UP</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 59j (29/10/2026)</t>
+          <t>Valide 58j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 98j (07/12/2026)</t>
+          <t>Valide 97j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>01/09/2026 12:26</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A27" s="8" t="inlineStr">
@@ -1965,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (09/10/2026)</t>
+          <t>Valide 38j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 91j (30/11/2026)</t>
+          <t>Valide 90j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2015,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 39j (09/10/2026)</t>
+          <t>Valide 38j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 91j (30/11/2026)</t>
+          <t>Valide 90j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2193,12 +2185,12 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 162j (09/02/2027)</t>
+          <t>Valide 161j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>162j</t>
+          <t>161j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
@@ -2208,7 +2200,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2255,12 +2247,12 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 162j (09/02/2027)</t>
+          <t>Valide 161j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>162j</t>
+          <t>161j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
@@ -2270,7 +2262,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2465,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 110j (19/12/2026)</t>
+          <t>Valide 109j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>109j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 333j (31/07/2027)</t>
+          <t>Valide 332j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2519,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 110j (19/12/2026)</t>
+          <t>Valide 109j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>110j</t>
+          <t>109j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 333j (31/07/2027)</t>
+          <t>Valide 332j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2733,12 +2725,12 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (13/10/2026)</t>
+          <t>Valide 42j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
@@ -2748,7 +2740,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>31/08/2026 14:56</t>
+          <t>01/09/2026 12:26</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 02/09/2026 12:07
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 21j (23/09/2026)</t>
+          <t>Expire dans 20j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>21j</t>
+          <t>20j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 184j (05/03/2027)</t>
+          <t>Valide 183j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 159j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>159j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 339j (07/08/2027)</t>
+          <t>Valide 338j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (02/11/2026)</t>
+          <t>Valide 60j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>61j</t>
+          <t>60j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 146j (26/01/2027)</t>
+          <t>Valide 145j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (20/11/2026)</t>
+          <t>Valide 79j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>80j</t>
+          <t>79j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (09/02/2027)</t>
+          <t>Valide 160j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>161j</t>
+          <t>160j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (28/02/2027)</t>
+          <t>Valide 178j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 159j (07/02/2027)</t>
+          <t>Valide 158j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>159j</t>
+          <t>158j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 323j (22/07/2027)</t>
+          <t>Valide 322j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 43j (14/10/2026)</t>
+          <t>Valide 42j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>43j</t>
+          <t>42j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (29/10/2026)</t>
+          <t>Valide 57j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 97j (07/12/2026)</t>
+          <t>Valide 96j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 58j (29/10/2026)</t>
+          <t>Valide 57j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 97j (07/12/2026)</t>
+          <t>Valide 96j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (09/10/2026)</t>
+          <t>Valide 37j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 90j (30/11/2026)</t>
+          <t>Valide 89j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 38j (09/10/2026)</t>
+          <t>Valide 37j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 90j (30/11/2026)</t>
+          <t>Valide 89j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 161j (09/02/2027)</t>
+          <t>Valide 160j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>161j</t>
+          <t>160j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (20/11/2026)</t>
+          <t>Valide 79j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 161j (09/02/2027)</t>
+          <t>Valide 160j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>161j</t>
+          <t>160j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 80j (20/11/2026)</t>
+          <t>Valide 79j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 109j (19/12/2026)</t>
+          <t>Valide 108j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>109j</t>
+          <t>108j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 332j (31/07/2027)</t>
+          <t>Valide 331j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 109j (19/12/2026)</t>
+          <t>Valide 108j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>109j</t>
+          <t>108j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 332j (31/07/2027)</t>
+          <t>Valide 331j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (13/10/2026)</t>
+          <t>Valide 41j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (10/10/2026)</t>
+          <t>Valide 38j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>01/09/2026 12:26</t>
+          <t>02/09/2026 12:00</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 03/09/2026 12:05
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 20j (23/09/2026)</t>
+          <t>Expire dans 19j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>20j</t>
+          <t>19j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 183j (05/03/2027)</t>
+          <t>Valide 182j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 157j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>157j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 338j (07/08/2027)</t>
+          <t>Valide 337j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (02/11/2026)</t>
+          <t>Valide 59j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>60j</t>
+          <t>59j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 145j (26/01/2027)</t>
+          <t>Valide 144j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (20/11/2026)</t>
+          <t>Valide 78j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>79j</t>
+          <t>78j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 61j (02/11/2026)</t>
+          <t>Valide 60j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (09/02/2027)</t>
+          <t>Valide 159j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>160j</t>
+          <t>159j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (28/02/2027)</t>
+          <t>Valide 177j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 158j (07/02/2027)</t>
+          <t>Valide 157j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>158j</t>
+          <t>157j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 322j (22/07/2027)</t>
+          <t>Valide 321j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 42j (14/10/2026)</t>
+          <t>Valide 41j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>42j</t>
+          <t>41j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (29/10/2026)</t>
+          <t>Valide 56j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 96j (07/12/2026)</t>
+          <t>Valide 95j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 57j (29/10/2026)</t>
+          <t>Valide 56j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 96j (07/12/2026)</t>
+          <t>Valide 95j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (09/10/2026)</t>
+          <t>Valide 36j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (30/11/2026)</t>
+          <t>Valide 88j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 37j (09/10/2026)</t>
+          <t>Valide 36j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (30/11/2026)</t>
+          <t>Valide 88j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 160j (09/02/2027)</t>
+          <t>Valide 159j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>160j</t>
+          <t>159j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 79j (20/11/2026)</t>
+          <t>Valide 78j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 160j (09/02/2027)</t>
+          <t>Valide 159j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>160j</t>
+          <t>159j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 79j (20/11/2026)</t>
+          <t>Valide 78j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 108j (19/12/2026)</t>
+          <t>Valide 107j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>108j</t>
+          <t>107j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 331j (31/07/2027)</t>
+          <t>Valide 330j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 108j (19/12/2026)</t>
+          <t>Valide 107j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>108j</t>
+          <t>107j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 331j (31/07/2027)</t>
+          <t>Valide 330j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (13/10/2026)</t>
+          <t>Valide 40j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (10/10/2026)</t>
+          <t>Valide 37j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>02/09/2026 12:00</t>
+          <t>03/09/2026 11:59</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 04/09/2026 12:08
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 19j (23/09/2026)</t>
+          <t>Expire dans 18j (23/09/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>19j</t>
+          <t>18j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 182j (05/03/2027)</t>
+          <t>Valide 181j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 157j (07/02/2027)</t>
+          <t>Valide 156j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>157j</t>
+          <t>156j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 337j (07/08/2027)</t>
+          <t>Valide 336j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (02/11/2026)</t>
+          <t>Valide 58j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>59j</t>
+          <t>58j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 144j (26/01/2027)</t>
+          <t>Valide 143j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (20/11/2026)</t>
+          <t>Valide 77j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>78j</t>
+          <t>77j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 60j (02/11/2026)</t>
+          <t>Valide 59j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (09/02/2027)</t>
+          <t>Valide 158j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>159j</t>
+          <t>158j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (28/02/2027)</t>
+          <t>Valide 176j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 157j (07/02/2027)</t>
+          <t>Valide 156j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>157j</t>
+          <t>156j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 321j (22/07/2027)</t>
+          <t>Valide 320j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 41j (14/10/2026)</t>
+          <t>Valide 40j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>41j</t>
+          <t>40j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (29/10/2026)</t>
+          <t>Valide 55j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 95j (07/12/2026)</t>
+          <t>Valide 94j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 56j (29/10/2026)</t>
+          <t>Valide 55j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 95j (07/12/2026)</t>
+          <t>Valide 94j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (09/10/2026)</t>
+          <t>Valide 35j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (30/11/2026)</t>
+          <t>Valide 87j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 36j (09/10/2026)</t>
+          <t>Valide 35j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 88j (30/11/2026)</t>
+          <t>Valide 87j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 159j (09/02/2027)</t>
+          <t>Valide 158j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>159j</t>
+          <t>158j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 78j (20/11/2026)</t>
+          <t>Valide 77j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 159j (09/02/2027)</t>
+          <t>Valide 158j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>159j</t>
+          <t>158j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 78j (20/11/2026)</t>
+          <t>Valide 77j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 107j (19/12/2026)</t>
+          <t>Valide 106j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>107j</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 330j (31/07/2027)</t>
+          <t>Valide 329j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 107j (19/12/2026)</t>
+          <t>Valide 106j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>107j</t>
+          <t>106j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 330j (31/07/2027)</t>
+          <t>Valide 329j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (13/10/2026)</t>
+          <t>Valide 39j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (10/10/2026)</t>
+          <t>Valide 36j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>03/09/2026 11:59</t>
+          <t>04/09/2026 12:01</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 05/09/2026 11:16
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 18j (23/09/2026)</t>
+          <t>Valide 89j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>18j</t>
+          <t>89j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 181j (05/03/2027)</t>
+          <t>Valide 180j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 156j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>156j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 336j (07/08/2027)</t>
+          <t>Valide 335j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (02/11/2026)</t>
+          <t>Valide 57j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>58j</t>
+          <t>57j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 143j (26/01/2027)</t>
+          <t>Valide 142j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (20/11/2026)</t>
+          <t>Valide 76j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>77j</t>
+          <t>76j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 59j (02/11/2026)</t>
+          <t>Valide 58j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (09/02/2027)</t>
+          <t>Valide 157j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>158j</t>
+          <t>157j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (28/02/2027)</t>
+          <t>Valide 175j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 156j (07/02/2027)</t>
+          <t>Valide 155j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>156j</t>
+          <t>155j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 320j (22/07/2027)</t>
+          <t>Valide 319j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 40j (14/10/2026)</t>
+          <t>Valide 39j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>40j</t>
+          <t>39j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (29/10/2026)</t>
+          <t>Valide 54j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 94j (07/12/2026)</t>
+          <t>Valide 93j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 55j (29/10/2026)</t>
+          <t>Valide 54j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 94j (07/12/2026)</t>
+          <t>Valide 93j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (09/10/2026)</t>
+          <t>Valide 34j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (30/11/2026)</t>
+          <t>Valide 86j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 35j (09/10/2026)</t>
+          <t>Valide 34j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (30/11/2026)</t>
+          <t>Valide 86j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 158j (09/02/2027)</t>
+          <t>Valide 157j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>158j</t>
+          <t>157j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 77j (20/11/2026)</t>
+          <t>Valide 76j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 158j (09/02/2027)</t>
+          <t>Valide 157j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>158j</t>
+          <t>157j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 77j (20/11/2026)</t>
+          <t>Valide 76j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 106j (19/12/2026)</t>
+          <t>Valide 105j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 329j (31/07/2027)</t>
+          <t>Valide 328j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 106j (19/12/2026)</t>
+          <t>Valide 105j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>106j</t>
+          <t>105j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 329j (31/07/2027)</t>
+          <t>Valide 328j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (13/10/2026)</t>
+          <t>Valide 38j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (10/10/2026)</t>
+          <t>Valide 35j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>04/09/2026 12:01</t>
+          <t>05/09/2026 11:11</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 06/09/2026 11:41
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (04/12/2026)</t>
+          <t>Valide 88j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>89j</t>
+          <t>88j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 180j (05/03/2027)</t>
+          <t>Valide 179j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 154j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>154j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 335j (07/08/2027)</t>
+          <t>Valide 334j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (02/11/2026)</t>
+          <t>Valide 56j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>57j</t>
+          <t>56j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 142j (26/01/2027)</t>
+          <t>Valide 141j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (20/11/2026)</t>
+          <t>Valide 75j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>76j</t>
+          <t>75j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 58j (02/11/2026)</t>
+          <t>Valide 57j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (09/02/2027)</t>
+          <t>Valide 156j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>157j</t>
+          <t>156j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (28/02/2027)</t>
+          <t>Valide 174j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 155j (07/02/2027)</t>
+          <t>Valide 154j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>155j</t>
+          <t>154j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 319j (22/07/2027)</t>
+          <t>Valide 318j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 39j (14/10/2026)</t>
+          <t>Valide 38j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>39j</t>
+          <t>38j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (29/10/2026)</t>
+          <t>Valide 53j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 93j (07/12/2026)</t>
+          <t>Valide 92j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 54j (29/10/2026)</t>
+          <t>Valide 53j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 93j (07/12/2026)</t>
+          <t>Valide 92j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (09/10/2026)</t>
+          <t>Valide 33j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (30/11/2026)</t>
+          <t>Valide 85j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 34j (09/10/2026)</t>
+          <t>Valide 33j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 86j (30/11/2026)</t>
+          <t>Valide 85j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 157j (09/02/2027)</t>
+          <t>Valide 156j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>157j</t>
+          <t>156j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 76j (20/11/2026)</t>
+          <t>Valide 75j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 157j (09/02/2027)</t>
+          <t>Valide 156j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>157j</t>
+          <t>156j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 76j (20/11/2026)</t>
+          <t>Valide 75j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 105j (19/12/2026)</t>
+          <t>Valide 104j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 328j (31/07/2027)</t>
+          <t>Valide 327j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 105j (19/12/2026)</t>
+          <t>Valide 104j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>105j</t>
+          <t>104j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 328j (31/07/2027)</t>
+          <t>Valide 327j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (13/10/2026)</t>
+          <t>Valide 37j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (10/10/2026)</t>
+          <t>Valide 34j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>05/09/2026 11:11</t>
+          <t>06/09/2026 11:34</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 07/09/2026 13:28
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (04/12/2026)</t>
+          <t>Valide 87j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>88j</t>
+          <t>87j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 179j (05/03/2027)</t>
+          <t>Valide 178j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 154j (07/02/2027)</t>
+          <t>Valide 153j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>154j</t>
+          <t>153j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 334j (07/08/2027)</t>
+          <t>Valide 333j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 56j (02/11/2026)</t>
+          <t>Valide 55j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>56j</t>
+          <t>55j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 141j (26/01/2027)</t>
+          <t>Valide 140j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (20/11/2026)</t>
+          <t>Valide 74j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>75j</t>
+          <t>74j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 57j (02/11/2026)</t>
+          <t>Valide 55j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (09/02/2027)</t>
+          <t>Valide 155j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>156j</t>
+          <t>155j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (28/02/2027)</t>
+          <t>Valide 173j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 154j (07/02/2027)</t>
+          <t>Valide 153j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>154j</t>
+          <t>153j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 318j (22/07/2027)</t>
+          <t>Valide 317j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 38j (14/10/2026)</t>
+          <t>Valide 37j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>38j</t>
+          <t>37j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (29/10/2026)</t>
+          <t>Valide 52j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 92j (07/12/2026)</t>
+          <t>Valide 91j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 53j (29/10/2026)</t>
+          <t>Valide 52j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 92j (07/12/2026)</t>
+          <t>Valide 91j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (09/10/2026)</t>
+          <t>Valide 32j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (30/11/2026)</t>
+          <t>Valide 84j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 33j (09/10/2026)</t>
+          <t>Valide 32j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 85j (30/11/2026)</t>
+          <t>Valide 84j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 156j (09/02/2027)</t>
+          <t>Valide 155j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>156j</t>
+          <t>155j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 75j (20/11/2026)</t>
+          <t>Valide 74j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 156j (09/02/2027)</t>
+          <t>Valide 155j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>156j</t>
+          <t>155j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 75j (20/11/2026)</t>
+          <t>Valide 74j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 104j (19/12/2026)</t>
+          <t>Valide 103j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 327j (31/07/2027)</t>
+          <t>Valide 326j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 104j (19/12/2026)</t>
+          <t>Valide 103j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>104j</t>
+          <t>103j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 327j (31/07/2027)</t>
+          <t>Valide 326j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (13/10/2026)</t>
+          <t>Valide 36j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (10/10/2026)</t>
+          <t>Valide 32j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>06/09/2026 11:34</t>
+          <t>07/09/2026 13:22</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 08/09/2026 12:08
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (04/12/2026)</t>
+          <t>Valide 86j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>87j</t>
+          <t>86j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 178j (05/03/2027)</t>
+          <t>Valide 177j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 153j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>153j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 333j (07/08/2027)</t>
+          <t>Valide 332j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (02/11/2026)</t>
+          <t>Valide 54j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>55j</t>
+          <t>54j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 140j (26/01/2027)</t>
+          <t>Valide 139j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (20/11/2026)</t>
+          <t>Valide 73j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>74j</t>
+          <t>73j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (09/02/2027)</t>
+          <t>Valide 154j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>155j</t>
+          <t>154j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 173j (28/02/2027)</t>
+          <t>Valide 172j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 153j (07/02/2027)</t>
+          <t>Valide 152j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>153j</t>
+          <t>152j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 317j (22/07/2027)</t>
+          <t>Valide 316j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 37j (14/10/2026)</t>
+          <t>Valide 36j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>37j</t>
+          <t>36j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (29/10/2026)</t>
+          <t>Valide 51j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 91j (07/12/2026)</t>
+          <t>Valide 90j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 52j (29/10/2026)</t>
+          <t>Valide 51j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 91j (07/12/2026)</t>
+          <t>Valide 90j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (09/10/2026)</t>
+          <t>Valide 31j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (30/11/2026)</t>
+          <t>Valide 83j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 32j (09/10/2026)</t>
+          <t>Valide 31j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 84j (30/11/2026)</t>
+          <t>Valide 83j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 155j (09/02/2027)</t>
+          <t>Valide 154j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>155j</t>
+          <t>154j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 74j (20/11/2026)</t>
+          <t>Valide 73j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 155j (09/02/2027)</t>
+          <t>Valide 154j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>155j</t>
+          <t>154j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 74j (20/11/2026)</t>
+          <t>Valide 73j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 103j (19/12/2026)</t>
+          <t>Valide 102j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 326j (31/07/2027)</t>
+          <t>Valide 325j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 103j (19/12/2026)</t>
+          <t>Valide 102j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>103j</t>
+          <t>102j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 326j (31/07/2027)</t>
+          <t>Valide 325j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,12 +2725,12 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (13/10/2026)</t>
+          <t>Valide 35j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>07/09/2026 13:22</t>
+          <t>08/09/2026 12:02</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 09/09/2026 12:19
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 86j (04/12/2026)</t>
+          <t>Valide 85j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>86j</t>
+          <t>85j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 177j (05/03/2027)</t>
+          <t>Valide 176j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 332j (07/08/2027)</t>
+          <t>Valide 331j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (02/11/2026)</t>
+          <t>Valide 53j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>54j</t>
+          <t>53j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 139j (26/01/2027)</t>
+          <t>Valide 138j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (20/11/2026)</t>
+          <t>Valide 72j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>73j</t>
+          <t>72j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 55j (02/11/2026)</t>
+          <t>Valide 54j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (09/02/2027)</t>
+          <t>Valide 153j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>154j</t>
+          <t>153j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 172j (28/02/2027)</t>
+          <t>Valide 171j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 152j (07/02/2027)</t>
+          <t>Valide 151j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>152j</t>
+          <t>151j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 316j (22/07/2027)</t>
+          <t>Valide 315j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 36j (14/10/2026)</t>
+          <t>Valide 35j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>36j</t>
+          <t>35j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (29/10/2026)</t>
+          <t>Valide 50j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 90j (07/12/2026)</t>
+          <t>Valide 89j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 51j (29/10/2026)</t>
+          <t>Valide 50j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 90j (07/12/2026)</t>
+          <t>Valide 89j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,25 +1957,29 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (09/10/2026)</t>
+          <t>Expire dans 30j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (30/11/2026)</t>
+          <t>Valide 82j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr"/>
+          <t>09/09/2026 12:12</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1" s="34">
       <c r="A30" s="3" t="inlineStr">
@@ -2007,25 +2011,29 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Valide 31j (09/10/2026)</t>
+          <t>Expire dans 30j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>31j</t>
+          <t>30j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 83j (30/11/2026)</t>
+          <t>Valide 82j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr"/>
+          <t>09/09/2026 12:12</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="31" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A31" s="8" t="inlineStr">
@@ -2185,22 +2193,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 154j (09/02/2027)</t>
+          <t>Valide 153j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>154j</t>
+          <t>153j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 73j (20/11/2026)</t>
+          <t>Valide 72j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2255,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 154j (09/02/2027)</t>
+          <t>Valide 153j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>154j</t>
+          <t>153j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 73j (20/11/2026)</t>
+          <t>Valide 72j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2465,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 102j (19/12/2026)</t>
+          <t>Valide 101j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 325j (31/07/2027)</t>
+          <t>Valide 324j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2519,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 102j (19/12/2026)</t>
+          <t>Valide 101j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>102j</t>
+          <t>101j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 325j (31/07/2027)</t>
+          <t>Valide 324j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2733,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (13/10/2026)</t>
+          <t>Valide 34j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (10/10/2026)</t>
+          <t>Valide 31j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>08/09/2026 12:02</t>
+          <t>09/09/2026 12:12</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: monitoring 10/09/2026 12:14
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 85j (04/12/2026)</t>
+          <t>Valide 84j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>85j</t>
+          <t>84j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 176j (05/03/2027)</t>
+          <t>Valide 175j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>Valide 150j (07/02/2027)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>Port 443 inaccessible (pas de SSL)</t>
+          <t>150j</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 331j (07/08/2027)</t>
+          <t>Valide 330j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (02/11/2026)</t>
+          <t>Valide 52j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>53j</t>
+          <t>52j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 138j (26/01/2027)</t>
+          <t>Valide 137j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (20/11/2026)</t>
+          <t>Valide 71j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>72j</t>
+          <t>71j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 54j (02/11/2026)</t>
+          <t>Valide 53j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (09/02/2027)</t>
+          <t>Valide 152j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>153j</t>
+          <t>152j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 171j (28/02/2027)</t>
+          <t>Valide 170j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 151j (07/02/2027)</t>
+          <t>Valide 150j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>151j</t>
+          <t>150j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 315j (22/07/2027)</t>
+          <t>Valide 314j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 35j (14/10/2026)</t>
+          <t>Valide 34j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>35j</t>
+          <t>34j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 50j (29/10/2026)</t>
+          <t>Valide 49j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 89j (07/12/2026)</t>
+          <t>Valide 88j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 50j (29/10/2026)</t>
+          <t>Valide 49j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>50j</t>
+          <t>49j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 89j (07/12/2026)</t>
+          <t>Valide 88j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,29 +1957,25 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (09/10/2026)</t>
+          <t>Expire dans 29j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 82j (30/11/2026)</t>
+          <t>Valide 81j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>10/09/2026 12:07</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1" s="34">
       <c r="A30" s="3" t="inlineStr">
@@ -2011,29 +2007,25 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 30j (09/10/2026)</t>
+          <t>Expire dans 29j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>30j</t>
+          <t>29j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 82j (30/11/2026)</t>
+          <t>Valide 81j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>10/09/2026 12:07</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31" hidden="1" ht="18" customHeight="1" s="34">
       <c r="A31" s="8" t="inlineStr">
@@ -2193,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 153j (09/02/2027)</t>
+          <t>Valide 152j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>153j</t>
+          <t>152j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 72j (20/11/2026)</t>
+          <t>Valide 71j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2255,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 153j (09/02/2027)</t>
+          <t>Valide 152j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>153j</t>
+          <t>152j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 72j (20/11/2026)</t>
+          <t>Valide 71j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2465,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 101j (19/12/2026)</t>
+          <t>Valide 100j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>101j</t>
+          <t>100j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 324j (31/07/2027)</t>
+          <t>Valide 323j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2519,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 101j (19/12/2026)</t>
+          <t>Valide 100j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>101j</t>
+          <t>100j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 324j (31/07/2027)</t>
+          <t>Valide 323j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
+          <t>10/09/2026 12:07</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2733,25 +2725,29 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (13/10/2026)</t>
+          <t>Valide 33j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Valide 31j (10/10/2026)</t>
+          <t>Expire dans 30j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>09/09/2026 12:12</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr"/>
+          <t>10/09/2026 12:07</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>email envoye</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1" s="34">
       <c r="A50" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: monitoring 11/09/2026 12:14
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 84j (04/12/2026)</t>
+          <t>Valide 83j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>84j</t>
+          <t>83j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 175j (05/03/2027)</t>
+          <t>Valide 174j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -976,22 +976,22 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Valide 150j (07/02/2027)</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>150j</t>
+          <t>Port 443 inaccessible (pas de SSL)</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 330j (07/08/2027)</t>
+          <t>Valide 329j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (02/11/2026)</t>
+          <t>Valide 51j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>52j</t>
+          <t>51j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 137j (26/01/2027)</t>
+          <t>Valide 136j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (20/11/2026)</t>
+          <t>Valide 70j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>71j</t>
+          <t>70j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 53j (02/11/2026)</t>
+          <t>Valide 52j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (09/02/2027)</t>
+          <t>Valide 151j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>152j</t>
+          <t>151j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 170j (28/02/2027)</t>
+          <t>Valide 169j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 150j (07/02/2027)</t>
+          <t>Valide 149j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>150j</t>
+          <t>149j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 314j (22/07/2027)</t>
+          <t>Valide 313j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 34j (14/10/2026)</t>
+          <t>Valide 33j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>34j</t>
+          <t>33j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 49j (29/10/2026)</t>
+          <t>Valide 48j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 88j (07/12/2026)</t>
+          <t>Valide 87j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 49j (29/10/2026)</t>
+          <t>Valide 48j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>49j</t>
+          <t>48j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 88j (07/12/2026)</t>
+          <t>Valide 87j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (09/10/2026)</t>
+          <t>Expire dans 28j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>28j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 81j (30/11/2026)</t>
+          <t>Valide 80j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 29j (09/10/2026)</t>
+          <t>Expire dans 28j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>29j</t>
+          <t>28j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 81j (30/11/2026)</t>
+          <t>Valide 80j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 152j (09/02/2027)</t>
+          <t>Valide 151j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>152j</t>
+          <t>151j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 71j (20/11/2026)</t>
+          <t>Valide 70j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 152j (09/02/2027)</t>
+          <t>Valide 151j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>152j</t>
+          <t>151j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 71j (20/11/2026)</t>
+          <t>Valide 70j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 100j (19/12/2026)</t>
+          <t>Valide 99j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>100j</t>
+          <t>99j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 323j (31/07/2027)</t>
+          <t>Valide 322j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 100j (19/12/2026)</t>
+          <t>Valide 99j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>100j</t>
+          <t>99j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 323j (31/07/2027)</t>
+          <t>Valide 322j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
+          <t>11/09/2026 12:05</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,29 +2725,25 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (13/10/2026)</t>
+          <t>Valide 32j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 30j (10/10/2026)</t>
+          <t>Expire dans 29j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>10/09/2026 12:07</t>
-        </is>
-      </c>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>email envoye</t>
-        </is>
-      </c>
+          <t>11/09/2026 12:05</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1" s="34">
       <c r="A50" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: monitoring 12/09/2026 11:39
</commit_message>
<xml_diff>
--- a/inventaire_monitoring.xlsx
+++ b/inventaire_monitoring.xlsx
@@ -842,22 +842,22 @@
       </c>
       <c r="L4" s="9" t="inlineStr">
         <is>
-          <t>Valide 83j (04/12/2026)</t>
+          <t>Valide 82j (04/12/2026)</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>83j</t>
+          <t>82j</t>
         </is>
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t>Valide 174j (05/03/2027)</t>
+          <t>Valide 173j (05/03/2027)</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -986,12 +986,12 @@
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>Valide 329j (07/08/2027)</t>
+          <t>Valide 328j (07/08/2027)</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L8" s="9" t="inlineStr">
         <is>
-          <t>Valide 51j (02/11/2026)</t>
+          <t>Valide 50j (02/11/2026)</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>51j</t>
+          <t>50j</t>
         </is>
       </c>
       <c r="N8" s="9" t="inlineStr">
         <is>
-          <t>Valide 136j (26/01/2027)</t>
+          <t>Valide 135j (26/01/2027)</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1152,22 +1152,22 @@
       </c>
       <c r="L10" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (20/11/2026)</t>
+          <t>Valide 69j (20/11/2026)</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>70j</t>
+          <t>69j</t>
         </is>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>Valide 52j (02/11/2026)</t>
+          <t>Valide 51j (02/11/2026)</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1258,22 +1258,22 @@
       </c>
       <c r="L12" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (09/02/2027)</t>
+          <t>Valide 150j (09/02/2027)</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>151j</t>
+          <t>150j</t>
         </is>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>Valide 169j (28/02/2027)</t>
+          <t>Valide 168j (28/02/2027)</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1580,22 +1580,22 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Valide 149j (07/02/2027)</t>
+          <t>Valide 148j (07/02/2027)</t>
         </is>
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>149j</t>
+          <t>148j</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Valide 313j (22/07/2027)</t>
+          <t>Valide 312j (22/07/2027)</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1650,12 +1650,12 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>Valide 33j (14/10/2026)</t>
+          <t>Valide 32j (14/10/2026)</t>
         </is>
       </c>
       <c r="M23" s="9" t="inlineStr">
         <is>
-          <t>33j</t>
+          <t>32j</t>
         </is>
       </c>
       <c r="N23" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1745,22 +1745,22 @@
       </c>
       <c r="L25" s="9" t="inlineStr">
         <is>
-          <t>Valide 48j (29/10/2026)</t>
+          <t>Valide 47j (29/10/2026)</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Valide 87j (07/12/2026)</t>
+          <t>Valide 86j (07/12/2026)</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1811,22 +1811,22 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Valide 48j (29/10/2026)</t>
+          <t>Valide 47j (29/10/2026)</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>48j</t>
+          <t>47j</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Valide 87j (07/12/2026)</t>
+          <t>Valide 86j (07/12/2026)</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -1957,22 +1957,22 @@
       </c>
       <c r="L29" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 28j (09/10/2026)</t>
+          <t>Expire dans 27j (09/10/2026)</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
         <is>
-          <t>28j</t>
+          <t>27j</t>
         </is>
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
-          <t>Valide 80j (30/11/2026)</t>
+          <t>Valide 79j (30/11/2026)</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2007,22 +2007,22 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Expire dans 28j (09/10/2026)</t>
+          <t>Expire dans 27j (09/10/2026)</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
         <is>
-          <t>28j</t>
+          <t>27j</t>
         </is>
       </c>
       <c r="N30" s="4" t="inlineStr">
         <is>
-          <t>Valide 80j (30/11/2026)</t>
+          <t>Valide 79j (30/11/2026)</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="L35" s="9" t="inlineStr">
         <is>
-          <t>Valide 151j (09/02/2027)</t>
+          <t>Valide 150j (09/02/2027)</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
         <is>
-          <t>151j</t>
+          <t>150j</t>
         </is>
       </c>
       <c r="N35" s="9" t="inlineStr">
         <is>
-          <t>Valide 70j (20/11/2026)</t>
+          <t>Valide 69j (20/11/2026)</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2247,22 +2247,22 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Valide 151j (09/02/2027)</t>
+          <t>Valide 150j (09/02/2027)</t>
         </is>
       </c>
       <c r="M36" s="4" t="inlineStr">
         <is>
-          <t>151j</t>
+          <t>150j</t>
         </is>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
-          <t>Valide 70j (20/11/2026)</t>
+          <t>Valide 69j (20/11/2026)</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2457,22 +2457,22 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>Valide 99j (19/12/2026)</t>
+          <t>Valide 98j (19/12/2026)</t>
         </is>
       </c>
       <c r="M42" s="4" t="inlineStr">
         <is>
-          <t>99j</t>
+          <t>98j</t>
         </is>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
-          <t>Valide 322j (31/07/2027)</t>
+          <t>Valide 321j (31/07/2027)</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -2511,22 +2511,22 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>Valide 99j (19/12/2026)</t>
+          <t>Valide 98j (19/12/2026)</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>99j</t>
+          <t>98j</t>
         </is>
       </c>
       <c r="N43" s="9" t="inlineStr">
         <is>
-          <t>Valide 322j (31/07/2027)</t>
+          <t>Valide 321j (31/07/2027)</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -2725,22 +2725,22 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>Valide 32j (13/10/2026)</t>
+          <t>Valide 31j (13/10/2026)</t>
         </is>
       </c>
       <c r="M49" s="9" t="inlineStr">
         <is>
-          <t>32j</t>
+          <t>31j</t>
         </is>
       </c>
       <c r="N49" s="9" t="inlineStr">
         <is>
-          <t>Expire dans 29j (10/10/2026)</t>
+          <t>Expire dans 28j (10/10/2026)</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>11/09/2026 12:05</t>
+          <t>12/09/2026 11:31</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>

</xml_diff>